<commit_message>
Refresh catalog prices and live validation
</commit_message>
<xml_diff>
--- a/data/catalog_500_exact_match.xlsx
+++ b/data/catalog_500_exact_match.xlsx
@@ -15800,7 +15800,7 @@
         <v>289</v>
       </c>
       <c r="K3" s="3">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L3" s="3">
         <v>289</v>
@@ -16175,7 +16175,7 @@
         <v>4736</v>
       </c>
       <c r="K6" s="3">
-        <v>6400</v>
+        <v>6403</v>
       </c>
       <c r="L6" s="3">
         <v>4736</v>
@@ -16303,7 +16303,7 @@
         <v>4159</v>
       </c>
       <c r="K7" s="3">
-        <v>5621</v>
+        <v>5622</v>
       </c>
       <c r="L7" s="3">
         <v>4159</v>
@@ -16457,12 +16457,14 @@
       <c r="S8">
         <v>0.25</v>
       </c>
-      <c r="T8" s="4"/>
+      <c r="T8" s="4">
+        <v>140</v>
+      </c>
       <c r="U8">
-        <v>185</v>
+        <v>100</v>
       </c>
       <c r="V8">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="W8" t="s">
         <v>145</v>
@@ -16554,7 +16556,7 @@
         <v>852</v>
       </c>
       <c r="K9">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="L9">
         <v>852</v>
@@ -16679,7 +16681,7 @@
         <v>3045</v>
       </c>
       <c r="K10">
-        <v>4115</v>
+        <v>4116</v>
       </c>
       <c r="L10">
         <v>3045</v>
@@ -16929,7 +16931,7 @@
         <v>426</v>
       </c>
       <c r="K12">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L12">
         <v>426</v>
@@ -17057,7 +17059,7 @@
         <v>12439</v>
       </c>
       <c r="K13">
-        <v>16810</v>
+        <v>16817</v>
       </c>
       <c r="L13">
         <v>12439</v>
@@ -17182,7 +17184,7 @@
         <v>6220</v>
       </c>
       <c r="K14">
-        <v>8406</v>
+        <v>8409</v>
       </c>
       <c r="L14">
         <v>6220</v>
@@ -17316,7 +17318,7 @@
         <v>6842</v>
       </c>
       <c r="K15">
-        <v>9246</v>
+        <v>9250</v>
       </c>
       <c r="L15">
         <v>6842</v>
@@ -17450,7 +17452,7 @@
         <v>6464</v>
       </c>
       <c r="K16">
-        <v>8736</v>
+        <v>8739</v>
       </c>
       <c r="L16">
         <v>6464</v>
@@ -17578,7 +17580,7 @@
         <v>12828</v>
       </c>
       <c r="K17">
-        <v>17336</v>
+        <v>17343</v>
       </c>
       <c r="L17">
         <v>12828</v>
@@ -17706,7 +17708,7 @@
         <v>7797</v>
       </c>
       <c r="K18">
-        <v>10537</v>
+        <v>10541</v>
       </c>
       <c r="L18">
         <v>7797</v>
@@ -17834,7 +17836,7 @@
         <v>17908</v>
       </c>
       <c r="K19">
-        <v>24200</v>
+        <v>24211</v>
       </c>
       <c r="L19">
         <v>17908</v>
@@ -17962,7 +17964,7 @@
         <v>4281</v>
       </c>
       <c r="K20">
-        <v>5786</v>
+        <v>5787</v>
       </c>
       <c r="L20">
         <v>4281</v>
@@ -18087,7 +18089,7 @@
         <v>2640</v>
       </c>
       <c r="K21">
-        <v>3568</v>
+        <v>3569</v>
       </c>
       <c r="L21">
         <v>2640</v>
@@ -18596,7 +18598,7 @@
         <v>3684</v>
       </c>
       <c r="K25">
-        <v>4979</v>
+        <v>4980</v>
       </c>
       <c r="L25">
         <v>3684</v>
@@ -18730,7 +18732,7 @@
         <v>17498</v>
       </c>
       <c r="K26">
-        <v>23646</v>
+        <v>23657</v>
       </c>
       <c r="L26">
         <v>17498</v>
@@ -18858,7 +18860,7 @@
         <v>1153</v>
       </c>
       <c r="K27">
-        <v>1559</v>
+        <v>1558</v>
       </c>
       <c r="L27">
         <v>1153</v>
@@ -19370,7 +19372,7 @@
         <v>97</v>
       </c>
       <c r="K31">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L31">
         <v>97</v>
@@ -19495,7 +19497,7 @@
         <v>917</v>
       </c>
       <c r="K32">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="L32">
         <v>917</v>
@@ -19757,7 +19759,7 @@
         <v>2098</v>
       </c>
       <c r="O34">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P34" t="s">
         <v>54</v>
@@ -20120,10 +20122,10 @@
         <v>108</v>
       </c>
       <c r="J37">
-        <v>4011</v>
+        <v>3530</v>
       </c>
       <c r="K37">
-        <v>5421</v>
+        <v>4772</v>
       </c>
       <c r="L37">
         <v>4011</v>
@@ -20207,7 +20209,7 @@
         <v>434</v>
       </c>
       <c r="AM37">
-        <v>4011</v>
+        <v>3530</v>
       </c>
       <c r="AO37" t="s">
         <v>427</v>
@@ -20254,10 +20256,10 @@
         <v>131</v>
       </c>
       <c r="J38">
-        <v>3246</v>
+        <v>3762</v>
       </c>
       <c r="K38">
-        <v>4387</v>
+        <v>5086</v>
       </c>
       <c r="L38">
         <v>3246</v>
@@ -20339,6 +20341,9 @@
       </c>
       <c r="AL38" t="s">
         <v>444</v>
+      </c>
+      <c r="AM38">
+        <v>3762</v>
       </c>
       <c r="AO38" t="s">
         <v>427</v>
@@ -20388,7 +20393,7 @@
         <v>2412</v>
       </c>
       <c r="K39">
-        <v>3260</v>
+        <v>3261</v>
       </c>
       <c r="L39">
         <v>2412</v>
@@ -20653,7 +20658,7 @@
         <v>173</v>
       </c>
       <c r="K41">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L41">
         <v>173</v>
@@ -21052,7 +21057,7 @@
         <v>9</v>
       </c>
       <c r="K44">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L44">
         <v>9</v>
@@ -21177,7 +21182,7 @@
         <v>11450</v>
       </c>
       <c r="K45">
-        <v>15473</v>
+        <v>15480</v>
       </c>
       <c r="L45">
         <v>11450</v>
@@ -21299,7 +21304,7 @@
         <v>335</v>
       </c>
       <c r="K46">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="L46">
         <v>335</v>
@@ -21549,7 +21554,7 @@
         <v>3065</v>
       </c>
       <c r="K48">
-        <v>4142</v>
+        <v>4143</v>
       </c>
       <c r="L48">
         <v>3065</v>
@@ -21677,7 +21682,7 @@
         <v>11259</v>
       </c>
       <c r="K49">
-        <v>15215</v>
+        <v>15222</v>
       </c>
       <c r="L49">
         <v>11259</v>
@@ -22177,7 +22182,7 @@
         <v>2604</v>
       </c>
       <c r="K53">
-        <v>3519</v>
+        <v>3520</v>
       </c>
       <c r="L53">
         <v>2604</v>
@@ -22561,7 +22566,7 @@
         <v>488</v>
       </c>
       <c r="K56">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L56">
         <v>488</v>
@@ -22686,7 +22691,7 @@
         <v>488</v>
       </c>
       <c r="K57">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L57">
         <v>488</v>
@@ -22811,7 +22816,7 @@
         <v>488</v>
       </c>
       <c r="K58">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L58">
         <v>488</v>
@@ -22936,7 +22941,7 @@
         <v>488</v>
       </c>
       <c r="K59">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L59">
         <v>488</v>
@@ -23061,7 +23066,7 @@
         <v>488</v>
       </c>
       <c r="K60">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L60">
         <v>488</v>
@@ -23186,7 +23191,7 @@
         <v>488</v>
       </c>
       <c r="K61">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L61">
         <v>488</v>
@@ -23311,7 +23316,7 @@
         <v>488</v>
       </c>
       <c r="K62">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L62">
         <v>488</v>
@@ -23436,7 +23441,7 @@
         <v>488</v>
       </c>
       <c r="K63">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="L63">
         <v>488</v>
@@ -23561,7 +23566,7 @@
         <v>889</v>
       </c>
       <c r="K64">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="L64">
         <v>889</v>
@@ -23811,7 +23816,7 @@
         <v>1008</v>
       </c>
       <c r="K66">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="L66">
         <v>1008</v>
@@ -24058,7 +24063,7 @@
         <v>118</v>
       </c>
       <c r="K68">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L68">
         <v>118</v>
@@ -24183,7 +24188,7 @@
         <v>118</v>
       </c>
       <c r="K69">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L69">
         <v>118</v>
@@ -24558,7 +24563,7 @@
         <v>641</v>
       </c>
       <c r="K72">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="L72">
         <v>641</v>
@@ -24680,7 +24685,7 @@
         <v>578</v>
       </c>
       <c r="K73">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="L73">
         <v>578</v>
@@ -24802,7 +24807,7 @@
         <v>578</v>
       </c>
       <c r="K74">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="L74">
         <v>578</v>
@@ -24924,7 +24929,7 @@
         <v>578</v>
       </c>
       <c r="K75">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="L75">
         <v>578</v>
@@ -25046,7 +25051,7 @@
         <v>326</v>
       </c>
       <c r="K76">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="L76">
         <v>326</v>
@@ -25168,7 +25173,7 @@
         <v>277</v>
       </c>
       <c r="K77">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="L77">
         <v>277</v>
@@ -25290,7 +25295,7 @@
         <v>277</v>
       </c>
       <c r="K78">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="L78">
         <v>277</v>
@@ -25412,7 +25417,7 @@
         <v>1699</v>
       </c>
       <c r="K79">
-        <v>2296</v>
+        <v>2297</v>
       </c>
       <c r="L79">
         <v>1699</v>
@@ -25537,7 +25542,7 @@
         <v>1998</v>
       </c>
       <c r="K80">
-        <v>2700</v>
+        <v>2701</v>
       </c>
       <c r="L80">
         <v>1998</v>
@@ -25662,7 +25667,7 @@
         <v>2444</v>
       </c>
       <c r="K81">
-        <v>3303</v>
+        <v>3304</v>
       </c>
       <c r="L81">
         <v>2444</v>
@@ -25912,7 +25917,7 @@
         <v>2416</v>
       </c>
       <c r="K83">
-        <v>3265</v>
+        <v>3266</v>
       </c>
       <c r="L83">
         <v>2416</v>
@@ -26162,7 +26167,7 @@
         <v>22556</v>
       </c>
       <c r="K85">
-        <v>30482</v>
+        <v>30495</v>
       </c>
       <c r="L85">
         <v>22556</v>
@@ -26412,7 +26417,7 @@
         <v>676</v>
       </c>
       <c r="K87">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="L87">
         <v>676</v>
@@ -26534,7 +26539,7 @@
         <v>2077</v>
       </c>
       <c r="K88">
-        <v>2807</v>
+        <v>2808</v>
       </c>
       <c r="L88">
         <v>2077</v>
@@ -26656,7 +26661,7 @@
         <v>513</v>
       </c>
       <c r="K89">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="L89">
         <v>513</v>
@@ -26900,7 +26905,7 @@
         <v>277</v>
       </c>
       <c r="K91">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="L91">
         <v>277</v>
@@ -27025,7 +27030,7 @@
         <v>69990</v>
       </c>
       <c r="K92">
-        <v>94582</v>
+        <v>94626</v>
       </c>
       <c r="L92">
         <v>69990</v>
@@ -27278,7 +27283,7 @@
         <v>9025</v>
       </c>
       <c r="K94">
-        <v>12196</v>
+        <v>12201</v>
       </c>
       <c r="L94">
         <v>9025</v>
@@ -27400,7 +27405,7 @@
         <v>1190</v>
       </c>
       <c r="K95">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="L95">
         <v>1190</v>
@@ -27522,7 +27527,7 @@
         <v>1190</v>
       </c>
       <c r="K96">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="L96">
         <v>1190</v>
@@ -27888,7 +27893,7 @@
         <v>13001</v>
       </c>
       <c r="K99">
-        <v>17569</v>
+        <v>17577</v>
       </c>
       <c r="L99">
         <v>13001</v>
@@ -28022,7 +28027,7 @@
         <v>2971</v>
       </c>
       <c r="K100">
-        <v>4015</v>
+        <v>4016</v>
       </c>
       <c r="L100">
         <v>2971</v>
@@ -28653,7 +28658,7 @@
         <v>3299</v>
       </c>
       <c r="K105">
-        <v>4459</v>
+        <v>4460</v>
       </c>
       <c r="L105">
         <v>3299</v>
@@ -28903,7 +28908,7 @@
         <v>2080</v>
       </c>
       <c r="K107">
-        <v>2811</v>
+        <v>2812</v>
       </c>
       <c r="L107">
         <v>2080</v>
@@ -29403,7 +29408,7 @@
         <v>2586</v>
       </c>
       <c r="K111">
-        <v>3495</v>
+        <v>3496</v>
       </c>
       <c r="L111">
         <v>2586</v>
@@ -29528,7 +29533,7 @@
         <v>3271</v>
       </c>
       <c r="K112">
-        <v>4421</v>
+        <v>4422</v>
       </c>
       <c r="L112">
         <v>3271</v>
@@ -29903,7 +29908,7 @@
         <v>3329</v>
       </c>
       <c r="K115">
-        <v>4499</v>
+        <v>4500</v>
       </c>
       <c r="L115">
         <v>3329</v>
@@ -30028,7 +30033,7 @@
         <v>2131</v>
       </c>
       <c r="K116">
-        <v>2880</v>
+        <v>2881</v>
       </c>
       <c r="L116">
         <v>2131</v>
@@ -30528,7 +30533,7 @@
         <v>2126</v>
       </c>
       <c r="K120">
-        <v>2873</v>
+        <v>2874</v>
       </c>
       <c r="L120">
         <v>2126</v>
@@ -30653,7 +30658,7 @@
         <v>3859</v>
       </c>
       <c r="K121">
-        <v>5215</v>
+        <v>5217</v>
       </c>
       <c r="L121">
         <v>3859</v>
@@ -31028,7 +31033,7 @@
         <v>3642</v>
       </c>
       <c r="K124">
-        <v>4922</v>
+        <v>4923</v>
       </c>
       <c r="L124">
         <v>3642</v>
@@ -31278,7 +31283,7 @@
         <v>1628</v>
       </c>
       <c r="K126">
-        <v>2200</v>
+        <v>2201</v>
       </c>
       <c r="L126">
         <v>1628</v>
@@ -31528,7 +31533,7 @@
         <v>4783</v>
       </c>
       <c r="K128">
-        <v>6464</v>
+        <v>6466</v>
       </c>
       <c r="L128">
         <v>4783</v>
@@ -31778,7 +31783,7 @@
         <v>3593</v>
       </c>
       <c r="K130">
-        <v>4856</v>
+        <v>4857</v>
       </c>
       <c r="L130">
         <v>3593</v>
@@ -32153,7 +32158,7 @@
         <v>2180</v>
       </c>
       <c r="K133">
-        <v>2946</v>
+        <v>2947</v>
       </c>
       <c r="L133">
         <v>2180</v>
@@ -32278,7 +32283,7 @@
         <v>3687</v>
       </c>
       <c r="K134">
-        <v>4983</v>
+        <v>4984</v>
       </c>
       <c r="L134">
         <v>3687</v>
@@ -33403,7 +33408,7 @@
         <v>2185</v>
       </c>
       <c r="K143">
-        <v>2953</v>
+        <v>2954</v>
       </c>
       <c r="L143">
         <v>2185</v>
@@ -33653,7 +33658,7 @@
         <v>792</v>
       </c>
       <c r="K145">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="L145">
         <v>792</v>
@@ -33778,7 +33783,7 @@
         <v>689</v>
       </c>
       <c r="K146">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="L146">
         <v>689</v>
@@ -33903,7 +33908,7 @@
         <v>3686</v>
       </c>
       <c r="K147">
-        <v>4982</v>
+        <v>4983</v>
       </c>
       <c r="L147">
         <v>3686</v>
@@ -34278,7 +34283,7 @@
         <v>8260</v>
       </c>
       <c r="K150">
-        <v>11163</v>
+        <v>11167</v>
       </c>
       <c r="L150">
         <v>8260</v>
@@ -34403,7 +34408,7 @@
         <v>7457</v>
       </c>
       <c r="K151">
-        <v>10078</v>
+        <v>10081</v>
       </c>
       <c r="L151">
         <v>7457</v>
@@ -34650,7 +34655,7 @@
         <v>4072</v>
       </c>
       <c r="K153">
-        <v>5503</v>
+        <v>5505</v>
       </c>
       <c r="L153">
         <v>4072</v>
@@ -34769,10 +34774,10 @@
         <v>95</v>
       </c>
       <c r="J154">
-        <v>1749</v>
+        <v>1399</v>
       </c>
       <c r="K154">
-        <v>2364</v>
+        <v>1891</v>
       </c>
       <c r="L154">
         <v>1749</v>
@@ -34856,7 +34861,7 @@
         <v>1347</v>
       </c>
       <c r="AM154">
-        <v>1749</v>
+        <v>1399</v>
       </c>
       <c r="AO154" t="s">
         <v>1341</v>
@@ -34915,7 +34920,7 @@
         <v>4521</v>
       </c>
       <c r="O155">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P155" t="s">
         <v>54</v>
@@ -35156,7 +35161,7 @@
         <v>10508</v>
       </c>
       <c r="K157">
-        <v>14200</v>
+        <v>14206</v>
       </c>
       <c r="L157">
         <v>10508</v>
@@ -35531,7 +35536,7 @@
         <v>2393</v>
       </c>
       <c r="K160">
-        <v>3234</v>
+        <v>3235</v>
       </c>
       <c r="L160">
         <v>2393</v>
@@ -35653,7 +35658,7 @@
         <v>3294</v>
       </c>
       <c r="K161">
-        <v>4452</v>
+        <v>4453</v>
       </c>
       <c r="L161">
         <v>3294</v>
@@ -35778,7 +35783,7 @@
         <v>3922</v>
       </c>
       <c r="K162">
-        <v>5300</v>
+        <v>5302</v>
       </c>
       <c r="L162">
         <v>3922</v>
@@ -35903,7 +35908,7 @@
         <v>2237</v>
       </c>
       <c r="K163">
-        <v>3023</v>
+        <v>3024</v>
       </c>
       <c r="L163">
         <v>2237</v>
@@ -36028,7 +36033,7 @@
         <v>687</v>
       </c>
       <c r="K164">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="L164">
         <v>687</v>
@@ -36153,7 +36158,7 @@
         <v>3627</v>
       </c>
       <c r="K165">
-        <v>4902</v>
+        <v>4903</v>
       </c>
       <c r="L165">
         <v>3627</v>
@@ -36275,7 +36280,7 @@
         <v>4689</v>
       </c>
       <c r="K166">
-        <v>6337</v>
+        <v>6339</v>
       </c>
       <c r="L166">
         <v>4689</v>
@@ -36397,7 +36402,7 @@
         <v>2611</v>
       </c>
       <c r="K167">
-        <v>3529</v>
+        <v>3530</v>
       </c>
       <c r="L167">
         <v>2611</v>
@@ -36641,7 +36646,7 @@
         <v>3405</v>
       </c>
       <c r="K169">
-        <v>4602</v>
+        <v>4603</v>
       </c>
       <c r="L169">
         <v>3405</v>
@@ -37019,7 +37024,7 @@
         <v>9360</v>
       </c>
       <c r="K172">
-        <v>12649</v>
+        <v>12654</v>
       </c>
       <c r="L172">
         <v>9360</v>
@@ -37787,7 +37792,7 @@
         <v>3479</v>
       </c>
       <c r="K178">
-        <v>4702</v>
+        <v>4703</v>
       </c>
       <c r="L178">
         <v>3479</v>
@@ -37915,7 +37920,7 @@
         <v>3479</v>
       </c>
       <c r="K179">
-        <v>4702</v>
+        <v>4703</v>
       </c>
       <c r="L179">
         <v>3479</v>
@@ -38043,7 +38048,7 @@
         <v>4476</v>
       </c>
       <c r="K180">
-        <v>6049</v>
+        <v>6051</v>
       </c>
       <c r="L180">
         <v>4476</v>
@@ -38171,7 +38176,7 @@
         <v>4476</v>
       </c>
       <c r="K181">
-        <v>6049</v>
+        <v>6051</v>
       </c>
       <c r="L181">
         <v>4476</v>
@@ -38299,7 +38304,7 @@
         <v>1284</v>
       </c>
       <c r="K182">
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="L182">
         <v>1284</v>
@@ -38424,7 +38429,7 @@
         <v>3238</v>
       </c>
       <c r="K183">
-        <v>4376</v>
+        <v>4377</v>
       </c>
       <c r="L183">
         <v>3238</v>
@@ -38668,7 +38673,7 @@
         <v>2905</v>
       </c>
       <c r="K185">
-        <v>3926</v>
+        <v>3927</v>
       </c>
       <c r="L185">
         <v>2905</v>
@@ -39043,7 +39048,7 @@
         <v>3082</v>
       </c>
       <c r="K188">
-        <v>4165</v>
+        <v>4166</v>
       </c>
       <c r="L188">
         <v>3082</v>
@@ -39168,7 +39173,7 @@
         <v>3930</v>
       </c>
       <c r="K189">
-        <v>5311</v>
+        <v>5313</v>
       </c>
       <c r="L189">
         <v>3930</v>
@@ -39662,7 +39667,7 @@
         <v>59</v>
       </c>
       <c r="K193">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L193">
         <v>59</v>
@@ -39787,7 +39792,7 @@
         <v>198</v>
       </c>
       <c r="K194">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L194">
         <v>198</v>
@@ -40162,7 +40167,7 @@
         <v>397</v>
       </c>
       <c r="K197">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L197">
         <v>397</v>
@@ -40409,7 +40414,7 @@
         <v>826</v>
       </c>
       <c r="K199">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="L199">
         <v>826</v>
@@ -41025,7 +41030,7 @@
         <v>4212</v>
       </c>
       <c r="K204">
-        <v>5692</v>
+        <v>5694</v>
       </c>
       <c r="L204">
         <v>4212</v>
@@ -41147,7 +41152,7 @@
         <v>780</v>
       </c>
       <c r="K205">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="L205">
         <v>780</v>
@@ -41269,7 +41274,7 @@
         <v>1139</v>
       </c>
       <c r="K206">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="L206">
         <v>1139</v>
@@ -41516,7 +41521,7 @@
         <v>3936</v>
       </c>
       <c r="K208">
-        <v>5319</v>
+        <v>5321</v>
       </c>
       <c r="L208">
         <v>3936</v>
@@ -41644,7 +41649,7 @@
         <v>3891</v>
       </c>
       <c r="K209">
-        <v>5259</v>
+        <v>5260</v>
       </c>
       <c r="L209">
         <v>3891</v>
@@ -41772,7 +41777,7 @@
         <v>2833</v>
       </c>
       <c r="K210">
-        <v>3829</v>
+        <v>3830</v>
       </c>
       <c r="L210">
         <v>2833</v>
@@ -41900,7 +41905,7 @@
         <v>3837</v>
       </c>
       <c r="K211">
-        <v>5186</v>
+        <v>5187</v>
       </c>
       <c r="L211">
         <v>3837</v>
@@ -42394,7 +42399,7 @@
         <v>1850</v>
       </c>
       <c r="K215">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="L215">
         <v>1850</v>
@@ -42641,7 +42646,7 @@
         <v>198</v>
       </c>
       <c r="K217">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L217">
         <v>198</v>
@@ -42891,7 +42896,7 @@
         <v>454</v>
       </c>
       <c r="K219">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="L219">
         <v>454</v>
@@ -43266,7 +43271,7 @@
         <v>75</v>
       </c>
       <c r="K222">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L222">
         <v>75</v>
@@ -43391,7 +43396,7 @@
         <v>2791</v>
       </c>
       <c r="K223">
-        <v>3772</v>
+        <v>3773</v>
       </c>
       <c r="L223">
         <v>2791</v>
@@ -43635,10 +43640,10 @@
         <v>473</v>
       </c>
       <c r="J225">
-        <v>6416</v>
+        <v>4170</v>
       </c>
       <c r="K225">
-        <v>8671</v>
+        <v>5637</v>
       </c>
       <c r="L225">
         <v>6416</v>
@@ -43719,7 +43724,7 @@
         <v>1928</v>
       </c>
       <c r="AM225">
-        <v>6416</v>
+        <v>4170</v>
       </c>
       <c r="AO225" t="s">
         <v>1907</v>
@@ -43885,10 +43890,10 @@
         <v>473</v>
       </c>
       <c r="J227">
-        <v>19781</v>
+        <v>13847</v>
       </c>
       <c r="K227">
-        <v>26732</v>
+        <v>18721</v>
       </c>
       <c r="L227">
         <v>19781</v>
@@ -43969,7 +43974,7 @@
         <v>1949</v>
       </c>
       <c r="AM227">
-        <v>19781</v>
+        <v>13847</v>
       </c>
       <c r="AO227" t="s">
         <v>1907</v>
@@ -44013,10 +44018,10 @@
         <v>473</v>
       </c>
       <c r="J228">
-        <v>19781</v>
+        <v>13847</v>
       </c>
       <c r="K228">
-        <v>26732</v>
+        <v>18721</v>
       </c>
       <c r="L228">
         <v>19781</v>
@@ -44097,7 +44102,7 @@
         <v>1956</v>
       </c>
       <c r="AM228">
-        <v>19781</v>
+        <v>13847</v>
       </c>
       <c r="AO228" t="s">
         <v>1907</v>
@@ -44144,7 +44149,7 @@
         <v>2637</v>
       </c>
       <c r="K229">
-        <v>3564</v>
+        <v>3565</v>
       </c>
       <c r="L229">
         <v>2637</v>
@@ -44269,7 +44274,7 @@
         <v>2637</v>
       </c>
       <c r="K230">
-        <v>3564</v>
+        <v>3565</v>
       </c>
       <c r="L230">
         <v>2637</v>
@@ -44397,7 +44402,7 @@
         <v>1955</v>
       </c>
       <c r="K231">
-        <v>2642</v>
+        <v>2643</v>
       </c>
       <c r="L231">
         <v>1955</v>
@@ -45010,7 +45015,7 @@
         <v>4360</v>
       </c>
       <c r="K236">
-        <v>5892</v>
+        <v>5894</v>
       </c>
       <c r="L236">
         <v>4360</v>
@@ -45257,7 +45262,7 @@
         <v>198</v>
       </c>
       <c r="K238">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L238">
         <v>198</v>
@@ -45507,7 +45512,7 @@
         <v>397</v>
       </c>
       <c r="K240">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="L240">
         <v>397</v>
@@ -45757,7 +45762,7 @@
         <v>2777</v>
       </c>
       <c r="K242">
-        <v>3753</v>
+        <v>3754</v>
       </c>
       <c r="L242">
         <v>2777</v>
@@ -45879,7 +45884,7 @@
         <v>198</v>
       </c>
       <c r="K243">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="L243">
         <v>198</v>
@@ -46379,7 +46384,7 @@
         <v>374</v>
       </c>
       <c r="K247">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L247">
         <v>374</v>
@@ -46504,7 +46509,7 @@
         <v>83</v>
       </c>
       <c r="K248">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L248">
         <v>83</v>
@@ -46629,7 +46634,7 @@
         <v>71</v>
       </c>
       <c r="K249">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L249">
         <v>71</v>
@@ -46754,7 +46759,7 @@
         <v>265</v>
       </c>
       <c r="K250">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="L250">
         <v>265</v>
@@ -47379,7 +47384,7 @@
         <v>2953</v>
       </c>
       <c r="K255">
-        <v>3991</v>
+        <v>3992</v>
       </c>
       <c r="L255">
         <v>2953</v>
@@ -47873,7 +47878,7 @@
         <v>3586</v>
       </c>
       <c r="K259">
-        <v>4846</v>
+        <v>4848</v>
       </c>
       <c r="L259">
         <v>3586</v>
@@ -48001,7 +48006,7 @@
         <v>3586</v>
       </c>
       <c r="K260">
-        <v>4846</v>
+        <v>4848</v>
       </c>
       <c r="L260">
         <v>3586</v>
@@ -48129,7 +48134,7 @@
         <v>3586</v>
       </c>
       <c r="K261">
-        <v>4846</v>
+        <v>4848</v>
       </c>
       <c r="L261">
         <v>3586</v>
@@ -48257,7 +48262,7 @@
         <v>3586</v>
       </c>
       <c r="K262">
-        <v>4846</v>
+        <v>4848</v>
       </c>
       <c r="L262">
         <v>3586</v>
@@ -48641,7 +48646,7 @@
         <v>10987</v>
       </c>
       <c r="K265">
-        <v>14848</v>
+        <v>14854</v>
       </c>
       <c r="L265">
         <v>10987</v>
@@ -48769,7 +48774,7 @@
         <v>497</v>
       </c>
       <c r="K266">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="L266">
         <v>497</v>
@@ -48888,10 +48893,10 @@
         <v>95</v>
       </c>
       <c r="J267">
-        <v>936</v>
+        <v>1100</v>
       </c>
       <c r="K267">
-        <v>1265</v>
+        <v>1487</v>
       </c>
       <c r="L267">
         <v>936</v>
@@ -48972,7 +48977,7 @@
         <v>2245</v>
       </c>
       <c r="AM267">
-        <v>936</v>
+        <v>1100</v>
       </c>
       <c r="AO267" t="s">
         <v>572</v>
@@ -49013,10 +49018,10 @@
         <v>95</v>
       </c>
       <c r="J268">
-        <v>2094</v>
+        <v>1540</v>
       </c>
       <c r="K268">
-        <v>2830</v>
+        <v>2082</v>
       </c>
       <c r="L268">
         <v>2094</v>
@@ -49097,7 +49102,7 @@
         <v>2254</v>
       </c>
       <c r="AM268">
-        <v>2094</v>
+        <v>1540</v>
       </c>
       <c r="AO268" t="s">
         <v>572</v>
@@ -49388,7 +49393,7 @@
         <v>425</v>
       </c>
       <c r="K271">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="L271">
         <v>425</v>
@@ -49513,7 +49518,7 @@
         <v>420</v>
       </c>
       <c r="K272">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="L272">
         <v>420</v>
@@ -49638,7 +49643,7 @@
         <v>2592</v>
       </c>
       <c r="K273">
-        <v>3503</v>
+        <v>3504</v>
       </c>
       <c r="L273">
         <v>2592</v>
@@ -49766,7 +49771,7 @@
         <v>8876</v>
       </c>
       <c r="K274">
-        <v>11995</v>
+        <v>12000</v>
       </c>
       <c r="L274">
         <v>8876</v>
@@ -50016,7 +50021,7 @@
         <v>61</v>
       </c>
       <c r="K276">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="L276">
         <v>61</v>
@@ -50138,7 +50143,7 @@
         <v>409</v>
       </c>
       <c r="K277">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="L277">
         <v>409</v>
@@ -50507,7 +50512,7 @@
         <v>2302</v>
       </c>
       <c r="K280">
-        <v>3111</v>
+        <v>3112</v>
       </c>
       <c r="L280">
         <v>2302</v>
@@ -50879,7 +50884,7 @@
         <v>405</v>
       </c>
       <c r="K283">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L283">
         <v>405</v>
@@ -51004,7 +51009,7 @@
         <v>2339</v>
       </c>
       <c r="K284">
-        <v>3161</v>
+        <v>3162</v>
       </c>
       <c r="L284">
         <v>2339</v>
@@ -51501,7 +51506,7 @@
         <v>460</v>
       </c>
       <c r="K288">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="L288">
         <v>460</v>
@@ -51751,7 +51756,7 @@
         <v>113</v>
       </c>
       <c r="K290">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L290">
         <v>113</v>
@@ -51876,7 +51881,7 @@
         <v>104</v>
       </c>
       <c r="K291">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L291">
         <v>104</v>
@@ -52254,7 +52259,7 @@
         <v>294</v>
       </c>
       <c r="K294">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="L294">
         <v>294</v>
@@ -52379,7 +52384,7 @@
         <v>242</v>
       </c>
       <c r="K295">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="L295">
         <v>242</v>
@@ -52504,7 +52509,7 @@
         <v>83</v>
       </c>
       <c r="K296">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L296">
         <v>83</v>
@@ -53016,10 +53021,10 @@
         <v>77</v>
       </c>
       <c r="J300">
-        <v>366</v>
+        <v>323</v>
       </c>
       <c r="K300">
-        <v>495</v>
+        <v>436</v>
       </c>
       <c r="L300">
         <v>366</v>
@@ -53097,7 +53102,7 @@
         <v>2497</v>
       </c>
       <c r="AM300">
-        <v>366</v>
+        <v>323</v>
       </c>
       <c r="AO300" t="s">
         <v>2480</v>
@@ -53141,10 +53146,10 @@
         <v>77</v>
       </c>
       <c r="J301">
-        <v>446</v>
+        <v>392</v>
       </c>
       <c r="K301">
-        <v>603</v>
+        <v>529</v>
       </c>
       <c r="L301">
         <v>446</v>
@@ -53222,7 +53227,7 @@
         <v>2512</v>
       </c>
       <c r="AM301">
-        <v>446</v>
+        <v>392</v>
       </c>
       <c r="AO301" t="s">
         <v>2480</v>
@@ -53272,7 +53277,7 @@
         <v>437</v>
       </c>
       <c r="K302">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="L302">
         <v>437</v>
@@ -53418,7 +53423,7 @@
         <v>4527</v>
       </c>
       <c r="O303">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P303" t="s">
         <v>54</v>
@@ -53543,7 +53548,7 @@
         <v>210</v>
       </c>
       <c r="O304">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P304" t="s">
         <v>54</v>
@@ -53668,7 +53673,7 @@
         <v>458</v>
       </c>
       <c r="O305">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="P305" t="s">
         <v>54</v>
@@ -53781,7 +53786,7 @@
         <v>200</v>
       </c>
       <c r="K306">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L306">
         <v>200</v>
@@ -53912,7 +53917,7 @@
         <v>231</v>
       </c>
       <c r="K307">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="L307">
         <v>231</v>
@@ -54043,7 +54048,7 @@
         <v>218</v>
       </c>
       <c r="K308">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="L308">
         <v>218</v>
@@ -54186,7 +54191,7 @@
         <v>794</v>
       </c>
       <c r="O309">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P309" t="s">
         <v>54</v>
@@ -54299,7 +54304,7 @@
         <v>209</v>
       </c>
       <c r="K310">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="L310">
         <v>209</v>
@@ -54430,7 +54435,7 @@
         <v>231</v>
       </c>
       <c r="K311">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="L311">
         <v>231</v>
@@ -54573,7 +54578,7 @@
         <v>700</v>
       </c>
       <c r="O312">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P312" t="s">
         <v>2601</v>
@@ -54692,7 +54697,7 @@
         <v>231</v>
       </c>
       <c r="K313">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="L313">
         <v>231</v>
@@ -54823,7 +54828,7 @@
         <v>267</v>
       </c>
       <c r="K314">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="L314">
         <v>267</v>
@@ -54966,7 +54971,7 @@
         <v>824</v>
       </c>
       <c r="O315">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P315" t="s">
         <v>54</v>
@@ -55091,7 +55096,7 @@
         <v>496</v>
       </c>
       <c r="O316">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P316" t="s">
         <v>54</v>
@@ -55216,7 +55221,7 @@
         <v>2014</v>
       </c>
       <c r="O317">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P317" t="s">
         <v>54</v>
@@ -55323,10 +55328,10 @@
         <v>77</v>
       </c>
       <c r="J318">
-        <v>23780</v>
+        <v>25237</v>
       </c>
       <c r="K318">
-        <v>32136</v>
+        <v>34120</v>
       </c>
       <c r="L318">
         <v>23780</v>
@@ -55402,6 +55407,9 @@
       </c>
       <c r="AL318" t="s">
         <v>2648</v>
+      </c>
+      <c r="AM318">
+        <v>25237</v>
       </c>
       <c r="AO318" t="s">
         <v>320</v>
@@ -55448,10 +55456,10 @@
         <v>213</v>
       </c>
       <c r="J319">
-        <v>338</v>
+        <v>298</v>
       </c>
       <c r="K319">
-        <v>457</v>
+        <v>402</v>
       </c>
       <c r="L319">
         <v>338</v>
@@ -55532,7 +55540,7 @@
         <v>1696</v>
       </c>
       <c r="AM319">
-        <v>338</v>
+        <v>298</v>
       </c>
       <c r="AO319" t="s">
         <v>320</v>
@@ -55579,7 +55587,7 @@
         <v>68</v>
       </c>
       <c r="K320">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L320">
         <v>68</v>
@@ -55704,10 +55712,10 @@
         <v>1671</v>
       </c>
       <c r="J321">
-        <v>1435</v>
+        <v>1755</v>
       </c>
       <c r="K321">
-        <v>1940</v>
+        <v>2372</v>
       </c>
       <c r="L321">
         <v>1435</v>
@@ -55786,6 +55794,9 @@
       </c>
       <c r="AL321" t="s">
         <v>2677</v>
+      </c>
+      <c r="AM321">
+        <v>1755</v>
       </c>
       <c r="AO321" t="s">
         <v>2673</v>
@@ -55960,10 +55971,10 @@
         <v>77</v>
       </c>
       <c r="J323">
-        <v>1749</v>
+        <v>1934</v>
       </c>
       <c r="K323">
-        <v>2364</v>
+        <v>2614</v>
       </c>
       <c r="L323">
         <v>1749</v>
@@ -56041,7 +56052,7 @@
         <v>2690</v>
       </c>
       <c r="AM323">
-        <v>1749</v>
+        <v>1934</v>
       </c>
       <c r="AN323">
         <v>2198</v>
@@ -56094,7 +56105,7 @@
         <v>2880</v>
       </c>
       <c r="K324">
-        <v>3892</v>
+        <v>3893</v>
       </c>
       <c r="L324">
         <v>2880</v>
@@ -56353,10 +56364,10 @@
         <v>77</v>
       </c>
       <c r="J326">
-        <v>394</v>
+        <v>347</v>
       </c>
       <c r="K326">
-        <v>533</v>
+        <v>469</v>
       </c>
       <c r="L326">
         <v>394</v>
@@ -56434,7 +56445,7 @@
         <v>2716</v>
       </c>
       <c r="AM326">
-        <v>394</v>
+        <v>347</v>
       </c>
       <c r="AO326" t="s">
         <v>427</v>
@@ -56484,7 +56495,7 @@
         <v>44</v>
       </c>
       <c r="K327">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L327">
         <v>44</v>
@@ -56612,7 +56623,7 @@
         <v>835</v>
       </c>
       <c r="K328">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="L328">
         <v>835</v>
@@ -57005,7 +57016,7 @@
         <v>101</v>
       </c>
       <c r="K331">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L331">
         <v>101</v>
@@ -57136,10 +57147,10 @@
         <v>131</v>
       </c>
       <c r="J332">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="K332">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="L332">
         <v>83</v>
@@ -57220,7 +57231,7 @@
         <v>2762</v>
       </c>
       <c r="AM332">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="AO332" t="s">
         <v>427</v>
@@ -57270,7 +57281,7 @@
         <v>2811</v>
       </c>
       <c r="K333">
-        <v>3799</v>
+        <v>3800</v>
       </c>
       <c r="L333">
         <v>2811</v>
@@ -57401,7 +57412,7 @@
         <v>3621</v>
       </c>
       <c r="K334">
-        <v>4894</v>
+        <v>4895</v>
       </c>
       <c r="L334">
         <v>3621</v>
@@ -57529,10 +57540,10 @@
         <v>77</v>
       </c>
       <c r="J335">
-        <v>433</v>
+        <v>380</v>
       </c>
       <c r="K335">
-        <v>586</v>
+        <v>513</v>
       </c>
       <c r="L335">
         <v>433</v>
@@ -57608,6 +57619,9 @@
       </c>
       <c r="AL335" t="s">
         <v>2785</v>
+      </c>
+      <c r="AM335">
+        <v>380</v>
       </c>
       <c r="AO335" t="s">
         <v>427</v>
@@ -57788,7 +57802,7 @@
         <v>4847</v>
       </c>
       <c r="K337">
-        <v>6550</v>
+        <v>6553</v>
       </c>
       <c r="L337">
         <v>4847</v>
@@ -57916,7 +57930,7 @@
         <v>338</v>
       </c>
       <c r="K338">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="L338">
         <v>338</v>
@@ -58047,7 +58061,7 @@
         <v>2456</v>
       </c>
       <c r="K339">
-        <v>3319</v>
+        <v>3320</v>
       </c>
       <c r="L339">
         <v>2456</v>
@@ -58175,10 +58189,10 @@
         <v>77</v>
       </c>
       <c r="J340">
-        <v>527</v>
+        <v>465</v>
       </c>
       <c r="K340">
-        <v>713</v>
+        <v>628</v>
       </c>
       <c r="L340">
         <v>527</v>
@@ -58254,6 +58268,9 @@
       </c>
       <c r="AL340" t="s">
         <v>2824</v>
+      </c>
+      <c r="AM340">
+        <v>465</v>
       </c>
       <c r="AO340" t="s">
         <v>427</v>
@@ -58693,10 +58710,10 @@
         <v>77</v>
       </c>
       <c r="J344">
-        <v>1162</v>
+        <v>1023</v>
       </c>
       <c r="K344">
-        <v>1571</v>
+        <v>1383</v>
       </c>
       <c r="L344">
         <v>1162</v>
@@ -58774,7 +58791,7 @@
         <v>2864</v>
       </c>
       <c r="AM344">
-        <v>1162</v>
+        <v>1023</v>
       </c>
       <c r="AO344" t="s">
         <v>427</v>
@@ -58821,10 +58838,10 @@
         <v>77</v>
       </c>
       <c r="J345">
-        <v>1228</v>
+        <v>1080</v>
       </c>
       <c r="K345">
-        <v>1660</v>
+        <v>1460</v>
       </c>
       <c r="L345">
         <v>1228</v>
@@ -58902,7 +58919,7 @@
         <v>2870</v>
       </c>
       <c r="AM345">
-        <v>1228</v>
+        <v>1080</v>
       </c>
       <c r="AO345" t="s">
         <v>427</v>
@@ -58952,7 +58969,7 @@
         <v>534</v>
       </c>
       <c r="K346">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="L346">
         <v>534</v>
@@ -59083,7 +59100,7 @@
         <v>487</v>
       </c>
       <c r="K347">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="L347">
         <v>487</v>
@@ -59211,10 +59228,10 @@
         <v>213</v>
       </c>
       <c r="J348">
-        <v>2457</v>
+        <v>2162</v>
       </c>
       <c r="K348">
-        <v>3321</v>
+        <v>2923</v>
       </c>
       <c r="L348">
         <v>2457</v>
@@ -59292,7 +59309,7 @@
         <v>2895</v>
       </c>
       <c r="AM348">
-        <v>2457</v>
+        <v>2162</v>
       </c>
       <c r="AO348" t="s">
         <v>427</v>
@@ -59339,10 +59356,10 @@
         <v>213</v>
       </c>
       <c r="J349">
-        <v>549</v>
+        <v>483</v>
       </c>
       <c r="K349">
-        <v>742</v>
+        <v>653</v>
       </c>
       <c r="L349">
         <v>549</v>
@@ -59423,7 +59440,7 @@
         <v>2908</v>
       </c>
       <c r="AM349">
-        <v>549</v>
+        <v>483</v>
       </c>
       <c r="AO349" t="s">
         <v>427</v>
@@ -59470,7 +59487,7 @@
         <v>667</v>
       </c>
       <c r="K350">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="L350">
         <v>667</v>
@@ -59616,7 +59633,7 @@
         <v>1719</v>
       </c>
       <c r="O351">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P351" t="s">
         <v>54</v>
@@ -59738,7 +59755,7 @@
         <v>2296</v>
       </c>
       <c r="O352">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P352" t="s">
         <v>54</v>
@@ -59848,7 +59865,7 @@
         <v>354</v>
       </c>
       <c r="K353">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L353">
         <v>354</v>
@@ -59976,10 +59993,10 @@
         <v>77</v>
       </c>
       <c r="J354">
-        <v>33969</v>
+        <v>29892</v>
       </c>
       <c r="K354">
-        <v>45905</v>
+        <v>40413</v>
       </c>
       <c r="L354">
         <v>33969</v>
@@ -60057,7 +60074,7 @@
         <v>2949</v>
       </c>
       <c r="AM354">
-        <v>33969</v>
+        <v>29892</v>
       </c>
       <c r="AO354" t="s">
         <v>2944</v>
@@ -60107,7 +60124,7 @@
         <v>3661</v>
       </c>
       <c r="K355">
-        <v>4948</v>
+        <v>4949</v>
       </c>
       <c r="L355">
         <v>3661</v>
@@ -60241,7 +60258,7 @@
         <v>4897</v>
       </c>
       <c r="K356">
-        <v>6618</v>
+        <v>6620</v>
       </c>
       <c r="L356">
         <v>4897</v>
@@ -60375,7 +60392,7 @@
         <v>4285</v>
       </c>
       <c r="K357">
-        <v>5791</v>
+        <v>5793</v>
       </c>
       <c r="L357">
         <v>4285</v>
@@ -60509,7 +60526,7 @@
         <v>4285</v>
       </c>
       <c r="K358">
-        <v>5791</v>
+        <v>5793</v>
       </c>
       <c r="L358">
         <v>4285</v>
@@ -60923,7 +60940,7 @@
         <v>2163</v>
       </c>
       <c r="O361">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P361" t="s">
         <v>54</v>
@@ -61051,7 +61068,7 @@
         <v>3460</v>
       </c>
       <c r="O362">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P362" t="s">
         <v>54</v>
@@ -61167,7 +61184,7 @@
         <v>2342</v>
       </c>
       <c r="K363">
-        <v>3165</v>
+        <v>3166</v>
       </c>
       <c r="L363">
         <v>2342</v>
@@ -61700,7 +61717,7 @@
         <v>2935</v>
       </c>
       <c r="K367">
-        <v>3967</v>
+        <v>3968</v>
       </c>
       <c r="L367">
         <v>2935</v>
@@ -61834,7 +61851,7 @@
         <v>3453</v>
       </c>
       <c r="K368">
-        <v>4667</v>
+        <v>4668</v>
       </c>
       <c r="L368">
         <v>3453</v>
@@ -61965,7 +61982,7 @@
         <v>3467</v>
       </c>
       <c r="K369">
-        <v>4686</v>
+        <v>4687</v>
       </c>
       <c r="L369">
         <v>3467</v>
@@ -62099,7 +62116,7 @@
         <v>3937</v>
       </c>
       <c r="K370">
-        <v>5321</v>
+        <v>5322</v>
       </c>
       <c r="L370">
         <v>3937</v>
@@ -62364,7 +62381,7 @@
         <v>131</v>
       </c>
       <c r="K372">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L372">
         <v>131</v>
@@ -62492,7 +62509,7 @@
         <v>988</v>
       </c>
       <c r="K373">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="L373">
         <v>988</v>
@@ -62754,7 +62771,7 @@
         <v>1861</v>
       </c>
       <c r="O375">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P375" t="s">
         <v>54</v>
@@ -62992,7 +63009,7 @@
         <v>749</v>
       </c>
       <c r="K377">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="L377">
         <v>749</v>
@@ -63120,7 +63137,7 @@
         <v>393</v>
       </c>
       <c r="K378">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="L378">
         <v>393</v>
@@ -63501,7 +63518,7 @@
         <v>568</v>
       </c>
       <c r="K381">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="L381">
         <v>568</v>
@@ -64007,10 +64024,10 @@
         <v>213</v>
       </c>
       <c r="J385">
-        <v>181</v>
+        <v>208</v>
       </c>
       <c r="K385">
-        <v>245</v>
+        <v>281</v>
       </c>
       <c r="L385">
         <v>181</v>
@@ -64086,6 +64103,9 @@
       </c>
       <c r="AL385" t="s">
         <v>3189</v>
+      </c>
+      <c r="AM385">
+        <v>208</v>
       </c>
       <c r="AO385" t="s">
         <v>2955</v>
@@ -64257,7 +64277,7 @@
         <v>447</v>
       </c>
       <c r="K387">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="L387">
         <v>447</v>
@@ -64382,7 +64402,7 @@
         <v>389</v>
       </c>
       <c r="K388">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="L388">
         <v>389</v>
@@ -64519,7 +64539,7 @@
         <v>2348</v>
       </c>
       <c r="O389">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P389" t="s">
         <v>54</v>
@@ -64632,10 +64652,10 @@
         <v>77</v>
       </c>
       <c r="J390">
-        <v>677</v>
+        <v>717</v>
       </c>
       <c r="K390">
-        <v>915</v>
+        <v>969</v>
       </c>
       <c r="L390">
         <v>677</v>
@@ -64713,7 +64733,7 @@
         <v>3216</v>
       </c>
       <c r="AM390">
-        <v>677</v>
+        <v>717</v>
       </c>
       <c r="AN390">
         <v>796</v>
@@ -65025,10 +65045,10 @@
         <v>213</v>
       </c>
       <c r="J393">
-        <v>440</v>
+        <v>583</v>
       </c>
       <c r="K393">
-        <v>595</v>
+        <v>788</v>
       </c>
       <c r="L393">
         <v>440</v>
@@ -65106,7 +65126,7 @@
         <v>3240</v>
       </c>
       <c r="AM393">
-        <v>440</v>
+        <v>583</v>
       </c>
       <c r="AN393">
         <v>610</v>
@@ -65156,10 +65176,10 @@
         <v>213</v>
       </c>
       <c r="J394">
-        <v>432</v>
+        <v>599</v>
       </c>
       <c r="K394">
-        <v>584</v>
+        <v>809</v>
       </c>
       <c r="L394">
         <v>432</v>
@@ -65237,7 +65257,7 @@
         <v>3250</v>
       </c>
       <c r="AM394">
-        <v>432</v>
+        <v>599</v>
       </c>
       <c r="AN394">
         <v>561</v>
@@ -65287,10 +65307,10 @@
         <v>213</v>
       </c>
       <c r="J395">
-        <v>711</v>
+        <v>659</v>
       </c>
       <c r="K395">
-        <v>961</v>
+        <v>890</v>
       </c>
       <c r="L395">
         <v>711</v>
@@ -65366,6 +65386,9 @@
       </c>
       <c r="AL395" t="s">
         <v>3260</v>
+      </c>
+      <c r="AM395">
+        <v>659</v>
       </c>
       <c r="AO395" t="s">
         <v>3245</v>
@@ -65412,10 +65435,10 @@
         <v>213</v>
       </c>
       <c r="J396">
-        <v>529</v>
+        <v>734</v>
       </c>
       <c r="K396">
-        <v>715</v>
+        <v>992</v>
       </c>
       <c r="L396">
         <v>529</v>
@@ -65493,7 +65516,7 @@
         <v>3266</v>
       </c>
       <c r="AM396">
-        <v>529</v>
+        <v>734</v>
       </c>
       <c r="AN396">
         <v>733</v>
@@ -65543,10 +65566,10 @@
         <v>213</v>
       </c>
       <c r="J397">
-        <v>964</v>
+        <v>1172</v>
       </c>
       <c r="K397">
-        <v>1303</v>
+        <v>1584</v>
       </c>
       <c r="L397">
         <v>964</v>
@@ -65624,7 +65647,7 @@
         <v>3273</v>
       </c>
       <c r="AM397">
-        <v>964</v>
+        <v>1172</v>
       </c>
       <c r="AO397" t="s">
         <v>3255</v>
@@ -65671,10 +65694,10 @@
         <v>213</v>
       </c>
       <c r="J398">
-        <v>474</v>
+        <v>706</v>
       </c>
       <c r="K398">
-        <v>641</v>
+        <v>954</v>
       </c>
       <c r="L398">
         <v>474</v>
@@ -65752,7 +65775,7 @@
         <v>3280</v>
       </c>
       <c r="AM398">
-        <v>474</v>
+        <v>706</v>
       </c>
       <c r="AN398">
         <v>578</v>
@@ -65802,10 +65825,10 @@
         <v>213</v>
       </c>
       <c r="J399">
-        <v>565</v>
+        <v>844</v>
       </c>
       <c r="K399">
-        <v>764</v>
+        <v>1141</v>
       </c>
       <c r="L399">
         <v>565</v>
@@ -65883,7 +65906,7 @@
         <v>3287</v>
       </c>
       <c r="AM399">
-        <v>565</v>
+        <v>844</v>
       </c>
       <c r="AN399">
         <v>691</v>
@@ -65933,10 +65956,10 @@
         <v>213</v>
       </c>
       <c r="J400">
-        <v>722</v>
+        <v>530</v>
       </c>
       <c r="K400">
-        <v>976</v>
+        <v>716</v>
       </c>
       <c r="L400">
         <v>722</v>
@@ -66017,7 +66040,7 @@
         <v>3294</v>
       </c>
       <c r="AM400">
-        <v>722</v>
+        <v>530</v>
       </c>
       <c r="AN400">
         <v>1030</v>
@@ -66067,10 +66090,10 @@
         <v>213</v>
       </c>
       <c r="J401">
-        <v>592</v>
+        <v>558</v>
       </c>
       <c r="K401">
-        <v>800</v>
+        <v>754</v>
       </c>
       <c r="L401">
         <v>592</v>
@@ -66151,7 +66174,7 @@
         <v>3303</v>
       </c>
       <c r="AM401">
-        <v>592</v>
+        <v>558</v>
       </c>
       <c r="AN401">
         <v>767</v>
@@ -66201,10 +66224,10 @@
         <v>213</v>
       </c>
       <c r="J402">
-        <v>437</v>
+        <v>599</v>
       </c>
       <c r="K402">
-        <v>591</v>
+        <v>809</v>
       </c>
       <c r="L402">
         <v>437</v>
@@ -66282,7 +66305,7 @@
         <v>3310</v>
       </c>
       <c r="AM402">
-        <v>437</v>
+        <v>599</v>
       </c>
       <c r="AN402">
         <v>547</v>
@@ -66332,10 +66355,10 @@
         <v>213</v>
       </c>
       <c r="J403">
-        <v>830</v>
+        <v>1140</v>
       </c>
       <c r="K403">
-        <v>1122</v>
+        <v>1541</v>
       </c>
       <c r="L403">
         <v>830</v>
@@ -66416,7 +66439,7 @@
         <v>3323</v>
       </c>
       <c r="AM403">
-        <v>830</v>
+        <v>1140</v>
       </c>
       <c r="AN403">
         <v>976</v>
@@ -66466,10 +66489,10 @@
         <v>213</v>
       </c>
       <c r="J404">
-        <v>659</v>
+        <v>740</v>
       </c>
       <c r="K404">
-        <v>891</v>
+        <v>1000</v>
       </c>
       <c r="L404">
         <v>659</v>
@@ -66550,7 +66573,7 @@
         <v>3328</v>
       </c>
       <c r="AM404">
-        <v>659</v>
+        <v>740</v>
       </c>
       <c r="AO404" t="s">
         <v>3298</v>
@@ -66597,10 +66620,10 @@
         <v>213</v>
       </c>
       <c r="J405">
-        <v>482</v>
+        <v>599</v>
       </c>
       <c r="K405">
-        <v>652</v>
+        <v>809</v>
       </c>
       <c r="L405">
         <v>482</v>
@@ -66681,7 +66704,7 @@
         <v>3336</v>
       </c>
       <c r="AM405">
-        <v>482</v>
+        <v>599</v>
       </c>
       <c r="AN405">
         <v>625</v>
@@ -66731,10 +66754,10 @@
         <v>213</v>
       </c>
       <c r="J406">
-        <v>678</v>
+        <v>583</v>
       </c>
       <c r="K406">
-        <v>917</v>
+        <v>788</v>
       </c>
       <c r="L406">
         <v>678</v>
@@ -66812,7 +66835,7 @@
         <v>3343</v>
       </c>
       <c r="AM406">
-        <v>678</v>
+        <v>583</v>
       </c>
       <c r="AO406" t="s">
         <v>3255</v>
@@ -66859,10 +66882,10 @@
         <v>213</v>
       </c>
       <c r="J407">
-        <v>896</v>
+        <v>583</v>
       </c>
       <c r="K407">
-        <v>1211</v>
+        <v>788</v>
       </c>
       <c r="L407">
         <v>896</v>
@@ -66940,7 +66963,7 @@
         <v>3350</v>
       </c>
       <c r="AM407">
-        <v>896</v>
+        <v>583</v>
       </c>
       <c r="AO407" t="s">
         <v>3298</v>
@@ -66987,10 +67010,10 @@
         <v>213</v>
       </c>
       <c r="J408">
-        <v>880</v>
+        <v>791</v>
       </c>
       <c r="K408">
-        <v>1190</v>
+        <v>1069</v>
       </c>
       <c r="L408">
         <v>880</v>
@@ -67068,7 +67091,7 @@
         <v>3357</v>
       </c>
       <c r="AM408">
-        <v>880</v>
+        <v>791</v>
       </c>
       <c r="AO408" t="s">
         <v>3241</v>
@@ -67115,10 +67138,10 @@
         <v>213</v>
       </c>
       <c r="J409">
-        <v>637</v>
+        <v>734</v>
       </c>
       <c r="K409">
-        <v>861</v>
+        <v>992</v>
       </c>
       <c r="L409">
         <v>637</v>
@@ -67199,7 +67222,7 @@
         <v>3363</v>
       </c>
       <c r="AM409">
-        <v>637</v>
+        <v>734</v>
       </c>
       <c r="AO409" t="s">
         <v>3314</v>
@@ -67246,10 +67269,10 @@
         <v>213</v>
       </c>
       <c r="J410">
-        <v>639</v>
+        <v>610</v>
       </c>
       <c r="K410">
-        <v>864</v>
+        <v>824</v>
       </c>
       <c r="L410">
         <v>639</v>
@@ -67327,7 +67350,7 @@
         <v>3373</v>
       </c>
       <c r="AM410">
-        <v>639</v>
+        <v>610</v>
       </c>
       <c r="AO410" t="s">
         <v>3298</v>
@@ -67374,10 +67397,10 @@
         <v>213</v>
       </c>
       <c r="J411">
-        <v>436</v>
+        <v>558</v>
       </c>
       <c r="K411">
-        <v>590</v>
+        <v>754</v>
       </c>
       <c r="L411">
         <v>436</v>
@@ -67455,7 +67478,7 @@
         <v>3378</v>
       </c>
       <c r="AM411">
-        <v>436</v>
+        <v>558</v>
       </c>
       <c r="AN411">
         <v>544</v>
@@ -67505,10 +67528,10 @@
         <v>213</v>
       </c>
       <c r="J412">
-        <v>592</v>
+        <v>649</v>
       </c>
       <c r="K412">
-        <v>800</v>
+        <v>877</v>
       </c>
       <c r="L412">
         <v>592</v>
@@ -67589,7 +67612,7 @@
         <v>3386</v>
       </c>
       <c r="AM412">
-        <v>592</v>
+        <v>649</v>
       </c>
       <c r="AO412" t="s">
         <v>3255</v>
@@ -67636,10 +67659,10 @@
         <v>213</v>
       </c>
       <c r="J413">
-        <v>619</v>
+        <v>636</v>
       </c>
       <c r="K413">
-        <v>837</v>
+        <v>859</v>
       </c>
       <c r="L413">
         <v>619</v>
@@ -67717,7 +67740,7 @@
         <v>3393</v>
       </c>
       <c r="AM413">
-        <v>619</v>
+        <v>636</v>
       </c>
       <c r="AO413" t="s">
         <v>3298</v>
@@ -67764,10 +67787,10 @@
         <v>213</v>
       </c>
       <c r="J414">
-        <v>1041</v>
+        <v>1392</v>
       </c>
       <c r="K414">
-        <v>1407</v>
+        <v>1881</v>
       </c>
       <c r="L414">
         <v>1041</v>
@@ -67848,7 +67871,7 @@
         <v>3400</v>
       </c>
       <c r="AM414">
-        <v>1041</v>
+        <v>1392</v>
       </c>
       <c r="AO414" t="s">
         <v>3298</v>
@@ -67895,10 +67918,10 @@
         <v>213</v>
       </c>
       <c r="J415">
-        <v>468</v>
+        <v>626</v>
       </c>
       <c r="K415">
-        <v>633</v>
+        <v>846</v>
       </c>
       <c r="L415">
         <v>468</v>
@@ -67976,7 +67999,7 @@
         <v>3408</v>
       </c>
       <c r="AM415">
-        <v>468</v>
+        <v>626</v>
       </c>
       <c r="AN415">
         <v>603</v>
@@ -68026,10 +68049,10 @@
         <v>213</v>
       </c>
       <c r="J416">
-        <v>835</v>
+        <v>583</v>
       </c>
       <c r="K416">
-        <v>1129</v>
+        <v>788</v>
       </c>
       <c r="L416">
         <v>835</v>
@@ -68107,7 +68130,7 @@
         <v>3416</v>
       </c>
       <c r="AM416">
-        <v>835</v>
+        <v>583</v>
       </c>
       <c r="AO416" t="s">
         <v>3411</v>
@@ -68154,10 +68177,10 @@
         <v>213</v>
       </c>
       <c r="J417">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="K417">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="L417">
         <v>578</v>
@@ -68235,7 +68258,7 @@
         <v>3423</v>
       </c>
       <c r="AM417">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="AO417" t="s">
         <v>3426</v>
@@ -68282,10 +68305,10 @@
         <v>213</v>
       </c>
       <c r="J418">
-        <v>548</v>
+        <v>530</v>
       </c>
       <c r="K418">
-        <v>741</v>
+        <v>716</v>
       </c>
       <c r="L418">
         <v>548</v>
@@ -68363,7 +68386,7 @@
         <v>3430</v>
       </c>
       <c r="AM418">
-        <v>548</v>
+        <v>530</v>
       </c>
       <c r="AN418">
         <v>710</v>
@@ -68413,10 +68436,10 @@
         <v>213</v>
       </c>
       <c r="J419">
-        <v>399</v>
+        <v>573</v>
       </c>
       <c r="K419">
-        <v>540</v>
+        <v>774</v>
       </c>
       <c r="L419">
         <v>399</v>
@@ -68494,7 +68517,7 @@
         <v>3437</v>
       </c>
       <c r="AM419">
-        <v>399</v>
+        <v>573</v>
       </c>
       <c r="AN419">
         <v>469</v>
@@ -68544,10 +68567,10 @@
         <v>213</v>
       </c>
       <c r="J420">
-        <v>606</v>
+        <v>742</v>
       </c>
       <c r="K420">
-        <v>819</v>
+        <v>1003</v>
       </c>
       <c r="L420">
         <v>606</v>
@@ -68625,7 +68648,7 @@
         <v>3443</v>
       </c>
       <c r="AM420">
-        <v>606</v>
+        <v>742</v>
       </c>
       <c r="AN420">
         <v>734</v>
@@ -68675,10 +68698,10 @@
         <v>213</v>
       </c>
       <c r="J421">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="K421">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="L421">
         <v>559</v>
@@ -68756,7 +68779,7 @@
         <v>3449</v>
       </c>
       <c r="AM421">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="AN421">
         <v>698</v>
@@ -68806,10 +68829,10 @@
         <v>213</v>
       </c>
       <c r="J422">
-        <v>534</v>
+        <v>573</v>
       </c>
       <c r="K422">
-        <v>722</v>
+        <v>774</v>
       </c>
       <c r="L422">
         <v>534</v>
@@ -68887,7 +68910,7 @@
         <v>3455</v>
       </c>
       <c r="AM422">
-        <v>534</v>
+        <v>573</v>
       </c>
       <c r="AO422" t="s">
         <v>3255</v>
@@ -68934,10 +68957,10 @@
         <v>213</v>
       </c>
       <c r="J423">
-        <v>428</v>
+        <v>626</v>
       </c>
       <c r="K423">
-        <v>579</v>
+        <v>846</v>
       </c>
       <c r="L423">
         <v>428</v>
@@ -69018,7 +69041,7 @@
         <v>3461</v>
       </c>
       <c r="AM423">
-        <v>428</v>
+        <v>626</v>
       </c>
       <c r="AN423">
         <v>522</v>
@@ -69068,10 +69091,10 @@
         <v>213</v>
       </c>
       <c r="J424">
-        <v>842</v>
+        <v>794</v>
       </c>
       <c r="K424">
-        <v>1138</v>
+        <v>1073</v>
       </c>
       <c r="L424">
         <v>842</v>
@@ -69152,7 +69175,7 @@
         <v>3469</v>
       </c>
       <c r="AM424">
-        <v>842</v>
+        <v>794</v>
       </c>
       <c r="AO424" t="s">
         <v>3298</v>
@@ -69199,10 +69222,10 @@
         <v>213</v>
       </c>
       <c r="J425">
-        <v>1478</v>
+        <v>910</v>
       </c>
       <c r="K425">
-        <v>1998</v>
+        <v>1230</v>
       </c>
       <c r="L425">
         <v>1478</v>
@@ -69283,7 +69306,7 @@
         <v>3481</v>
       </c>
       <c r="AM425">
-        <v>1478</v>
+        <v>910</v>
       </c>
       <c r="AO425" t="s">
         <v>2921</v>
@@ -69327,10 +69350,10 @@
         <v>213</v>
       </c>
       <c r="J426">
-        <v>1108</v>
+        <v>780</v>
       </c>
       <c r="K426">
-        <v>1498</v>
+        <v>1054</v>
       </c>
       <c r="L426">
         <v>1108</v>
@@ -69408,7 +69431,7 @@
         <v>3489</v>
       </c>
       <c r="AM426">
-        <v>1108</v>
+        <v>780</v>
       </c>
       <c r="AO426" t="s">
         <v>3241</v>
@@ -69452,10 +69475,10 @@
         <v>213</v>
       </c>
       <c r="J427">
-        <v>865</v>
+        <v>782</v>
       </c>
       <c r="K427">
-        <v>1169</v>
+        <v>1057</v>
       </c>
       <c r="L427">
         <v>865</v>
@@ -69536,7 +69559,7 @@
         <v>3493</v>
       </c>
       <c r="AM427">
-        <v>865</v>
+        <v>782</v>
       </c>
       <c r="AO427" t="s">
         <v>3497</v>
@@ -69580,10 +69603,10 @@
         <v>213</v>
       </c>
       <c r="J428">
-        <v>1021</v>
+        <v>809</v>
       </c>
       <c r="K428">
-        <v>1380</v>
+        <v>1093</v>
       </c>
       <c r="L428">
         <v>1021</v>
@@ -69664,7 +69687,7 @@
         <v>3501</v>
       </c>
       <c r="AM428">
-        <v>1021</v>
+        <v>809</v>
       </c>
       <c r="AO428" t="s">
         <v>3314</v>
@@ -69708,10 +69731,10 @@
         <v>213</v>
       </c>
       <c r="J429">
-        <v>573</v>
+        <v>319</v>
       </c>
       <c r="K429">
-        <v>775</v>
+        <v>431</v>
       </c>
       <c r="L429">
         <v>573</v>
@@ -69792,7 +69815,7 @@
         <v>3508</v>
       </c>
       <c r="AM429">
-        <v>573</v>
+        <v>319</v>
       </c>
       <c r="AO429" t="s">
         <v>3497</v>
@@ -69836,10 +69859,10 @@
         <v>213</v>
       </c>
       <c r="J430">
-        <v>677</v>
+        <v>1068</v>
       </c>
       <c r="K430">
-        <v>915</v>
+        <v>1443</v>
       </c>
       <c r="L430">
         <v>677</v>
@@ -69920,7 +69943,7 @@
         <v>3515</v>
       </c>
       <c r="AM430">
-        <v>677</v>
+        <v>1068</v>
       </c>
       <c r="AN430">
         <v>827</v>
@@ -69967,10 +69990,10 @@
         <v>213</v>
       </c>
       <c r="J431">
-        <v>786</v>
+        <v>601</v>
       </c>
       <c r="K431">
-        <v>1063</v>
+        <v>812</v>
       </c>
       <c r="L431">
         <v>786</v>
@@ -70051,7 +70074,7 @@
         <v>3522</v>
       </c>
       <c r="AM431">
-        <v>786</v>
+        <v>601</v>
       </c>
       <c r="AO431" t="s">
         <v>3241</v>
@@ -70095,10 +70118,10 @@
         <v>213</v>
       </c>
       <c r="J432">
-        <v>930</v>
+        <v>835</v>
       </c>
       <c r="K432">
-        <v>1257</v>
+        <v>1128</v>
       </c>
       <c r="L432">
         <v>930</v>
@@ -70179,7 +70202,7 @@
         <v>3528</v>
       </c>
       <c r="AM432">
-        <v>930</v>
+        <v>835</v>
       </c>
       <c r="AO432" t="s">
         <v>3255</v>
@@ -70223,10 +70246,10 @@
         <v>213</v>
       </c>
       <c r="J433">
-        <v>2437</v>
+        <v>2667</v>
       </c>
       <c r="K433">
-        <v>3294</v>
+        <v>3605</v>
       </c>
       <c r="L433">
         <v>2437</v>
@@ -70307,7 +70330,7 @@
         <v>3536</v>
       </c>
       <c r="AM433">
-        <v>2437</v>
+        <v>2667</v>
       </c>
       <c r="AO433" t="s">
         <v>3255</v>
@@ -70351,10 +70374,10 @@
         <v>213</v>
       </c>
       <c r="J434">
-        <v>551</v>
+        <v>788</v>
       </c>
       <c r="K434">
-        <v>745</v>
+        <v>1065</v>
       </c>
       <c r="L434">
         <v>551</v>
@@ -70435,7 +70458,7 @@
         <v>3544</v>
       </c>
       <c r="AM434">
-        <v>551</v>
+        <v>788</v>
       </c>
       <c r="AO434" t="s">
         <v>3411</v>
@@ -70479,10 +70502,10 @@
         <v>213</v>
       </c>
       <c r="J435">
-        <v>841</v>
+        <v>502</v>
       </c>
       <c r="K435">
-        <v>1137</v>
+        <v>678</v>
       </c>
       <c r="L435">
         <v>841</v>
@@ -70563,7 +70586,7 @@
         <v>3550</v>
       </c>
       <c r="AM435">
-        <v>841</v>
+        <v>502</v>
       </c>
       <c r="AO435" t="s">
         <v>3497</v>
@@ -70607,10 +70630,10 @@
         <v>213</v>
       </c>
       <c r="J436">
-        <v>328</v>
+        <v>151</v>
       </c>
       <c r="K436">
-        <v>444</v>
+        <v>204</v>
       </c>
       <c r="L436">
         <v>328</v>
@@ -70688,7 +70711,7 @@
         <v>3557</v>
       </c>
       <c r="AM436">
-        <v>328</v>
+        <v>151</v>
       </c>
       <c r="AO436" t="s">
         <v>3411</v>
@@ -70732,10 +70755,10 @@
         <v>108</v>
       </c>
       <c r="J437">
-        <v>318</v>
+        <v>281</v>
       </c>
       <c r="K437">
-        <v>430</v>
+        <v>379</v>
       </c>
       <c r="L437">
         <v>318</v>
@@ -70816,7 +70839,7 @@
         <v>3562</v>
       </c>
       <c r="AM437">
-        <v>318</v>
+        <v>281</v>
       </c>
       <c r="AO437" t="s">
         <v>3563</v>
@@ -70863,7 +70886,7 @@
         <v>10236</v>
       </c>
       <c r="K438">
-        <v>13833</v>
+        <v>13839</v>
       </c>
       <c r="L438">
         <v>10236</v>
@@ -70994,7 +71017,7 @@
         <v>5817</v>
       </c>
       <c r="K439">
-        <v>7861</v>
+        <v>7864</v>
       </c>
       <c r="L439">
         <v>5817</v>
@@ -71134,7 +71157,7 @@
         <v>3333</v>
       </c>
       <c r="O440">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P440" t="s">
         <v>54</v>
@@ -71244,10 +71267,10 @@
         <v>77</v>
       </c>
       <c r="J441">
-        <v>560</v>
+        <v>884</v>
       </c>
       <c r="K441">
-        <v>757</v>
+        <v>1195</v>
       </c>
       <c r="L441">
         <v>560</v>
@@ -71325,7 +71348,7 @@
         <v>3596</v>
       </c>
       <c r="AM441">
-        <v>560</v>
+        <v>884</v>
       </c>
       <c r="AN441">
         <v>659</v>
@@ -71372,10 +71395,10 @@
         <v>213</v>
       </c>
       <c r="J442">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="K442">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="L442">
         <v>243</v>
@@ -71453,7 +71476,7 @@
         <v>3607</v>
       </c>
       <c r="AM442">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="AO442" t="s">
         <v>3314</v>
@@ -71500,7 +71523,7 @@
         <v>82</v>
       </c>
       <c r="K443">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L443">
         <v>82</v>
@@ -71640,7 +71663,7 @@
         <v>505</v>
       </c>
       <c r="O444">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P444" t="s">
         <v>54</v>
@@ -71765,7 +71788,7 @@
         <v>168</v>
       </c>
       <c r="O445">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P445" t="s">
         <v>54</v>
@@ -71875,7 +71898,7 @@
         <v>93</v>
       </c>
       <c r="K446">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="L446">
         <v>93</v>
@@ -72012,7 +72035,7 @@
         <v>205</v>
       </c>
       <c r="O447">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P447" t="s">
         <v>2601</v>
@@ -72140,7 +72163,7 @@
         <v>10712</v>
       </c>
       <c r="O448">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P448" t="s">
         <v>54</v>
@@ -72247,10 +72270,10 @@
         <v>213</v>
       </c>
       <c r="J449">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="K449">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="L449">
         <v>405</v>
@@ -72328,7 +72351,7 @@
         <v>3654</v>
       </c>
       <c r="AM449">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="AO449" t="s">
         <v>3314</v>
@@ -72375,7 +72398,7 @@
         <v>110</v>
       </c>
       <c r="K450">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="L450">
         <v>110</v>
@@ -72515,7 +72538,7 @@
         <v>135</v>
       </c>
       <c r="O451">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P451" t="s">
         <v>54</v>
@@ -72622,10 +72645,10 @@
         <v>213</v>
       </c>
       <c r="J452">
-        <v>1780</v>
+        <v>1807</v>
       </c>
       <c r="K452">
-        <v>2406</v>
+        <v>2443</v>
       </c>
       <c r="L452">
         <v>1780</v>
@@ -72703,7 +72726,7 @@
         <v>3675</v>
       </c>
       <c r="AM452">
-        <v>1780</v>
+        <v>1807</v>
       </c>
       <c r="AO452" t="s">
         <v>3314</v>
@@ -72750,10 +72773,10 @@
         <v>213</v>
       </c>
       <c r="J453">
-        <v>1765</v>
+        <v>1792</v>
       </c>
       <c r="K453">
-        <v>2386</v>
+        <v>2422</v>
       </c>
       <c r="L453">
         <v>1765</v>
@@ -72834,7 +72857,7 @@
         <v>3683</v>
       </c>
       <c r="AM453">
-        <v>1765</v>
+        <v>1792</v>
       </c>
       <c r="AO453" t="s">
         <v>3314</v>
@@ -72896,7 +72919,7 @@
         <v>407</v>
       </c>
       <c r="O454">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P454" t="s">
         <v>54</v>
@@ -73006,7 +73029,7 @@
         <v>44</v>
       </c>
       <c r="K455">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L455">
         <v>44</v>
@@ -73131,7 +73154,7 @@
         <v>213</v>
       </c>
       <c r="J456">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K456">
         <v>128</v>
@@ -73212,7 +73235,7 @@
         <v>3704</v>
       </c>
       <c r="AM456">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AO456" t="s">
         <v>3314</v>
@@ -73256,7 +73279,7 @@
         <v>213</v>
       </c>
       <c r="J457">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K457">
         <v>78</v>
@@ -73337,7 +73360,7 @@
         <v>3711</v>
       </c>
       <c r="AM457">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AO457" t="s">
         <v>3314</v>
@@ -73396,7 +73419,7 @@
         <v>121</v>
       </c>
       <c r="O458">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P458" t="s">
         <v>54</v>
@@ -73521,7 +73544,7 @@
         <v>856</v>
       </c>
       <c r="O459">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P459" t="s">
         <v>54</v>
@@ -73634,10 +73657,10 @@
         <v>213</v>
       </c>
       <c r="J460">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="K460">
-        <v>923</v>
+        <v>936</v>
       </c>
       <c r="L460">
         <v>683</v>
@@ -73715,7 +73738,7 @@
         <v>3734</v>
       </c>
       <c r="AM460">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="AO460" t="s">
         <v>3314</v>
@@ -73759,10 +73782,10 @@
         <v>213</v>
       </c>
       <c r="J461">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="K461">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="L461">
         <v>417</v>
@@ -73840,7 +73863,7 @@
         <v>3741</v>
       </c>
       <c r="AM461">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="AO461" t="s">
         <v>3314</v>
@@ -73899,7 +73922,7 @@
         <v>3564</v>
       </c>
       <c r="O462">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P462" t="s">
         <v>54</v>
@@ -74006,10 +74029,10 @@
         <v>213</v>
       </c>
       <c r="J463">
-        <v>2038</v>
+        <v>2069</v>
       </c>
       <c r="K463">
-        <v>2755</v>
+        <v>2797</v>
       </c>
       <c r="L463">
         <v>2038</v>
@@ -74090,7 +74113,7 @@
         <v>3756</v>
       </c>
       <c r="AM463">
-        <v>2038</v>
+        <v>2069</v>
       </c>
       <c r="AO463" t="s">
         <v>3314</v>
@@ -74134,10 +74157,10 @@
         <v>213</v>
       </c>
       <c r="J464">
-        <v>1713</v>
+        <v>1739</v>
       </c>
       <c r="K464">
-        <v>2315</v>
+        <v>2351</v>
       </c>
       <c r="L464">
         <v>1713</v>
@@ -74218,7 +74241,7 @@
         <v>3764</v>
       </c>
       <c r="AM464">
-        <v>1713</v>
+        <v>1739</v>
       </c>
       <c r="AO464" t="s">
         <v>3255</v>
@@ -74277,7 +74300,7 @@
         <v>1430</v>
       </c>
       <c r="O465">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P465" t="s">
         <v>54</v>
@@ -74387,10 +74410,10 @@
         <v>213</v>
       </c>
       <c r="J466">
-        <v>5036</v>
+        <v>5113</v>
       </c>
       <c r="K466">
-        <v>6806</v>
+        <v>6912</v>
       </c>
       <c r="L466">
         <v>5036</v>
@@ -74471,7 +74494,7 @@
         <v>3779</v>
       </c>
       <c r="AM466">
-        <v>5036</v>
+        <v>5113</v>
       </c>
       <c r="AO466" t="s">
         <v>3255</v>
@@ -74515,10 +74538,10 @@
         <v>213</v>
       </c>
       <c r="J467">
-        <v>9629</v>
+        <v>9776</v>
       </c>
       <c r="K467">
-        <v>13013</v>
+        <v>13217</v>
       </c>
       <c r="L467">
         <v>9629</v>
@@ -74596,7 +74619,7 @@
         <v>3785</v>
       </c>
       <c r="AM467">
-        <v>9629</v>
+        <v>9776</v>
       </c>
       <c r="AO467" t="s">
         <v>3314</v>
@@ -74655,7 +74678,7 @@
         <v>1063</v>
       </c>
       <c r="O468">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="P468" t="s">
         <v>54</v>
@@ -74762,10 +74785,10 @@
         <v>213</v>
       </c>
       <c r="J469">
-        <v>34827</v>
+        <v>35356</v>
       </c>
       <c r="K469">
-        <v>47064</v>
+        <v>47801</v>
       </c>
       <c r="L469">
         <v>34827</v>
@@ -74846,7 +74869,7 @@
         <v>3798</v>
       </c>
       <c r="AM469">
-        <v>34827</v>
+        <v>35356</v>
       </c>
       <c r="AO469" t="s">
         <v>3314</v>
@@ -74890,10 +74913,10 @@
         <v>213</v>
       </c>
       <c r="J470">
-        <v>1082</v>
+        <v>467</v>
       </c>
       <c r="K470">
-        <v>1463</v>
+        <v>631</v>
       </c>
       <c r="L470">
         <v>1082</v>
@@ -74972,6 +74995,9 @@
       </c>
       <c r="AL470" t="s">
         <v>3806</v>
+      </c>
+      <c r="AM470">
+        <v>467</v>
       </c>
       <c r="AO470" t="s">
         <v>3497</v>
@@ -75015,10 +75041,10 @@
         <v>213</v>
       </c>
       <c r="J471">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="K471">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="L471">
         <v>301</v>
@@ -75096,7 +75122,7 @@
         <v>3814</v>
       </c>
       <c r="AM471">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="AO471" t="s">
         <v>3314</v>
@@ -75140,10 +75166,10 @@
         <v>213</v>
       </c>
       <c r="J472">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="K472">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="L472">
         <v>417</v>
@@ -75221,7 +75247,7 @@
         <v>3821</v>
       </c>
       <c r="AM472">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="AO472" t="s">
         <v>3314</v>
@@ -75280,7 +75306,7 @@
         <v>101</v>
       </c>
       <c r="O473">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P473" t="s">
         <v>54</v>
@@ -75396,7 +75422,7 @@
         <v>50</v>
       </c>
       <c r="K474">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L474">
         <v>50</v>
@@ -75521,7 +75547,7 @@
         <v>65</v>
       </c>
       <c r="K475">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L475">
         <v>65</v>
@@ -75658,7 +75684,7 @@
         <v>8028</v>
       </c>
       <c r="O476">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P476" t="s">
         <v>54</v>
@@ -75771,7 +75797,7 @@
         <v>11420</v>
       </c>
       <c r="K477">
-        <v>15433</v>
+        <v>15439</v>
       </c>
       <c r="L477">
         <v>11420</v>
@@ -75902,7 +75928,7 @@
         <v>954</v>
       </c>
       <c r="K478">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="L478">
         <v>954</v>
@@ -76045,7 +76071,7 @@
         <v>1087</v>
       </c>
       <c r="O479">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P479" t="s">
         <v>54</v>
@@ -76170,7 +76196,7 @@
         <v>151</v>
       </c>
       <c r="O480">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P480" t="s">
         <v>54</v>
@@ -76283,7 +76309,7 @@
         <v>892</v>
       </c>
       <c r="K481">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="L481">
         <v>892</v>
@@ -76414,7 +76440,7 @@
         <v>517</v>
       </c>
       <c r="K482">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="L482">
         <v>517</v>
@@ -76557,7 +76583,7 @@
         <v>626</v>
       </c>
       <c r="O483">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P483" t="s">
         <v>54</v>
@@ -76667,7 +76693,7 @@
         <v>190</v>
       </c>
       <c r="K484">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="L484">
         <v>190</v>
@@ -76798,7 +76824,7 @@
         <v>2916</v>
       </c>
       <c r="K485">
-        <v>3941</v>
+        <v>3942</v>
       </c>
       <c r="L485">
         <v>2916</v>
@@ -77191,7 +77217,7 @@
         <v>849</v>
       </c>
       <c r="K488">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="L488">
         <v>849</v>
@@ -77331,7 +77357,7 @@
         <v>229</v>
       </c>
       <c r="O489">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="P489" t="s">
         <v>54</v>
@@ -77447,7 +77473,7 @@
         <v>2968</v>
       </c>
       <c r="K490">
-        <v>4011</v>
+        <v>4012</v>
       </c>
       <c r="L490">
         <v>2968</v>
@@ -77706,7 +77732,7 @@
         <v>258</v>
       </c>
       <c r="K492">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="L492">
         <v>258</v>
@@ -77962,7 +77988,7 @@
         <v>440</v>
       </c>
       <c r="K494">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="L494">
         <v>440</v>
@@ -78090,7 +78116,7 @@
         <v>405</v>
       </c>
       <c r="K495">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="L495">
         <v>405</v>
@@ -78221,7 +78247,7 @@
         <v>923</v>
       </c>
       <c r="K496">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="L496">
         <v>923</v>
@@ -78349,7 +78375,7 @@
         <v>923</v>
       </c>
       <c r="K497">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="L497">
         <v>923</v>
@@ -78480,7 +78506,7 @@
         <v>513</v>
       </c>
       <c r="K498">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="L498">
         <v>513</v>
@@ -78745,7 +78771,7 @@
         <v>9104</v>
       </c>
       <c r="O500">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P500" t="s">
         <v>54</v>
@@ -78858,10 +78884,10 @@
         <v>213</v>
       </c>
       <c r="J501">
-        <v>1155</v>
+        <v>769</v>
       </c>
       <c r="K501">
-        <v>1561</v>
+        <v>1039</v>
       </c>
       <c r="L501">
         <v>1155</v>
@@ -78942,7 +78968,7 @@
         <v>4054</v>
       </c>
       <c r="AM501">
-        <v>1155</v>
+        <v>769</v>
       </c>
       <c r="AO501" t="s">
         <v>3298</v>

</xml_diff>

<commit_message>
Correct catalog dimensions and classifications
</commit_message>
<xml_diff>
--- a/data/catalog_500_exact_match.xlsx
+++ b/data/catalog_500_exact_match.xlsx
@@ -15838,6 +15838,11 @@
       <c r="W3" s="3" t="s">
         <v>80</v>
       </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y3" s="3" t="s">
         <v>59</v>
       </c>
@@ -16457,15 +16462,9 @@
       <c r="S8">
         <v>0.25</v>
       </c>
-      <c r="T8" s="4">
-        <v>140</v>
-      </c>
-      <c r="U8">
-        <v>100</v>
-      </c>
-      <c r="V8">
-        <v>60</v>
-      </c>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
       <c r="W8" t="s">
         <v>145</v>
       </c>
@@ -16955,7 +16954,7 @@
         <v>188</v>
       </c>
       <c r="S12">
-        <v>1.4</v>
+        <v>50</v>
       </c>
       <c r="T12">
         <v>250</v>
@@ -17208,7 +17207,7 @@
         <v>215</v>
       </c>
       <c r="S14">
-        <v>2100</v>
+        <v>2190</v>
       </c>
       <c r="T14">
         <v>460</v>
@@ -17342,13 +17341,13 @@
         <v>226</v>
       </c>
       <c r="S15">
-        <v>2500</v>
+        <v>2680</v>
       </c>
       <c r="T15">
         <v>510</v>
       </c>
       <c r="U15">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="V15">
         <v>230</v>
@@ -17479,10 +17478,10 @@
         <v>0.9</v>
       </c>
       <c r="T16">
-        <v>361.5</v>
+        <v>375</v>
       </c>
       <c r="U16">
-        <v>60</v>
+        <v>280</v>
       </c>
       <c r="V16">
         <v>70</v>
@@ -17607,10 +17606,10 @@
         <v>0.9</v>
       </c>
       <c r="T17">
-        <v>361.5</v>
+        <v>600</v>
       </c>
       <c r="U17">
-        <v>60</v>
+        <v>360</v>
       </c>
       <c r="V17">
         <v>70</v>
@@ -17735,10 +17734,10 @@
         <v>0.9</v>
       </c>
       <c r="T18">
-        <v>361.5</v>
+        <v>380</v>
       </c>
       <c r="U18">
-        <v>60</v>
+        <v>380</v>
       </c>
       <c r="V18">
         <v>70</v>
@@ -17863,10 +17862,10 @@
         <v>0.9</v>
       </c>
       <c r="T19">
-        <v>361.5</v>
+        <v>510</v>
       </c>
       <c r="U19">
-        <v>60</v>
+        <v>460</v>
       </c>
       <c r="V19">
         <v>70</v>
@@ -18622,16 +18621,16 @@
         <v>322</v>
       </c>
       <c r="S25">
-        <v>9.5</v>
+        <v>150</v>
       </c>
       <c r="T25">
         <v>129</v>
       </c>
       <c r="U25">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="V25">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="W25" t="s">
         <v>323</v>
@@ -18759,13 +18758,13 @@
         <v>9.5</v>
       </c>
       <c r="T26">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="U26">
-        <v>35</v>
+        <v>350</v>
       </c>
       <c r="V26">
-        <v>30</v>
+        <v>300</v>
       </c>
       <c r="W26" t="s">
         <v>334</v>
@@ -19262,7 +19261,7 @@
         <v>364</v>
       </c>
       <c r="S30">
-        <v>9.5</v>
+        <v>100</v>
       </c>
       <c r="T30">
         <v>80</v>
@@ -20149,16 +20148,16 @@
         <v>431</v>
       </c>
       <c r="S37">
-        <v>1060</v>
+        <v>1270</v>
       </c>
       <c r="T37">
         <v>340</v>
       </c>
       <c r="U37">
-        <v>340</v>
+        <v>135</v>
       </c>
       <c r="V37">
-        <v>340</v>
+        <v>190</v>
       </c>
       <c r="W37" t="s">
         <v>432</v>
@@ -20283,16 +20282,16 @@
         <v>441</v>
       </c>
       <c r="S38">
-        <v>567.5675</v>
+        <v>1260</v>
       </c>
       <c r="T38">
         <v>340</v>
       </c>
       <c r="U38">
-        <v>340</v>
+        <v>135</v>
       </c>
       <c r="V38">
-        <v>340</v>
+        <v>190</v>
       </c>
       <c r="W38" t="s">
         <v>442</v>
@@ -20417,13 +20416,13 @@
         <v>450</v>
       </c>
       <c r="S39">
-        <v>0.82499999999999996</v>
+        <v>850</v>
       </c>
       <c r="T39">
-        <v>180</v>
+        <v>1800</v>
       </c>
       <c r="U39">
-        <v>19</v>
+        <v>190</v>
       </c>
       <c r="V39">
         <v>61</v>
@@ -20551,7 +20550,7 @@
         <v>461</v>
       </c>
       <c r="S40">
-        <v>392</v>
+        <v>350</v>
       </c>
       <c r="T40">
         <v>200</v>
@@ -20564,6 +20563,11 @@
       </c>
       <c r="W40" t="s">
         <v>462</v>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>8512309009</t>
+        </is>
       </c>
       <c r="Y40" t="s">
         <v>59</v>
@@ -20682,7 +20686,7 @@
         <v>475</v>
       </c>
       <c r="S41">
-        <v>0.7</v>
+        <v>30</v>
       </c>
       <c r="T41">
         <v>180</v>
@@ -20816,7 +20820,7 @@
         <v>487</v>
       </c>
       <c r="S42">
-        <v>96.5</v>
+        <v>410</v>
       </c>
       <c r="T42">
         <v>70</v>
@@ -20950,7 +20954,7 @@
         <v>496</v>
       </c>
       <c r="S43">
-        <v>392</v>
+        <v>30</v>
       </c>
       <c r="T43">
         <v>73</v>
@@ -20963,6 +20967,11 @@
       </c>
       <c r="W43" t="s">
         <v>497</v>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>9405420039</t>
+        </is>
       </c>
       <c r="Y43" t="s">
         <v>59</v>
@@ -21220,6 +21229,11 @@
       <c r="W45" t="s">
         <v>523</v>
       </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>8306100000</t>
+        </is>
+      </c>
       <c r="Y45" t="s">
         <v>59</v>
       </c>
@@ -21709,16 +21723,21 @@
         <v>9.5</v>
       </c>
       <c r="T49">
-        <v>130.5</v>
+        <v>1100</v>
       </c>
       <c r="U49">
-        <v>110</v>
+        <v>240</v>
       </c>
       <c r="V49">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="W49" t="s">
         <v>560</v>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
       </c>
       <c r="Y49" t="s">
         <v>59</v>
@@ -21845,6 +21864,11 @@
       <c r="W50" t="s">
         <v>570</v>
       </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>5607491100</t>
+        </is>
+      </c>
       <c r="Y50" t="s">
         <v>59</v>
       </c>
@@ -21967,6 +21991,11 @@
       <c r="W51" t="s">
         <v>580</v>
       </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>6216000000</t>
+        </is>
+      </c>
       <c r="Y51" t="s">
         <v>59</v>
       </c>
@@ -22075,7 +22104,7 @@
         <v>589</v>
       </c>
       <c r="S52">
-        <v>1.5</v>
+        <v>300</v>
       </c>
       <c r="T52">
         <v>349</v>
@@ -22088,6 +22117,11 @@
       </c>
       <c r="W52" t="s">
         <v>590</v>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
       </c>
       <c r="Y52" t="s">
         <v>59</v>
@@ -22206,16 +22240,16 @@
         <v>599</v>
       </c>
       <c r="S53">
-        <v>1.5</v>
+        <v>1500</v>
       </c>
       <c r="T53">
         <v>380</v>
       </c>
       <c r="U53">
-        <v>36</v>
+        <v>280</v>
       </c>
       <c r="V53">
-        <v>18</v>
+        <v>130</v>
       </c>
       <c r="W53" t="s">
         <v>600</v>
@@ -23979,6 +24013,11 @@
       <c r="W67" t="s">
         <v>691</v>
       </c>
+      <c r="X67" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y67" t="s">
         <v>59</v>
       </c>
@@ -24340,7 +24379,7 @@
         <v>65</v>
       </c>
       <c r="T70">
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="U70">
         <v>140</v>
@@ -24350,6 +24389,11 @@
       </c>
       <c r="W70" t="s">
         <v>713</v>
+      </c>
+      <c r="X70" t="inlineStr">
+        <is>
+          <t>9208900000</t>
+        </is>
       </c>
       <c r="Y70" t="s">
         <v>59</v>
@@ -24476,6 +24520,11 @@
       <c r="W71" t="s">
         <v>722</v>
       </c>
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y71" t="s">
         <v>59</v>
       </c>
@@ -24601,6 +24650,11 @@
       <c r="W72" t="s">
         <v>730</v>
       </c>
+      <c r="X72" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y72" t="s">
         <v>59</v>
       </c>
@@ -24723,6 +24777,11 @@
       <c r="W73" t="s">
         <v>739</v>
       </c>
+      <c r="X73" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y73" t="s">
         <v>59</v>
       </c>
@@ -24845,6 +24904,11 @@
       <c r="W74" t="s">
         <v>745</v>
       </c>
+      <c r="X74" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y74" t="s">
         <v>59</v>
       </c>
@@ -24967,6 +25031,11 @@
       <c r="W75" t="s">
         <v>751</v>
       </c>
+      <c r="X75" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y75" t="s">
         <v>59</v>
       </c>
@@ -25089,6 +25158,11 @@
       <c r="W76" t="s">
         <v>757</v>
       </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y76" t="s">
         <v>59</v>
       </c>
@@ -25211,6 +25285,11 @@
       <c r="W77" t="s">
         <v>763</v>
       </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y77" t="s">
         <v>59</v>
       </c>
@@ -25333,6 +25412,11 @@
       <c r="W78" t="s">
         <v>769</v>
       </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y78" t="s">
         <v>59</v>
       </c>
@@ -25955,6 +26039,11 @@
       <c r="W83" t="s">
         <v>809</v>
       </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y83" t="s">
         <v>59</v>
       </c>
@@ -26083,6 +26172,11 @@
       <c r="W84" t="s">
         <v>819</v>
       </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y84" t="s">
         <v>59</v>
       </c>
@@ -26330,6 +26424,11 @@
       <c r="W86" t="s">
         <v>837</v>
       </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>9405420039</t>
+        </is>
+      </c>
       <c r="Y86" t="s">
         <v>59</v>
       </c>
@@ -26455,6 +26554,11 @@
       <c r="W87" t="s">
         <v>845</v>
       </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>9405420039</t>
+        </is>
+      </c>
       <c r="Y87" t="s">
         <v>59</v>
       </c>
@@ -26577,6 +26681,11 @@
       <c r="W88" t="s">
         <v>852</v>
       </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>9208900000</t>
+        </is>
+      </c>
       <c r="Y88" t="s">
         <v>59</v>
       </c>
@@ -26699,6 +26808,11 @@
       <c r="W89" t="s">
         <v>860</v>
       </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y89" t="s">
         <v>59</v>
       </c>
@@ -26821,6 +26935,11 @@
       <c r="W90" t="s">
         <v>867</v>
       </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y90" t="s">
         <v>59</v>
       </c>
@@ -27054,7 +27173,7 @@
         <v>882</v>
       </c>
       <c r="S92">
-        <v>11.7</v>
+        <v>11700</v>
       </c>
       <c r="T92">
         <v>100</v>
@@ -27321,6 +27440,11 @@
       <c r="W94" t="s">
         <v>901</v>
       </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>8536908500</t>
+        </is>
+      </c>
       <c r="Y94" t="s">
         <v>59</v>
       </c>
@@ -27443,6 +27567,11 @@
       <c r="W95" t="s">
         <v>910</v>
       </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>8536109000</t>
+        </is>
+      </c>
       <c r="Y95" t="s">
         <v>59</v>
       </c>
@@ -27565,6 +27694,11 @@
       <c r="W96" t="s">
         <v>918</v>
       </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>8536109000</t>
+        </is>
+      </c>
       <c r="Y96" t="s">
         <v>59</v>
       </c>
@@ -27687,6 +27821,11 @@
       <c r="W97" t="s">
         <v>926</v>
       </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>8536109000</t>
+        </is>
+      </c>
       <c r="Y97" t="s">
         <v>59</v>
       </c>
@@ -27809,6 +27948,11 @@
       <c r="W98" t="s">
         <v>934</v>
       </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>8536109000</t>
+        </is>
+      </c>
       <c r="Y98" t="s">
         <v>59</v>
       </c>
@@ -27917,13 +28061,13 @@
         <v>945</v>
       </c>
       <c r="S99">
-        <v>0.25</v>
+        <v>730</v>
       </c>
       <c r="T99">
         <v>48</v>
       </c>
       <c r="U99">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="V99">
         <v>48</v>
@@ -28051,7 +28195,7 @@
         <v>957</v>
       </c>
       <c r="S100">
-        <v>1.4</v>
+        <v>120</v>
       </c>
       <c r="T100">
         <v>250</v>
@@ -28196,6 +28340,11 @@
       <c r="W101" t="s">
         <v>967</v>
       </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>6216000000</t>
+        </is>
+      </c>
       <c r="Y101" t="s">
         <v>59</v>
       </c>
@@ -34446,6 +34595,11 @@
       <c r="W151" t="s">
         <v>1320</v>
       </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>8413603900</t>
+        </is>
+      </c>
       <c r="Y151" t="s">
         <v>59</v>
       </c>
@@ -34693,6 +34847,11 @@
       <c r="W153" t="s">
         <v>1335</v>
       </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>8413810000</t>
+        </is>
+      </c>
       <c r="Y153" t="s">
         <v>59</v>
       </c>
@@ -35077,6 +35236,11 @@
       <c r="W156" t="s">
         <v>1366</v>
       </c>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y156" t="s">
         <v>59</v>
       </c>
@@ -35574,6 +35738,11 @@
       <c r="W160" t="s">
         <v>1393</v>
       </c>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y160" t="s">
         <v>59</v>
       </c>
@@ -36196,6 +36365,11 @@
       <c r="W165" t="s">
         <v>1435</v>
       </c>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y165" t="s">
         <v>59</v>
       </c>
@@ -36318,6 +36492,11 @@
       <c r="W166" t="s">
         <v>1445</v>
       </c>
+      <c r="X166" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y166" t="s">
         <v>59</v>
       </c>
@@ -36440,6 +36619,11 @@
       <c r="W167" t="s">
         <v>1455</v>
       </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y167" t="s">
         <v>59</v>
       </c>
@@ -36562,6 +36746,11 @@
       <c r="W168" t="s">
         <v>1465</v>
       </c>
+      <c r="X168" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y168" t="s">
         <v>59</v>
       </c>
@@ -36684,6 +36873,11 @@
       <c r="W169" t="s">
         <v>1477</v>
       </c>
+      <c r="X169" t="inlineStr">
+        <is>
+          <t>8536109000</t>
+        </is>
+      </c>
       <c r="Y169" t="s">
         <v>59</v>
       </c>
@@ -38342,6 +38536,11 @@
       <c r="W182" t="s">
         <v>1585</v>
       </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>7616999008</t>
+        </is>
+      </c>
       <c r="Y182" t="s">
         <v>59</v>
       </c>
@@ -38467,6 +38666,11 @@
       <c r="W183" t="s">
         <v>1594</v>
       </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y183" t="s">
         <v>59</v>
       </c>
@@ -38589,6 +38793,11 @@
       <c r="W184" t="s">
         <v>1603</v>
       </c>
+      <c r="X184" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y184" t="s">
         <v>59</v>
       </c>
@@ -39086,6 +39295,11 @@
       <c r="W188" t="s">
         <v>1638</v>
       </c>
+      <c r="X188" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y188" t="s">
         <v>59</v>
       </c>
@@ -39211,6 +39425,11 @@
       <c r="W189" t="s">
         <v>1648</v>
       </c>
+      <c r="X189" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y189" t="s">
         <v>59</v>
       </c>
@@ -40330,6 +40549,11 @@
       <c r="W198" t="s">
         <v>1722</v>
       </c>
+      <c r="X198" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y198" t="s">
         <v>59</v>
       </c>
@@ -40452,6 +40676,11 @@
       <c r="W199" t="s">
         <v>1729</v>
       </c>
+      <c r="X199" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y199" t="s">
         <v>59</v>
       </c>
@@ -40699,6 +40928,11 @@
       <c r="W201" t="s">
         <v>1745</v>
       </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>7616999008</t>
+        </is>
+      </c>
       <c r="Y201" t="s">
         <v>59</v>
       </c>
@@ -40824,6 +41058,11 @@
       <c r="W202" t="s">
         <v>1753</v>
       </c>
+      <c r="X202" t="inlineStr">
+        <is>
+          <t>8536908500</t>
+        </is>
+      </c>
       <c r="Y202" t="s">
         <v>59</v>
       </c>
@@ -40946,6 +41185,11 @@
       <c r="W203" t="s">
         <v>1760</v>
       </c>
+      <c r="X203" t="inlineStr">
+        <is>
+          <t>8536908500</t>
+        </is>
+      </c>
       <c r="Y203" t="s">
         <v>59</v>
       </c>
@@ -41068,6 +41312,11 @@
       <c r="W204" t="s">
         <v>1766</v>
       </c>
+      <c r="X204" t="inlineStr">
+        <is>
+          <t>8414598000</t>
+        </is>
+      </c>
       <c r="Y204" t="s">
         <v>59</v>
       </c>
@@ -41312,6 +41561,11 @@
       <c r="W206" t="s">
         <v>1780</v>
       </c>
+      <c r="X206" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y206" t="s">
         <v>59</v>
       </c>
@@ -41437,6 +41691,11 @@
       <c r="W207" t="s">
         <v>1788</v>
       </c>
+      <c r="X207" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y207" t="s">
         <v>59</v>
       </c>
@@ -42071,6 +42330,11 @@
       <c r="W212" t="s">
         <v>1831</v>
       </c>
+      <c r="X212" t="inlineStr">
+        <is>
+          <t>3924100000</t>
+        </is>
+      </c>
       <c r="Y212" t="s">
         <v>59</v>
       </c>
@@ -42193,6 +42457,11 @@
       <c r="W213" t="s">
         <v>1837</v>
       </c>
+      <c r="X213" t="inlineStr">
+        <is>
+          <t>3924100000</t>
+        </is>
+      </c>
       <c r="Y213" t="s">
         <v>59</v>
       </c>
@@ -42315,6 +42584,11 @@
       <c r="W214" t="s">
         <v>1843</v>
       </c>
+      <c r="X214" t="inlineStr">
+        <is>
+          <t>3924100000</t>
+        </is>
+      </c>
       <c r="Y214" t="s">
         <v>59</v>
       </c>
@@ -42437,6 +42711,11 @@
       <c r="W215" t="s">
         <v>1849</v>
       </c>
+      <c r="X215" t="inlineStr">
+        <is>
+          <t>3924100000</t>
+        </is>
+      </c>
       <c r="Y215" t="s">
         <v>59</v>
       </c>
@@ -42559,6 +42838,11 @@
       <c r="W216" t="s">
         <v>1855</v>
       </c>
+      <c r="X216" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y216" t="s">
         <v>59</v>
       </c>
@@ -43434,6 +43718,11 @@
       <c r="W223" t="s">
         <v>1914</v>
       </c>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>9031809800</t>
+        </is>
+      </c>
       <c r="Y223" t="s">
         <v>59</v>
       </c>
@@ -43556,6 +43845,11 @@
       <c r="W224" t="s">
         <v>1923</v>
       </c>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>7616999008</t>
+        </is>
+      </c>
       <c r="Y224" t="s">
         <v>59</v>
       </c>
@@ -44565,6 +44859,11 @@
       <c r="W232" t="s">
         <v>1989</v>
       </c>
+      <c r="X232" t="inlineStr">
+        <is>
+          <t>6216000000</t>
+        </is>
+      </c>
       <c r="Y232" t="s">
         <v>59</v>
       </c>
@@ -44687,6 +44986,11 @@
       <c r="W233" t="s">
         <v>1993</v>
       </c>
+      <c r="X233" t="inlineStr">
+        <is>
+          <t>6216000000</t>
+        </is>
+      </c>
       <c r="Y233" t="s">
         <v>59</v>
       </c>
@@ -44809,6 +45113,11 @@
       <c r="W234" t="s">
         <v>1999</v>
       </c>
+      <c r="X234" t="inlineStr">
+        <is>
+          <t>9026108900</t>
+        </is>
+      </c>
       <c r="Y234" t="s">
         <v>59</v>
       </c>
@@ -44931,6 +45240,11 @@
       <c r="W235" t="s">
         <v>2009</v>
       </c>
+      <c r="X235" t="inlineStr">
+        <is>
+          <t>9026108900</t>
+        </is>
+      </c>
       <c r="Y235" t="s">
         <v>59</v>
       </c>
@@ -45053,6 +45367,11 @@
       <c r="W236" t="s">
         <v>2016</v>
       </c>
+      <c r="X236" t="inlineStr">
+        <is>
+          <t>9104000000</t>
+        </is>
+      </c>
       <c r="Y236" t="s">
         <v>59</v>
       </c>
@@ -47172,6 +47491,11 @@
       <c r="W253" t="s">
         <v>2143</v>
       </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>7616999008</t>
+        </is>
+      </c>
       <c r="Y253" t="s">
         <v>59</v>
       </c>
@@ -47672,6 +47996,11 @@
       <c r="W257" t="s">
         <v>2170</v>
       </c>
+      <c r="X257" t="inlineStr">
+        <is>
+          <t>5607491100</t>
+        </is>
+      </c>
       <c r="Y257" t="s">
         <v>59</v>
       </c>
@@ -47794,6 +48123,11 @@
       <c r="W258" t="s">
         <v>2177</v>
       </c>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>5607491100</t>
+        </is>
+      </c>
       <c r="Y258" t="s">
         <v>59</v>
       </c>
@@ -48812,6 +49146,11 @@
       <c r="W266" t="s">
         <v>2242</v>
       </c>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y266" t="s">
         <v>59</v>
       </c>
@@ -49184,6 +49523,11 @@
       <c r="W269" t="s">
         <v>2262</v>
       </c>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>5607491100</t>
+        </is>
+      </c>
       <c r="Y269" t="s">
         <v>59</v>
       </c>
@@ -50059,6 +50403,11 @@
       <c r="W276" t="s">
         <v>2315</v>
       </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y276" t="s">
         <v>59</v>
       </c>
@@ -50181,6 +50530,11 @@
       <c r="W277" t="s">
         <v>2322</v>
       </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y277" t="s">
         <v>59</v>
       </c>
@@ -50303,6 +50657,11 @@
       <c r="W278" t="s">
         <v>2328</v>
       </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y278" t="s">
         <v>59</v>
       </c>
@@ -50425,6 +50784,11 @@
       <c r="W279" t="s">
         <v>2334</v>
       </c>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y279" t="s">
         <v>59</v>
       </c>
@@ -50550,6 +50914,11 @@
       <c r="W280" t="s">
         <v>2343</v>
       </c>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>9405420039</t>
+        </is>
+      </c>
       <c r="Y280" t="s">
         <v>59</v>
       </c>
@@ -53062,6 +53431,11 @@
       <c r="W300" t="s">
         <v>2501</v>
       </c>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>8536699008</t>
+        </is>
+      </c>
       <c r="Y300" t="s">
         <v>59</v>
       </c>
@@ -53187,6 +53561,11 @@
       <c r="W301" t="s">
         <v>2510</v>
       </c>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>9405420039</t>
+        </is>
+      </c>
       <c r="Y301" t="s">
         <v>59</v>
       </c>
@@ -53449,6 +53828,11 @@
       <c r="W303" t="s">
         <v>2531</v>
       </c>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>8536508008</t>
+        </is>
+      </c>
       <c r="Y303" t="s">
         <v>59</v>
       </c>
@@ -55247,6 +55631,11 @@
       <c r="W317" t="s">
         <v>2643</v>
       </c>
+      <c r="X317" t="inlineStr">
+        <is>
+          <t>8536699008</t>
+        </is>
+      </c>
       <c r="Y317" t="s">
         <v>59</v>
       </c>
@@ -55369,6 +55758,11 @@
       <c r="W318" t="s">
         <v>2651</v>
       </c>
+      <c r="X318" t="inlineStr">
+        <is>
+          <t>3923301090</t>
+        </is>
+      </c>
       <c r="Y318" t="s">
         <v>59</v>
       </c>
@@ -55625,6 +56019,11 @@
       <c r="W320" t="s">
         <v>2667</v>
       </c>
+      <c r="X320" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y320" t="s">
         <v>59</v>
       </c>
@@ -55881,6 +56280,11 @@
       <c r="W322" t="s">
         <v>2684</v>
       </c>
+      <c r="X322" t="inlineStr">
+        <is>
+          <t>7616999008</t>
+        </is>
+      </c>
       <c r="Y322" t="s">
         <v>59</v>
       </c>
@@ -56012,6 +56416,11 @@
       <c r="W323" t="s">
         <v>2693</v>
       </c>
+      <c r="X323" t="inlineStr">
+        <is>
+          <t>7616999008</t>
+        </is>
+      </c>
       <c r="Y323" t="s">
         <v>59</v>
       </c>
@@ -56143,6 +56552,11 @@
       <c r="W324" t="s">
         <v>2702</v>
       </c>
+      <c r="X324" t="inlineStr">
+        <is>
+          <t>3923301090</t>
+        </is>
+      </c>
       <c r="Y324" t="s">
         <v>59</v>
       </c>
@@ -56274,6 +56688,11 @@
       <c r="W325" t="s">
         <v>2711</v>
       </c>
+      <c r="X325" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y325" t="s">
         <v>59</v>
       </c>
@@ -56405,6 +56824,11 @@
       <c r="W326" t="s">
         <v>2718</v>
       </c>
+      <c r="X326" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y326" t="s">
         <v>59</v>
       </c>
@@ -56533,6 +56957,11 @@
       <c r="W327" t="s">
         <v>2727</v>
       </c>
+      <c r="X327" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y327" t="s">
         <v>59</v>
       </c>
@@ -56661,6 +57090,11 @@
       <c r="W328" t="s">
         <v>2734</v>
       </c>
+      <c r="X328" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y328" t="s">
         <v>59</v>
       </c>
@@ -56792,6 +57226,11 @@
       <c r="W329" t="s">
         <v>2742</v>
       </c>
+      <c r="X329" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y329" t="s">
         <v>59</v>
       </c>
@@ -56923,6 +57362,11 @@
       <c r="W330" t="s">
         <v>2749</v>
       </c>
+      <c r="X330" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y330" t="s">
         <v>59</v>
       </c>
@@ -57319,6 +57763,11 @@
       <c r="W333" t="s">
         <v>2771</v>
       </c>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y333" t="s">
         <v>59</v>
       </c>
@@ -57450,6 +57899,11 @@
       <c r="W334" t="s">
         <v>2780</v>
       </c>
+      <c r="X334" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y334" t="s">
         <v>59</v>
       </c>
@@ -57581,6 +58035,11 @@
       <c r="W335" t="s">
         <v>2788</v>
       </c>
+      <c r="X335" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y335" t="s">
         <v>59</v>
       </c>
@@ -57709,6 +58168,11 @@
       <c r="W336" t="s">
         <v>2795</v>
       </c>
+      <c r="X336" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y336" t="s">
         <v>59</v>
       </c>
@@ -57840,6 +58304,11 @@
       <c r="W337" t="s">
         <v>2803</v>
       </c>
+      <c r="X337" t="inlineStr">
+        <is>
+          <t>8536699008</t>
+        </is>
+      </c>
       <c r="Y337" t="s">
         <v>59</v>
       </c>
@@ -57968,6 +58437,11 @@
       <c r="W338" t="s">
         <v>2811</v>
       </c>
+      <c r="X338" t="inlineStr">
+        <is>
+          <t>8537109800</t>
+        </is>
+      </c>
       <c r="Y338" t="s">
         <v>59</v>
       </c>
@@ -58099,6 +58573,11 @@
       <c r="W339" t="s">
         <v>2818</v>
       </c>
+      <c r="X339" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y339" t="s">
         <v>59</v>
       </c>
@@ -58230,6 +58709,11 @@
       <c r="W340" t="s">
         <v>2827</v>
       </c>
+      <c r="X340" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y340" t="s">
         <v>59</v>
       </c>
@@ -58358,6 +58842,11 @@
       <c r="W341" t="s">
         <v>2835</v>
       </c>
+      <c r="X341" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y341" t="s">
         <v>59</v>
       </c>
@@ -58489,6 +58978,11 @@
       <c r="W342" t="s">
         <v>2843</v>
       </c>
+      <c r="X342" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y342" t="s">
         <v>59</v>
       </c>
@@ -58620,6 +59114,11 @@
       <c r="W343" t="s">
         <v>2851</v>
       </c>
+      <c r="X343" t="inlineStr">
+        <is>
+          <t>5607491100</t>
+        </is>
+      </c>
       <c r="Y343" t="s">
         <v>59</v>
       </c>
@@ -58751,6 +59250,11 @@
       <c r="W344" t="s">
         <v>2860</v>
       </c>
+      <c r="X344" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y344" t="s">
         <v>59</v>
       </c>
@@ -58879,6 +59383,11 @@
       <c r="W345" t="s">
         <v>2873</v>
       </c>
+      <c r="X345" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y345" t="s">
         <v>59</v>
       </c>
@@ -59007,6 +59516,11 @@
       <c r="W346" t="s">
         <v>2882</v>
       </c>
+      <c r="X346" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y346" t="s">
         <v>59</v>
       </c>
@@ -59138,6 +59652,11 @@
       <c r="W347" t="s">
         <v>2890</v>
       </c>
+      <c r="X347" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y347" t="s">
         <v>59</v>
       </c>
@@ -59269,6 +59788,11 @@
       <c r="W348" t="s">
         <v>2898</v>
       </c>
+      <c r="X348" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y348" t="s">
         <v>59</v>
       </c>
@@ -59659,6 +60183,11 @@
       <c r="W351" t="s">
         <v>2924</v>
       </c>
+      <c r="X351" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y351" t="s">
         <v>59</v>
       </c>
@@ -59781,6 +60310,11 @@
       <c r="W352" t="s">
         <v>2931</v>
       </c>
+      <c r="X352" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y352" t="s">
         <v>59</v>
       </c>
@@ -60034,6 +60568,11 @@
       <c r="W354" t="s">
         <v>2948</v>
       </c>
+      <c r="X354" t="inlineStr">
+        <is>
+          <t>8479899707</t>
+        </is>
+      </c>
       <c r="Y354" t="s">
         <v>59</v>
       </c>
@@ -61222,6 +61761,11 @@
       <c r="W363" t="s">
         <v>3023</v>
       </c>
+      <c r="X363" t="inlineStr">
+        <is>
+          <t>7318158900</t>
+        </is>
+      </c>
       <c r="Y363" t="s">
         <v>59</v>
       </c>
@@ -62288,6 +62832,11 @@
       <c r="W371" t="s">
         <v>3088</v>
       </c>
+      <c r="X371" t="inlineStr">
+        <is>
+          <t>9026108900</t>
+        </is>
+      </c>
       <c r="Y371" t="s">
         <v>59</v>
       </c>
@@ -62419,6 +62968,11 @@
       <c r="W372" t="s">
         <v>3096</v>
       </c>
+      <c r="X372" t="inlineStr">
+        <is>
+          <t>8536699008</t>
+        </is>
+      </c>
       <c r="Y372" t="s">
         <v>59</v>
       </c>
@@ -62547,6 +63101,11 @@
       <c r="W373" t="s">
         <v>3104</v>
       </c>
+      <c r="X373" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y373" t="s">
         <v>59</v>
       </c>
@@ -62672,6 +63231,11 @@
       <c r="W374" t="s">
         <v>3109</v>
       </c>
+      <c r="X374" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y374" t="s">
         <v>59</v>
       </c>
@@ -62797,6 +63361,11 @@
       <c r="W375" t="s">
         <v>3114</v>
       </c>
+      <c r="X375" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y375" t="s">
         <v>59</v>
       </c>
@@ -62919,6 +63488,11 @@
       <c r="W376" t="s">
         <v>3122</v>
       </c>
+      <c r="X376" t="inlineStr">
+        <is>
+          <t>9026108900</t>
+        </is>
+      </c>
       <c r="Y376" t="s">
         <v>59</v>
       </c>
@@ -63047,6 +63621,11 @@
       <c r="W377" t="s">
         <v>3131</v>
       </c>
+      <c r="X377" t="inlineStr">
+        <is>
+          <t>9030339900</t>
+        </is>
+      </c>
       <c r="Y377" t="s">
         <v>59</v>
       </c>
@@ -63175,6 +63754,11 @@
       <c r="W378" t="s">
         <v>3138</v>
       </c>
+      <c r="X378" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y378" t="s">
         <v>59</v>
       </c>
@@ -63303,6 +63887,11 @@
       <c r="W379" t="s">
         <v>3145</v>
       </c>
+      <c r="X379" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y379" t="s">
         <v>59</v>
       </c>
@@ -63428,6 +64017,11 @@
       <c r="W380" t="s">
         <v>3151</v>
       </c>
+      <c r="X380" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y380" t="s">
         <v>59</v>
       </c>
@@ -63556,6 +64150,11 @@
       <c r="W381" t="s">
         <v>3158</v>
       </c>
+      <c r="X381" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y381" t="s">
         <v>59</v>
       </c>
@@ -63684,6 +64283,11 @@
       <c r="W382" t="s">
         <v>3165</v>
       </c>
+      <c r="X382" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y382" t="s">
         <v>59</v>
       </c>
@@ -63812,6 +64416,11 @@
       <c r="W383" t="s">
         <v>3174</v>
       </c>
+      <c r="X383" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y383" t="s">
         <v>59</v>
       </c>
@@ -64065,6 +64674,11 @@
       <c r="W385" t="s">
         <v>3188</v>
       </c>
+      <c r="X385" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y385" t="s">
         <v>59</v>
       </c>
@@ -64190,6 +64804,11 @@
       <c r="W386" t="s">
         <v>3192</v>
       </c>
+      <c r="X386" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y386" t="s">
         <v>59</v>
       </c>
@@ -64315,6 +64934,11 @@
       <c r="W387" t="s">
         <v>3196</v>
       </c>
+      <c r="X387" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y387" t="s">
         <v>59</v>
       </c>
@@ -64440,6 +65064,11 @@
       <c r="W388" t="s">
         <v>3202</v>
       </c>
+      <c r="X388" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y388" t="s">
         <v>59</v>
       </c>
@@ -64693,6 +65322,11 @@
       <c r="W390" t="s">
         <v>3220</v>
       </c>
+      <c r="X390" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y390" t="s">
         <v>59</v>
       </c>
@@ -64824,6 +65458,11 @@
       <c r="W391" t="s">
         <v>3228</v>
       </c>
+      <c r="X391" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y391" t="s">
         <v>59</v>
       </c>
@@ -64955,6 +65594,11 @@
       <c r="W392" t="s">
         <v>3235</v>
       </c>
+      <c r="X392" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y392" t="s">
         <v>59</v>
       </c>
@@ -65086,6 +65730,11 @@
       <c r="W393" t="s">
         <v>3244</v>
       </c>
+      <c r="X393" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y393" t="s">
         <v>59</v>
       </c>
@@ -65217,6 +65866,11 @@
       <c r="W394" t="s">
         <v>3253</v>
       </c>
+      <c r="X394" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y394" t="s">
         <v>59</v>
       </c>
@@ -65348,6 +66002,11 @@
       <c r="W395" t="s">
         <v>3262</v>
       </c>
+      <c r="X395" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y395" t="s">
         <v>59</v>
       </c>
@@ -65476,6 +66135,11 @@
       <c r="W396" t="s">
         <v>3268</v>
       </c>
+      <c r="X396" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y396" t="s">
         <v>59</v>
       </c>
@@ -65607,6 +66271,11 @@
       <c r="W397" t="s">
         <v>3275</v>
       </c>
+      <c r="X397" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y397" t="s">
         <v>59</v>
       </c>
@@ -65735,6 +66404,11 @@
       <c r="W398" t="s">
         <v>3282</v>
       </c>
+      <c r="X398" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y398" t="s">
         <v>59</v>
       </c>
@@ -65866,6 +66540,11 @@
       <c r="W399" t="s">
         <v>3290</v>
       </c>
+      <c r="X399" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y399" t="s">
         <v>59</v>
       </c>
@@ -66265,6 +66944,11 @@
       <c r="W402" t="s">
         <v>3313</v>
       </c>
+      <c r="X402" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y402" t="s">
         <v>59</v>
       </c>
@@ -66795,6 +67479,11 @@
       <c r="W406" t="s">
         <v>3345</v>
       </c>
+      <c r="X406" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y406" t="s">
         <v>59</v>
       </c>
@@ -66923,6 +67612,11 @@
       <c r="W407" t="s">
         <v>3353</v>
       </c>
+      <c r="X407" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y407" t="s">
         <v>59</v>
       </c>
@@ -67051,6 +67745,11 @@
       <c r="W408" t="s">
         <v>3359</v>
       </c>
+      <c r="X408" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y408" t="s">
         <v>59</v>
       </c>
@@ -67310,6 +68009,11 @@
       <c r="W410" t="s">
         <v>3372</v>
       </c>
+      <c r="X410" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y410" t="s">
         <v>59</v>
       </c>
@@ -67438,6 +68142,11 @@
       <c r="W411" t="s">
         <v>3381</v>
       </c>
+      <c r="X411" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y411" t="s">
         <v>59</v>
       </c>
@@ -67700,6 +68409,11 @@
       <c r="W413" t="s">
         <v>3395</v>
       </c>
+      <c r="X413" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y413" t="s">
         <v>59</v>
       </c>
@@ -67959,6 +68673,11 @@
       <c r="W415" t="s">
         <v>3410</v>
       </c>
+      <c r="X415" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y415" t="s">
         <v>59</v>
       </c>
@@ -68090,6 +68809,11 @@
       <c r="W416" t="s">
         <v>3418</v>
       </c>
+      <c r="X416" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y416" t="s">
         <v>59</v>
       </c>
@@ -68218,6 +68942,11 @@
       <c r="W417" t="s">
         <v>3425</v>
       </c>
+      <c r="X417" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y417" t="s">
         <v>59</v>
       </c>
@@ -68346,6 +69075,11 @@
       <c r="W418" t="s">
         <v>3432</v>
       </c>
+      <c r="X418" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y418" t="s">
         <v>59</v>
       </c>
@@ -68477,6 +69211,11 @@
       <c r="W419" t="s">
         <v>3439</v>
       </c>
+      <c r="X419" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y419" t="s">
         <v>59</v>
       </c>
@@ -68608,6 +69347,11 @@
       <c r="W420" t="s">
         <v>3445</v>
       </c>
+      <c r="X420" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y420" t="s">
         <v>59</v>
       </c>
@@ -68739,6 +69483,11 @@
       <c r="W421" t="s">
         <v>3451</v>
       </c>
+      <c r="X421" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y421" t="s">
         <v>59</v>
       </c>
@@ -68870,6 +69619,11 @@
       <c r="W422" t="s">
         <v>3457</v>
       </c>
+      <c r="X422" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y422" t="s">
         <v>59</v>
       </c>
@@ -69391,6 +70145,11 @@
       <c r="W426" t="s">
         <v>3488</v>
       </c>
+      <c r="X426" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y426" t="s">
         <v>59</v>
       </c>
@@ -70671,6 +71430,11 @@
       <c r="W436" t="s">
         <v>3559</v>
       </c>
+      <c r="X436" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y436" t="s">
         <v>59</v>
       </c>
@@ -71055,6 +71819,11 @@
       <c r="W439" t="s">
         <v>3582</v>
       </c>
+      <c r="X439" t="inlineStr">
+        <is>
+          <t>7318220008</t>
+        </is>
+      </c>
       <c r="Y439" t="s">
         <v>59</v>
       </c>
@@ -71183,6 +71952,11 @@
       <c r="W440" t="s">
         <v>3591</v>
       </c>
+      <c r="X440" t="inlineStr">
+        <is>
+          <t>8512309009</t>
+        </is>
+      </c>
       <c r="Y440" t="s">
         <v>59</v>
       </c>
@@ -71308,6 +72082,11 @@
       <c r="W441" t="s">
         <v>3599</v>
       </c>
+      <c r="X441" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y441" t="s">
         <v>59</v>
       </c>
@@ -71436,6 +72215,11 @@
       <c r="W442" t="s">
         <v>3606</v>
       </c>
+      <c r="X442" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y442" t="s">
         <v>59</v>
       </c>
@@ -71814,6 +72598,11 @@
       <c r="W445" t="s">
         <v>3629</v>
       </c>
+      <c r="X445" t="inlineStr">
+        <is>
+          <t>7318158900</t>
+        </is>
+      </c>
       <c r="Y445" t="s">
         <v>59</v>
       </c>
@@ -71936,6 +72725,11 @@
       <c r="W446" t="s">
         <v>3634</v>
       </c>
+      <c r="X446" t="inlineStr">
+        <is>
+          <t>7318158900</t>
+        </is>
+      </c>
       <c r="Y446" t="s">
         <v>59</v>
       </c>
@@ -72061,6 +72855,11 @@
       <c r="W447" t="s">
         <v>3640</v>
       </c>
+      <c r="X447" t="inlineStr">
+        <is>
+          <t>7318169109</t>
+        </is>
+      </c>
       <c r="Y447" t="s">
         <v>59</v>
       </c>
@@ -72189,6 +72988,11 @@
       <c r="W448" t="s">
         <v>3646</v>
       </c>
+      <c r="X448" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y448" t="s">
         <v>59</v>
       </c>
@@ -72311,6 +73115,11 @@
       <c r="W449" t="s">
         <v>3653</v>
       </c>
+      <c r="X449" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y449" t="s">
         <v>59</v>
       </c>
@@ -72436,6 +73245,11 @@
       <c r="W450" t="s">
         <v>3660</v>
       </c>
+      <c r="X450" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y450" t="s">
         <v>59</v>
       </c>
@@ -72564,6 +73378,11 @@
       <c r="W451" t="s">
         <v>3667</v>
       </c>
+      <c r="X451" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y451" t="s">
         <v>59</v>
       </c>
@@ -72686,6 +73505,11 @@
       <c r="W452" t="s">
         <v>3674</v>
       </c>
+      <c r="X452" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y452" t="s">
         <v>59</v>
       </c>
@@ -72945,6 +73769,11 @@
       <c r="W454" t="s">
         <v>3688</v>
       </c>
+      <c r="X454" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y454" t="s">
         <v>59</v>
       </c>
@@ -73067,6 +73896,11 @@
       <c r="W455" t="s">
         <v>3696</v>
       </c>
+      <c r="X455" t="inlineStr">
+        <is>
+          <t>8484900000</t>
+        </is>
+      </c>
       <c r="Y455" t="s">
         <v>59</v>
       </c>
@@ -73195,6 +74029,11 @@
       <c r="W456" t="s">
         <v>3703</v>
       </c>
+      <c r="X456" t="inlineStr">
+        <is>
+          <t>8484900000</t>
+        </is>
+      </c>
       <c r="Y456" t="s">
         <v>59</v>
       </c>
@@ -73320,6 +74159,11 @@
       <c r="W457" t="s">
         <v>3710</v>
       </c>
+      <c r="X457" t="inlineStr">
+        <is>
+          <t>8484900000</t>
+        </is>
+      </c>
       <c r="Y457" t="s">
         <v>59</v>
       </c>
@@ -73445,6 +74289,11 @@
       <c r="W458" t="s">
         <v>3717</v>
       </c>
+      <c r="X458" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y458" t="s">
         <v>59</v>
       </c>
@@ -73698,6 +74547,11 @@
       <c r="W460" t="s">
         <v>3733</v>
       </c>
+      <c r="X460" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y460" t="s">
         <v>59</v>
       </c>
@@ -73823,6 +74677,11 @@
       <c r="W461" t="s">
         <v>3740</v>
       </c>
+      <c r="X461" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y461" t="s">
         <v>59</v>
       </c>
@@ -73948,6 +74807,11 @@
       <c r="W462" t="s">
         <v>3747</v>
       </c>
+      <c r="X462" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y462" t="s">
         <v>59</v>
       </c>
@@ -74579,6 +75443,11 @@
       <c r="W467" t="s">
         <v>3784</v>
       </c>
+      <c r="X467" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y467" t="s">
         <v>59</v>
       </c>
@@ -74704,6 +75573,11 @@
       <c r="W468" t="s">
         <v>3790</v>
       </c>
+      <c r="X468" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y468" t="s">
         <v>59</v>
       </c>
@@ -75082,6 +75956,11 @@
       <c r="W471" t="s">
         <v>3813</v>
       </c>
+      <c r="X471" t="inlineStr">
+        <is>
+          <t>8421230000</t>
+        </is>
+      </c>
       <c r="Y471" t="s">
         <v>59</v>
       </c>
@@ -75207,6 +76086,11 @@
       <c r="W472" t="s">
         <v>3820</v>
       </c>
+      <c r="X472" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y472" t="s">
         <v>59</v>
       </c>
@@ -75460,6 +76344,11 @@
       <c r="W474" t="s">
         <v>3836</v>
       </c>
+      <c r="X474" t="inlineStr">
+        <is>
+          <t>7318220008</t>
+        </is>
+      </c>
       <c r="Y474" t="s">
         <v>59</v>
       </c>
@@ -75585,6 +76474,11 @@
       <c r="W475" t="s">
         <v>3843</v>
       </c>
+      <c r="X475" t="inlineStr">
+        <is>
+          <t>7318240008</t>
+        </is>
+      </c>
       <c r="Y475" t="s">
         <v>59</v>
       </c>
@@ -75710,6 +76604,11 @@
       <c r="W476" t="s">
         <v>3851</v>
       </c>
+      <c r="X476" t="inlineStr">
+        <is>
+          <t>8512400009</t>
+        </is>
+      </c>
       <c r="Y476" t="s">
         <v>59</v>
       </c>
@@ -75835,6 +76734,11 @@
       <c r="W477" t="s">
         <v>3860</v>
       </c>
+      <c r="X477" t="inlineStr">
+        <is>
+          <t>8409910008</t>
+        </is>
+      </c>
       <c r="Y477" t="s">
         <v>59</v>
       </c>
@@ -75966,6 +76870,11 @@
       <c r="W478" t="s">
         <v>3868</v>
       </c>
+      <c r="X478" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y478" t="s">
         <v>59</v>
       </c>
@@ -76097,6 +77006,11 @@
       <c r="W479" t="s">
         <v>3877</v>
       </c>
+      <c r="X479" t="inlineStr">
+        <is>
+          <t>7318240008</t>
+        </is>
+      </c>
       <c r="Y479" t="s">
         <v>59</v>
       </c>
@@ -76347,6 +77261,11 @@
       <c r="W481" t="s">
         <v>3894</v>
       </c>
+      <c r="X481" t="inlineStr">
+        <is>
+          <t>8536699008</t>
+        </is>
+      </c>
       <c r="Y481" t="s">
         <v>59</v>
       </c>
@@ -76478,6 +77397,11 @@
       <c r="W482" t="s">
         <v>3902</v>
       </c>
+      <c r="X482" t="inlineStr">
+        <is>
+          <t>8536699008</t>
+        </is>
+      </c>
       <c r="Y482" t="s">
         <v>59</v>
       </c>
@@ -76609,6 +77533,11 @@
       <c r="W483" t="s">
         <v>3910</v>
       </c>
+      <c r="X483" t="inlineStr">
+        <is>
+          <t>8536508008</t>
+        </is>
+      </c>
       <c r="Y483" t="s">
         <v>59</v>
       </c>
@@ -76993,6 +77922,11 @@
       <c r="W486" t="s">
         <v>3938</v>
       </c>
+      <c r="X486" t="inlineStr">
+        <is>
+          <t>8536901000</t>
+        </is>
+      </c>
       <c r="Y486" t="s">
         <v>59</v>
       </c>
@@ -77255,6 +78189,11 @@
       <c r="W488" t="s">
         <v>3955</v>
       </c>
+      <c r="X488" t="inlineStr">
+        <is>
+          <t>3926909709</t>
+        </is>
+      </c>
       <c r="Y488" t="s">
         <v>59</v>
       </c>
@@ -77511,6 +78450,11 @@
       <c r="W490" t="s">
         <v>3971</v>
       </c>
+      <c r="X490" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y490" t="s">
         <v>59</v>
       </c>
@@ -77770,6 +78714,11 @@
       <c r="W492" t="s">
         <v>3987</v>
       </c>
+      <c r="X492" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y492" t="s">
         <v>59</v>
       </c>
@@ -77898,6 +78847,11 @@
       <c r="W493" t="s">
         <v>3995</v>
       </c>
+      <c r="X493" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y493" t="s">
         <v>59</v>
       </c>
@@ -78026,6 +78980,11 @@
       <c r="W494" t="s">
         <v>4003</v>
       </c>
+      <c r="X494" t="inlineStr">
+        <is>
+          <t>7326909807</t>
+        </is>
+      </c>
       <c r="Y494" t="s">
         <v>59</v>
       </c>
@@ -78285,6 +79244,11 @@
       <c r="W496" t="s">
         <v>4016</v>
       </c>
+      <c r="X496" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y496" t="s">
         <v>59</v>
       </c>
@@ -78413,6 +79377,11 @@
       <c r="W497" t="s">
         <v>4024</v>
       </c>
+      <c r="X497" t="inlineStr">
+        <is>
+          <t>9405490039</t>
+        </is>
+      </c>
       <c r="Y497" t="s">
         <v>59</v>
       </c>
@@ -78671,6 +79640,11 @@
       </c>
       <c r="W499" t="s">
         <v>4040</v>
+      </c>
+      <c r="X499" t="inlineStr">
+        <is>
+          <t>8536508008</t>
+        </is>
       </c>
       <c r="Y499" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Fix verified weights and dimensions
</commit_message>
<xml_diff>
--- a/data/catalog_500_exact_match.xlsx
+++ b/data/catalog_500_exact_match.xlsx
@@ -34581,7 +34581,7 @@
         <v>1319</v>
       </c>
       <c r="S151">
-        <v>2.46</v>
+        <v>2460</v>
       </c>
       <c r="T151">
         <v>180</v>
@@ -34959,9 +34959,7 @@
       <c r="R154" s="7" t="s">
         <v>1343</v>
       </c>
-      <c r="S154">
-        <v>0.2</v>
-      </c>
+      <c r="S154"/>
       <c r="T154">
         <v>100</v>
       </c>
@@ -35031,9 +35029,7 @@
       <c r="AQ154" t="s">
         <v>70</v>
       </c>
-      <c r="AS154" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS154"/>
     </row>
     <row r="155" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
@@ -35090,9 +35086,7 @@
       <c r="R155" s="7" t="s">
         <v>1353</v>
       </c>
-      <c r="S155">
-        <v>250</v>
-      </c>
+      <c r="S155"/>
       <c r="T155">
         <v>141</v>
       </c>
@@ -35162,9 +35156,7 @@
       <c r="AR155" t="s">
         <v>1359</v>
       </c>
-      <c r="AS155" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS155"/>
     </row>
     <row r="156" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
@@ -37245,13 +37237,13 @@
         <v>2</v>
       </c>
       <c r="T172">
-        <v>400</v>
+        <v>840</v>
       </c>
       <c r="U172">
         <v>250</v>
       </c>
       <c r="V172">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="W172" t="s">
         <v>1503</v>
@@ -45855,7 +45847,7 @@
         <v>2048</v>
       </c>
       <c r="S240">
-        <v>0.04</v>
+        <v>40</v>
       </c>
       <c r="T240">
         <v>70</v>
@@ -52520,9 +52512,7 @@
       <c r="R293" s="7" t="s">
         <v>2444</v>
       </c>
-      <c r="S293">
-        <v>0.6</v>
-      </c>
+      <c r="S293"/>
       <c r="T293">
         <v>250</v>
       </c>
@@ -52592,9 +52582,7 @@
       <c r="AR293" t="s">
         <v>2450</v>
       </c>
-      <c r="AS293" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS293"/>
     </row>
     <row r="294" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
@@ -53151,9 +53139,7 @@
       <c r="R298" s="7" t="s">
         <v>2483</v>
       </c>
-      <c r="S298">
-        <v>0.25</v>
-      </c>
+      <c r="S298"/>
       <c r="T298">
         <v>140</v>
       </c>
@@ -53223,9 +53209,7 @@
       <c r="AQ298" t="s">
         <v>70</v>
       </c>
-      <c r="AS298" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS298"/>
     </row>
     <row r="299" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
@@ -53282,17 +53266,15 @@
       <c r="R299" s="7" t="s">
         <v>2491</v>
       </c>
-      <c r="S299">
-        <v>0.25</v>
-      </c>
+      <c r="S299"/>
       <c r="T299">
         <v>150</v>
       </c>
       <c r="U299">
-        <v>150</v>
+        <v>83</v>
       </c>
       <c r="V299">
-        <v>150</v>
+        <v>47</v>
       </c>
       <c r="W299" t="s">
         <v>2492</v>
@@ -53357,9 +53339,7 @@
       <c r="AR299" t="s">
         <v>2494</v>
       </c>
-      <c r="AS299" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS299"/>
     </row>
     <row r="300" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
@@ -53416,9 +53396,7 @@
       <c r="R300" s="7" t="s">
         <v>2500</v>
       </c>
-      <c r="S300">
-        <v>300</v>
-      </c>
+      <c r="S300"/>
       <c r="T300">
         <v>200</v>
       </c>
@@ -53487,9 +53465,7 @@
       <c r="AQ300" t="s">
         <v>70</v>
       </c>
-      <c r="AS300" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS300"/>
     </row>
     <row r="301" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
@@ -53546,9 +53522,7 @@
       <c r="R301" s="7" t="s">
         <v>2509</v>
       </c>
-      <c r="S301">
-        <v>500</v>
-      </c>
+      <c r="S301"/>
       <c r="T301">
         <v>57</v>
       </c>
@@ -53620,9 +53594,7 @@
       <c r="AR301" t="s">
         <v>2514</v>
       </c>
-      <c r="AS301" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS301"/>
     </row>
     <row r="302" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
@@ -53679,9 +53651,7 @@
       <c r="R302" s="7" t="s">
         <v>2519</v>
       </c>
-      <c r="S302">
-        <v>0.7</v>
-      </c>
+      <c r="S302"/>
       <c r="T302">
         <v>127</v>
       </c>
@@ -53754,9 +53724,7 @@
       <c r="AR302" t="s">
         <v>2523</v>
       </c>
-      <c r="AS302" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS302"/>
     </row>
     <row r="303" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
@@ -53813,9 +53781,7 @@
       <c r="R303" s="7" t="s">
         <v>2530</v>
       </c>
-      <c r="S303">
-        <v>1000</v>
-      </c>
+      <c r="S303"/>
       <c r="T303">
         <v>160</v>
       </c>
@@ -53823,7 +53789,7 @@
         <v>160</v>
       </c>
       <c r="V303">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="W303" t="s">
         <v>2531</v>
@@ -53884,9 +53850,7 @@
       <c r="AR303" t="s">
         <v>2533</v>
       </c>
-      <c r="AS303" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS303"/>
     </row>
     <row r="304" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
@@ -53943,9 +53907,7 @@
       <c r="R304" s="7" t="s">
         <v>2539</v>
       </c>
-      <c r="S304">
-        <v>0.25</v>
-      </c>
+      <c r="S304"/>
       <c r="T304">
         <v>140</v>
       </c>
@@ -54009,9 +53971,7 @@
       <c r="AQ304" t="s">
         <v>70</v>
       </c>
-      <c r="AS304" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS304"/>
     </row>
     <row r="305" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
@@ -54068,9 +54028,7 @@
       <c r="R305" s="7" t="s">
         <v>2548</v>
       </c>
-      <c r="S305">
-        <v>0.25</v>
-      </c>
+      <c r="S305"/>
       <c r="T305">
         <v>140</v>
       </c>
@@ -54134,9 +54092,7 @@
       <c r="AQ305" t="s">
         <v>70</v>
       </c>
-      <c r="AS305" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS305"/>
     </row>
     <row r="306" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
@@ -54193,9 +54149,7 @@
       <c r="R306" s="7" t="s">
         <v>2557</v>
       </c>
-      <c r="S306">
-        <v>0.25</v>
-      </c>
+      <c r="S306"/>
       <c r="T306">
         <v>140</v>
       </c>
@@ -54265,9 +54219,7 @@
       <c r="AQ306" t="s">
         <v>70</v>
       </c>
-      <c r="AS306" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS306"/>
     </row>
     <row r="307" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
@@ -54324,9 +54276,7 @@
       <c r="R307" s="7" t="s">
         <v>2565</v>
       </c>
-      <c r="S307">
-        <v>0.25</v>
-      </c>
+      <c r="S307"/>
       <c r="T307">
         <v>140</v>
       </c>
@@ -54396,9 +54346,7 @@
       <c r="AQ307" t="s">
         <v>70</v>
       </c>
-      <c r="AS307" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS307"/>
     </row>
     <row r="308" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
@@ -54455,9 +54403,7 @@
       <c r="R308" s="7" t="s">
         <v>2572</v>
       </c>
-      <c r="S308">
-        <v>0.25</v>
-      </c>
+      <c r="S308"/>
       <c r="T308">
         <v>140</v>
       </c>
@@ -54527,9 +54473,7 @@
       <c r="AQ308" t="s">
         <v>70</v>
       </c>
-      <c r="AS308" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS308"/>
     </row>
     <row r="309" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
@@ -54586,9 +54530,7 @@
       <c r="R309" s="7" t="s">
         <v>2579</v>
       </c>
-      <c r="S309">
-        <v>0.25</v>
-      </c>
+      <c r="S309"/>
       <c r="T309">
         <v>140</v>
       </c>
@@ -54652,9 +54594,7 @@
       <c r="AQ309" t="s">
         <v>70</v>
       </c>
-      <c r="AS309" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS309"/>
     </row>
     <row r="310" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
@@ -54711,9 +54651,7 @@
       <c r="R310" s="7" t="s">
         <v>2587</v>
       </c>
-      <c r="S310">
-        <v>0.25</v>
-      </c>
+      <c r="S310"/>
       <c r="T310">
         <v>140</v>
       </c>
@@ -54783,9 +54721,7 @@
       <c r="AQ310" t="s">
         <v>70</v>
       </c>
-      <c r="AS310" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS310"/>
     </row>
     <row r="311" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
@@ -54842,9 +54778,7 @@
       <c r="R311" s="7" t="s">
         <v>2594</v>
       </c>
-      <c r="S311">
-        <v>0.25</v>
-      </c>
+      <c r="S311"/>
       <c r="T311">
         <v>140</v>
       </c>
@@ -54914,9 +54848,7 @@
       <c r="AQ311" t="s">
         <v>70</v>
       </c>
-      <c r="AS311" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS311"/>
     </row>
     <row r="312" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
@@ -54973,9 +54905,7 @@
       <c r="R312" s="7" t="s">
         <v>2603</v>
       </c>
-      <c r="S312">
-        <v>0.25</v>
-      </c>
+      <c r="S312"/>
       <c r="T312">
         <v>140</v>
       </c>
@@ -55045,9 +54975,7 @@
       <c r="AQ312" t="s">
         <v>70</v>
       </c>
-      <c r="AS312" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS312"/>
     </row>
     <row r="313" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
@@ -55104,9 +55032,7 @@
       <c r="R313" s="7" t="s">
         <v>2611</v>
       </c>
-      <c r="S313">
-        <v>0.25</v>
-      </c>
+      <c r="S313"/>
       <c r="T313">
         <v>140</v>
       </c>
@@ -55176,9 +55102,7 @@
       <c r="AQ313" t="s">
         <v>70</v>
       </c>
-      <c r="AS313" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS313"/>
     </row>
     <row r="314" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
@@ -55235,9 +55159,7 @@
       <c r="R314" s="7" t="s">
         <v>2619</v>
       </c>
-      <c r="S314">
-        <v>0.25</v>
-      </c>
+      <c r="S314"/>
       <c r="T314">
         <v>140</v>
       </c>
@@ -55307,9 +55229,7 @@
       <c r="AQ314" t="s">
         <v>70</v>
       </c>
-      <c r="AS314" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS314"/>
     </row>
     <row r="315" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
@@ -55366,9 +55286,7 @@
       <c r="R315" s="7" t="s">
         <v>2627</v>
       </c>
-      <c r="S315">
-        <v>0.25</v>
-      </c>
+      <c r="S315"/>
       <c r="T315">
         <v>140</v>
       </c>
@@ -55432,9 +55350,7 @@
       <c r="AQ315" t="s">
         <v>70</v>
       </c>
-      <c r="AS315" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS315"/>
     </row>
     <row r="316" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
@@ -55491,9 +55407,7 @@
       <c r="R316" s="7" t="s">
         <v>2634</v>
       </c>
-      <c r="S316">
-        <v>0.25</v>
-      </c>
+      <c r="S316"/>
       <c r="T316">
         <v>140</v>
       </c>
@@ -55557,9 +55471,7 @@
       <c r="AQ316" t="s">
         <v>70</v>
       </c>
-      <c r="AS316" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS316"/>
     </row>
     <row r="317" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
@@ -55616,9 +55528,7 @@
       <c r="R317" s="7" t="s">
         <v>2642</v>
       </c>
-      <c r="S317">
-        <v>1000</v>
-      </c>
+      <c r="S317"/>
       <c r="T317">
         <v>200</v>
       </c>
@@ -55684,9 +55594,7 @@
       <c r="AQ317" t="s">
         <v>70</v>
       </c>
-      <c r="AS317" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS317"/>
     </row>
     <row r="318" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
@@ -55753,7 +55661,7 @@
         <v>350</v>
       </c>
       <c r="V318">
-        <v>220</v>
+        <v>270</v>
       </c>
       <c r="W318" t="s">
         <v>2651</v>
@@ -55876,9 +55784,7 @@
       <c r="R319" s="7" t="s">
         <v>2658</v>
       </c>
-      <c r="S319">
-        <v>0.82499999999999996</v>
-      </c>
+      <c r="S319"/>
       <c r="T319">
         <v>142.5</v>
       </c>
@@ -55945,9 +55851,7 @@
       <c r="AQ319" t="s">
         <v>70</v>
       </c>
-      <c r="AS319" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS319"/>
     </row>
     <row r="320" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
@@ -56004,9 +55908,7 @@
       <c r="R320" s="7" t="s">
         <v>2666</v>
       </c>
-      <c r="S320">
-        <v>100</v>
-      </c>
+      <c r="S320"/>
       <c r="T320">
         <v>200</v>
       </c>
@@ -56078,9 +55980,7 @@
       <c r="AQ320" t="s">
         <v>70</v>
       </c>
-      <c r="AS320" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS320"/>
     </row>
     <row r="321" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
@@ -56137,9 +56037,7 @@
       <c r="R321" s="7" t="s">
         <v>2675</v>
       </c>
-      <c r="S321">
-        <v>1</v>
-      </c>
+      <c r="S321"/>
       <c r="T321">
         <v>220</v>
       </c>
@@ -56206,9 +56104,7 @@
       <c r="AQ321" t="s">
         <v>70</v>
       </c>
-      <c r="AS321" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS321"/>
     </row>
     <row r="322" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
@@ -56673,9 +56569,7 @@
       <c r="R325" s="7" t="s">
         <v>2710</v>
       </c>
-      <c r="S325">
-        <v>29.5</v>
-      </c>
+      <c r="S325"/>
       <c r="T325">
         <v>285</v>
       </c>
@@ -56750,9 +56644,7 @@
       <c r="AR325" t="s">
         <v>2713</v>
       </c>
-      <c r="AS325" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS325"/>
     </row>
     <row r="326" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
@@ -56816,10 +56708,10 @@
         <v>61</v>
       </c>
       <c r="U326">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="V326">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="W326" t="s">
         <v>2718</v>
@@ -56942,9 +56834,7 @@
       <c r="R327" s="7" t="s">
         <v>2726</v>
       </c>
-      <c r="S327">
-        <v>30</v>
-      </c>
+      <c r="S327"/>
       <c r="T327">
         <v>200</v>
       </c>
@@ -57016,9 +56906,7 @@
       <c r="AQ327" t="s">
         <v>70</v>
       </c>
-      <c r="AS327" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS327"/>
     </row>
     <row r="328" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
@@ -57075,9 +56963,7 @@
       <c r="R328" s="7" t="s">
         <v>2733</v>
       </c>
-      <c r="S328">
-        <v>1000</v>
-      </c>
+      <c r="S328"/>
       <c r="T328">
         <v>200</v>
       </c>
@@ -57152,9 +57038,7 @@
       <c r="AR328" t="s">
         <v>2736</v>
       </c>
-      <c r="AS328" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS328"/>
     </row>
     <row r="329" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
@@ -57211,9 +57095,7 @@
       <c r="R329" s="7" t="s">
         <v>2741</v>
       </c>
-      <c r="S329">
-        <v>1000</v>
-      </c>
+      <c r="S329"/>
       <c r="T329">
         <v>200</v>
       </c>
@@ -57288,9 +57170,7 @@
       <c r="AR329" t="s">
         <v>2744</v>
       </c>
-      <c r="AS329" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS329"/>
     </row>
     <row r="330" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
@@ -57347,9 +57227,7 @@
       <c r="R330" s="7" t="s">
         <v>2748</v>
       </c>
-      <c r="S330">
-        <v>1000</v>
-      </c>
+      <c r="S330"/>
       <c r="T330">
         <v>200</v>
       </c>
@@ -57424,9 +57302,7 @@
       <c r="AR330" t="s">
         <v>2751</v>
       </c>
-      <c r="AS330" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS330"/>
     </row>
     <row r="331" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
@@ -57483,17 +57359,15 @@
       <c r="R331" s="7" t="s">
         <v>2756</v>
       </c>
-      <c r="S331">
-        <v>96.5</v>
-      </c>
+      <c r="S331"/>
       <c r="T331">
         <v>64</v>
       </c>
       <c r="U331">
-        <v>64</v>
+        <v>22.5</v>
       </c>
       <c r="V331">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="W331" t="s">
         <v>2757</v>
@@ -57558,9 +57432,7 @@
       <c r="AR331" t="s">
         <v>2759</v>
       </c>
-      <c r="AS331" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS331"/>
     </row>
     <row r="332" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
@@ -57617,17 +57489,15 @@
       <c r="R332" s="7" t="s">
         <v>2764</v>
       </c>
-      <c r="S332">
-        <v>96.5</v>
-      </c>
+      <c r="S332"/>
       <c r="T332">
         <v>64</v>
       </c>
       <c r="U332">
-        <v>64</v>
+        <v>22.5</v>
       </c>
       <c r="V332">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="W332" t="s">
         <v>2765</v>
@@ -57689,9 +57559,7 @@
       <c r="AR332" t="s">
         <v>2759</v>
       </c>
-      <c r="AS332" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS332"/>
     </row>
     <row r="333" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
@@ -58020,9 +57888,7 @@
       <c r="R335" s="7" t="s">
         <v>2787</v>
       </c>
-      <c r="S335">
-        <v>900</v>
-      </c>
+      <c r="S335"/>
       <c r="T335">
         <v>145</v>
       </c>
@@ -58094,9 +57960,7 @@
       <c r="AR335" t="s">
         <v>2790</v>
       </c>
-      <c r="AS335" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS335"/>
     </row>
     <row r="336" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
@@ -58153,9 +58017,7 @@
       <c r="R336" s="7" t="s">
         <v>2794</v>
       </c>
-      <c r="S336">
-        <v>900</v>
-      </c>
+      <c r="S336"/>
       <c r="T336">
         <v>206</v>
       </c>
@@ -58230,9 +58092,7 @@
       <c r="AR336" t="s">
         <v>2797</v>
       </c>
-      <c r="AS336" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS336"/>
     </row>
     <row r="337" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
@@ -58289,9 +58149,7 @@
       <c r="R337" s="7" t="s">
         <v>2802</v>
       </c>
-      <c r="S337">
-        <v>300</v>
-      </c>
+      <c r="S337"/>
       <c r="T337">
         <v>107</v>
       </c>
@@ -58363,9 +58221,7 @@
       <c r="AR337" t="s">
         <v>2805</v>
       </c>
-      <c r="AS337" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS337"/>
     </row>
     <row r="338" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
@@ -58422,9 +58278,7 @@
       <c r="R338" s="7" t="s">
         <v>2810</v>
       </c>
-      <c r="S338">
-        <v>1000</v>
-      </c>
+      <c r="S338"/>
       <c r="T338">
         <v>64</v>
       </c>
@@ -58499,9 +58353,7 @@
       <c r="AR338" t="s">
         <v>2813</v>
       </c>
-      <c r="AS338" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS338"/>
     </row>
     <row r="339" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
@@ -58558,9 +58410,7 @@
       <c r="R339" s="7" t="s">
         <v>2710</v>
       </c>
-      <c r="S339">
-        <v>29.5</v>
-      </c>
+      <c r="S339"/>
       <c r="T339">
         <v>300</v>
       </c>
@@ -58635,9 +58485,7 @@
       <c r="AR339" t="s">
         <v>2821</v>
       </c>
-      <c r="AS339" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS339"/>
     </row>
     <row r="340" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
@@ -58694,9 +58542,7 @@
       <c r="R340" s="7" t="s">
         <v>2826</v>
       </c>
-      <c r="S340">
-        <v>1000</v>
-      </c>
+      <c r="S340"/>
       <c r="T340">
         <v>70</v>
       </c>
@@ -58768,9 +58614,7 @@
       <c r="AR340" t="s">
         <v>2829</v>
       </c>
-      <c r="AS340" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS340"/>
     </row>
     <row r="341" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
@@ -58827,9 +58671,7 @@
       <c r="R341" s="7" t="s">
         <v>2834</v>
       </c>
-      <c r="S341">
-        <v>1000</v>
-      </c>
+      <c r="S341"/>
       <c r="T341">
         <v>101</v>
       </c>
@@ -58904,9 +58746,7 @@
       <c r="AR341" t="s">
         <v>2837</v>
       </c>
-      <c r="AS341" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS341"/>
     </row>
     <row r="342" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
@@ -59906,9 +59746,7 @@
       <c r="R349" s="7" t="s">
         <v>2906</v>
       </c>
-      <c r="S349">
-        <v>44</v>
-      </c>
+      <c r="S349"/>
       <c r="T349">
         <v>230</v>
       </c>
@@ -59975,9 +59813,7 @@
       <c r="AQ349" t="s">
         <v>70</v>
       </c>
-      <c r="AS349" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS349"/>
     </row>
     <row r="350" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
@@ -60034,9 +59870,7 @@
       <c r="R350" s="7" t="s">
         <v>2914</v>
       </c>
-      <c r="S350">
-        <v>0.25</v>
-      </c>
+      <c r="S350"/>
       <c r="T350">
         <v>107</v>
       </c>
@@ -60109,9 +59943,7 @@
       <c r="AR350" t="s">
         <v>2805</v>
       </c>
-      <c r="AS350" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS350"/>
     </row>
     <row r="351" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
@@ -60168,9 +60000,7 @@
       <c r="R351" s="7" t="s">
         <v>2923</v>
       </c>
-      <c r="S351">
-        <v>44</v>
-      </c>
+      <c r="S351"/>
       <c r="T351">
         <v>180</v>
       </c>
@@ -60236,9 +60066,7 @@
       <c r="AQ351" t="s">
         <v>70</v>
       </c>
-      <c r="AS351" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS351"/>
     </row>
     <row r="352" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
@@ -60295,9 +60123,7 @@
       <c r="R352" s="7" t="s">
         <v>2930</v>
       </c>
-      <c r="S352">
-        <v>44</v>
-      </c>
+      <c r="S352"/>
       <c r="T352">
         <v>180</v>
       </c>
@@ -60363,9 +60189,7 @@
       <c r="AQ352" t="s">
         <v>70</v>
       </c>
-      <c r="AS352" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS352"/>
     </row>
     <row r="353" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
@@ -60422,9 +60246,7 @@
       <c r="R353" s="7" t="s">
         <v>2937</v>
       </c>
-      <c r="S353">
-        <v>0.6</v>
-      </c>
+      <c r="S353"/>
       <c r="T353">
         <v>200</v>
       </c>
@@ -60494,9 +60316,7 @@
       <c r="AQ353" t="s">
         <v>70</v>
       </c>
-      <c r="AS353" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS353"/>
     </row>
     <row r="354" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
@@ -60553,9 +60373,7 @@
       <c r="R354" s="7" t="s">
         <v>2947</v>
       </c>
-      <c r="S354">
-        <v>1500</v>
-      </c>
+      <c r="S354"/>
       <c r="T354">
         <v>200</v>
       </c>
@@ -60627,9 +60445,7 @@
       <c r="AR354" t="s">
         <v>2951</v>
       </c>
-      <c r="AS354" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS354"/>
     </row>
     <row r="355" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
@@ -60686,9 +60502,7 @@
       <c r="R355" s="7" t="s">
         <v>2957</v>
       </c>
-      <c r="S355">
-        <v>3.5</v>
-      </c>
+      <c r="S355"/>
       <c r="T355">
         <v>320</v>
       </c>
@@ -60761,9 +60575,7 @@
       <c r="AR355" t="s">
         <v>2961</v>
       </c>
-      <c r="AS355" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS355"/>
     </row>
     <row r="356" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
@@ -60820,9 +60632,7 @@
       <c r="R356" s="7" t="s">
         <v>2966</v>
       </c>
-      <c r="S356">
-        <v>3.5</v>
-      </c>
+      <c r="S356"/>
       <c r="T356">
         <v>320</v>
       </c>
@@ -60895,9 +60705,7 @@
       <c r="AR356" t="s">
         <v>2969</v>
       </c>
-      <c r="AS356" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS356"/>
     </row>
     <row r="357" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
@@ -60954,9 +60762,7 @@
       <c r="R357" s="7" t="s">
         <v>2974</v>
       </c>
-      <c r="S357">
-        <v>3.5</v>
-      </c>
+      <c r="S357"/>
       <c r="T357">
         <v>320</v>
       </c>
@@ -61029,9 +60835,7 @@
       <c r="AR357" t="s">
         <v>2977</v>
       </c>
-      <c r="AS357" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS357"/>
     </row>
     <row r="358" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
@@ -61088,9 +60892,7 @@
       <c r="R358" s="7" t="s">
         <v>2982</v>
       </c>
-      <c r="S358">
-        <v>3.5</v>
-      </c>
+      <c r="S358"/>
       <c r="T358">
         <v>320</v>
       </c>
@@ -61163,9 +60965,7 @@
       <c r="AR358" t="s">
         <v>2985</v>
       </c>
-      <c r="AS358" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS358"/>
     </row>
     <row r="359" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
@@ -61222,9 +61022,7 @@
       <c r="R359" s="7" t="s">
         <v>2990</v>
       </c>
-      <c r="S359">
-        <v>3.5</v>
-      </c>
+      <c r="S359"/>
       <c r="T359">
         <v>320</v>
       </c>
@@ -61297,9 +61095,7 @@
       <c r="AR359" t="s">
         <v>2993</v>
       </c>
-      <c r="AS359" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS359"/>
     </row>
     <row r="360" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
@@ -61356,9 +61152,7 @@
       <c r="R360" s="7" t="s">
         <v>2998</v>
       </c>
-      <c r="S360">
-        <v>3.5</v>
-      </c>
+      <c r="S360"/>
       <c r="T360">
         <v>320</v>
       </c>
@@ -61431,9 +61225,7 @@
       <c r="AR360" t="s">
         <v>3001</v>
       </c>
-      <c r="AS360" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS360"/>
     </row>
     <row r="361" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
@@ -61490,9 +61282,7 @@
       <c r="R361" s="7" t="s">
         <v>3006</v>
       </c>
-      <c r="S361">
-        <v>3.5</v>
-      </c>
+      <c r="S361"/>
       <c r="T361">
         <v>320</v>
       </c>
@@ -61559,9 +61349,7 @@
       <c r="AR361" t="s">
         <v>3009</v>
       </c>
-      <c r="AS361" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS361"/>
     </row>
     <row r="362" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
@@ -61618,9 +61406,7 @@
       <c r="R362" s="7" t="s">
         <v>3014</v>
       </c>
-      <c r="S362">
-        <v>3.5</v>
-      </c>
+      <c r="S362"/>
       <c r="T362">
         <v>320</v>
       </c>
@@ -61687,9 +61473,7 @@
       <c r="AR362" t="s">
         <v>3017</v>
       </c>
-      <c r="AS362" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS362"/>
     </row>
     <row r="363" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
@@ -61746,9 +61530,7 @@
       <c r="R363" s="7" t="s">
         <v>3022</v>
       </c>
-      <c r="S363">
-        <v>1500</v>
-      </c>
+      <c r="S363"/>
       <c r="T363">
         <v>200</v>
       </c>
@@ -61823,9 +61605,7 @@
       <c r="AR363" t="s">
         <v>3026</v>
       </c>
-      <c r="AS363" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS363"/>
     </row>
     <row r="364" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
@@ -61882,9 +61662,7 @@
       <c r="R364" s="7" t="s">
         <v>3031</v>
       </c>
-      <c r="S364">
-        <v>3.5</v>
-      </c>
+      <c r="S364"/>
       <c r="T364">
         <v>320</v>
       </c>
@@ -61957,9 +61735,7 @@
       <c r="AR364" t="s">
         <v>3034</v>
       </c>
-      <c r="AS364" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS364"/>
     </row>
     <row r="365" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
@@ -62016,9 +61792,7 @@
       <c r="R365" s="7" t="s">
         <v>3039</v>
       </c>
-      <c r="S365">
-        <v>3.5</v>
-      </c>
+      <c r="S365"/>
       <c r="T365">
         <v>320</v>
       </c>
@@ -62091,9 +61865,7 @@
       <c r="AR365" t="s">
         <v>3042</v>
       </c>
-      <c r="AS365" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS365"/>
     </row>
     <row r="366" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
@@ -62150,9 +61922,7 @@
       <c r="R366" s="7" t="s">
         <v>3047</v>
       </c>
-      <c r="S366">
-        <v>3.5</v>
-      </c>
+      <c r="S366"/>
       <c r="T366">
         <v>320</v>
       </c>
@@ -62225,9 +61995,7 @@
       <c r="AR366" t="s">
         <v>3050</v>
       </c>
-      <c r="AS366" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS366"/>
     </row>
     <row r="367" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
@@ -62284,9 +62052,7 @@
       <c r="R367" s="7" t="s">
         <v>3055</v>
       </c>
-      <c r="S367">
-        <v>3.5</v>
-      </c>
+      <c r="S367"/>
       <c r="T367">
         <v>320</v>
       </c>
@@ -62359,9 +62125,7 @@
       <c r="AR367" t="s">
         <v>3058</v>
       </c>
-      <c r="AS367" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS367"/>
     </row>
     <row r="368" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
@@ -62418,9 +62182,7 @@
       <c r="R368" s="7" t="s">
         <v>3063</v>
       </c>
-      <c r="S368">
-        <v>3.5</v>
-      </c>
+      <c r="S368"/>
       <c r="T368">
         <v>320</v>
       </c>
@@ -62490,9 +62252,7 @@
       <c r="AR368" t="s">
         <v>3066</v>
       </c>
-      <c r="AS368" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS368"/>
     </row>
     <row r="369" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
@@ -62549,9 +62309,7 @@
       <c r="R369" s="7" t="s">
         <v>3071</v>
       </c>
-      <c r="S369">
-        <v>3.5</v>
-      </c>
+      <c r="S369"/>
       <c r="T369">
         <v>320</v>
       </c>
@@ -62624,9 +62382,7 @@
       <c r="AR369" t="s">
         <v>3074</v>
       </c>
-      <c r="AS369" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS369"/>
     </row>
     <row r="370" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
@@ -62683,9 +62439,7 @@
       <c r="R370" s="7" t="s">
         <v>3079</v>
       </c>
-      <c r="S370">
-        <v>3.5</v>
-      </c>
+      <c r="S370"/>
       <c r="T370">
         <v>320</v>
       </c>
@@ -62758,9 +62512,7 @@
       <c r="AR370" t="s">
         <v>3082</v>
       </c>
-      <c r="AS370" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS370"/>
     </row>
     <row r="371" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
@@ -62817,9 +62569,7 @@
       <c r="R371" s="7" t="s">
         <v>3087</v>
       </c>
-      <c r="S371">
-        <v>0.2</v>
-      </c>
+      <c r="S371"/>
       <c r="T371">
         <v>225</v>
       </c>
@@ -62894,9 +62644,7 @@
       <c r="AR371" t="s">
         <v>3090</v>
       </c>
-      <c r="AS371" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS371"/>
     </row>
     <row r="372" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
@@ -62953,9 +62701,7 @@
       <c r="R372" s="7" t="s">
         <v>3095</v>
       </c>
-      <c r="S372">
-        <v>300</v>
-      </c>
+      <c r="S372"/>
       <c r="T372">
         <v>200</v>
       </c>
@@ -63027,9 +62773,7 @@
       <c r="AQ372" t="s">
         <v>70</v>
       </c>
-      <c r="AS372" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS372"/>
     </row>
     <row r="373" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
@@ -63086,9 +62830,7 @@
       <c r="R373" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S373">
-        <v>44</v>
-      </c>
+      <c r="S373"/>
       <c r="T373">
         <v>180</v>
       </c>
@@ -63157,9 +62899,7 @@
       <c r="AQ373" t="s">
         <v>70</v>
       </c>
-      <c r="AS373" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS373"/>
     </row>
     <row r="374" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
@@ -63216,9 +62956,7 @@
       <c r="R374" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S374">
-        <v>44</v>
-      </c>
+      <c r="S374"/>
       <c r="T374">
         <v>180</v>
       </c>
@@ -63287,9 +63025,7 @@
       <c r="AQ374" t="s">
         <v>70</v>
       </c>
-      <c r="AS374" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS374"/>
     </row>
     <row r="375" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
@@ -63346,9 +63082,7 @@
       <c r="R375" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S375">
-        <v>44</v>
-      </c>
+      <c r="S375"/>
       <c r="T375">
         <v>180</v>
       </c>
@@ -63414,9 +63148,7 @@
       <c r="AQ375" t="s">
         <v>70</v>
       </c>
-      <c r="AS375" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS375"/>
     </row>
     <row r="376" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
@@ -63473,9 +63205,7 @@
       <c r="R376" s="7" t="s">
         <v>3121</v>
       </c>
-      <c r="S376">
-        <v>150</v>
-      </c>
+      <c r="S376"/>
       <c r="T376">
         <v>200</v>
       </c>
@@ -63547,9 +63277,7 @@
       <c r="AQ376" t="s">
         <v>70</v>
       </c>
-      <c r="AS376" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS376"/>
     </row>
     <row r="377" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
@@ -63606,9 +63334,7 @@
       <c r="R377" s="7" t="s">
         <v>3130</v>
       </c>
-      <c r="S377">
-        <v>300</v>
-      </c>
+      <c r="S377"/>
       <c r="T377">
         <v>200</v>
       </c>
@@ -63680,9 +63406,7 @@
       <c r="AQ377" t="s">
         <v>70</v>
       </c>
-      <c r="AS377" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS377"/>
     </row>
     <row r="378" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
@@ -63739,9 +63463,7 @@
       <c r="R378" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S378">
-        <v>44</v>
-      </c>
+      <c r="S378"/>
       <c r="T378">
         <v>180</v>
       </c>
@@ -63813,9 +63535,7 @@
       <c r="AR378" t="s">
         <v>3141</v>
       </c>
-      <c r="AS378" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS378"/>
     </row>
     <row r="379" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
@@ -63872,9 +63592,7 @@
       <c r="R379" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S379">
-        <v>44</v>
-      </c>
+      <c r="S379"/>
       <c r="T379">
         <v>180</v>
       </c>
@@ -63943,9 +63661,7 @@
       <c r="AQ379" t="s">
         <v>70</v>
       </c>
-      <c r="AS379" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS379"/>
     </row>
     <row r="380" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
@@ -64002,9 +63718,7 @@
       <c r="R380" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S380">
-        <v>44</v>
-      </c>
+      <c r="S380"/>
       <c r="T380">
         <v>180</v>
       </c>
@@ -64076,9 +63790,7 @@
       <c r="AR380" t="s">
         <v>3154</v>
       </c>
-      <c r="AS380" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS380"/>
     </row>
     <row r="381" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
@@ -64135,9 +63847,7 @@
       <c r="R381" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S381">
-        <v>44</v>
-      </c>
+      <c r="S381"/>
       <c r="T381">
         <v>180</v>
       </c>
@@ -64209,9 +63919,7 @@
       <c r="AR381" t="s">
         <v>3161</v>
       </c>
-      <c r="AS381" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS381"/>
     </row>
     <row r="382" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
@@ -64268,9 +63976,7 @@
       <c r="R382" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S382">
-        <v>44</v>
-      </c>
+      <c r="S382"/>
       <c r="T382">
         <v>180</v>
       </c>
@@ -64342,9 +64048,7 @@
       <c r="AR382" t="s">
         <v>3168</v>
       </c>
-      <c r="AS382" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS382"/>
     </row>
     <row r="383" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
@@ -64401,9 +64105,7 @@
       <c r="R383" s="7" t="s">
         <v>3173</v>
       </c>
-      <c r="S383">
-        <v>44</v>
-      </c>
+      <c r="S383"/>
       <c r="T383">
         <v>180</v>
       </c>
@@ -64472,9 +64174,7 @@
       <c r="AQ383" t="s">
         <v>70</v>
       </c>
-      <c r="AS383" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS383"/>
     </row>
     <row r="384" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
@@ -64531,9 +64231,7 @@
       <c r="R384" s="7" t="s">
         <v>3181</v>
       </c>
-      <c r="S384">
-        <v>44</v>
-      </c>
+      <c r="S384"/>
       <c r="T384">
         <v>230</v>
       </c>
@@ -64600,9 +64298,7 @@
       <c r="AQ384" t="s">
         <v>70</v>
       </c>
-      <c r="AS384" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS384"/>
     </row>
     <row r="385" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
@@ -64659,9 +64355,7 @@
       <c r="R385" s="7" t="s">
         <v>3173</v>
       </c>
-      <c r="S385">
-        <v>44</v>
-      </c>
+      <c r="S385"/>
       <c r="T385">
         <v>180</v>
       </c>
@@ -64730,9 +64424,7 @@
       <c r="AQ385" t="s">
         <v>70</v>
       </c>
-      <c r="AS385" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS385"/>
     </row>
     <row r="386" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
@@ -64789,9 +64481,7 @@
       <c r="R386" s="7" t="s">
         <v>3173</v>
       </c>
-      <c r="S386">
-        <v>44</v>
-      </c>
+      <c r="S386"/>
       <c r="T386">
         <v>180</v>
       </c>
@@ -64860,9 +64550,7 @@
       <c r="AQ386" t="s">
         <v>70</v>
       </c>
-      <c r="AS386" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS386"/>
     </row>
     <row r="387" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
@@ -64919,9 +64607,7 @@
       <c r="R387" s="7" t="s">
         <v>3173</v>
       </c>
-      <c r="S387">
-        <v>44</v>
-      </c>
+      <c r="S387"/>
       <c r="T387">
         <v>180</v>
       </c>
@@ -64990,9 +64676,7 @@
       <c r="AQ387" t="s">
         <v>70</v>
       </c>
-      <c r="AS387" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS387"/>
     </row>
     <row r="388" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
@@ -65049,9 +64733,7 @@
       <c r="R388" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S388">
-        <v>44</v>
-      </c>
+      <c r="S388"/>
       <c r="T388">
         <v>180</v>
       </c>
@@ -65120,9 +64802,7 @@
       <c r="AQ388" t="s">
         <v>70</v>
       </c>
-      <c r="AS388" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS388"/>
     </row>
     <row r="389" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
@@ -65307,9 +64987,7 @@
       <c r="R390" s="7" t="s">
         <v>3219</v>
       </c>
-      <c r="S390">
-        <v>1000</v>
-      </c>
+      <c r="S390"/>
       <c r="T390">
         <v>200</v>
       </c>
@@ -65384,9 +65062,7 @@
       <c r="AR390" t="s">
         <v>3222</v>
       </c>
-      <c r="AS390" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS390"/>
     </row>
     <row r="391" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
@@ -65443,9 +65119,7 @@
       <c r="R391" s="7" t="s">
         <v>3227</v>
       </c>
-      <c r="S391">
-        <v>1000</v>
-      </c>
+      <c r="S391"/>
       <c r="T391">
         <v>89</v>
       </c>
@@ -65520,9 +65194,7 @@
       <c r="AR391" t="s">
         <v>3230</v>
       </c>
-      <c r="AS391" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS391"/>
     </row>
     <row r="392" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
@@ -65579,9 +65251,7 @@
       <c r="R392" s="7" t="s">
         <v>2881</v>
       </c>
-      <c r="S392">
-        <v>300</v>
-      </c>
+      <c r="S392"/>
       <c r="T392">
         <v>167</v>
       </c>
@@ -65656,9 +65326,7 @@
       <c r="AR392" t="s">
         <v>3237</v>
       </c>
-      <c r="AS392" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS392"/>
     </row>
     <row r="393" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
@@ -65715,9 +65383,7 @@
       <c r="R393" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S393">
-        <v>44</v>
-      </c>
+      <c r="S393"/>
       <c r="T393">
         <v>180</v>
       </c>
@@ -65792,9 +65458,7 @@
       <c r="AR393" t="s">
         <v>3247</v>
       </c>
-      <c r="AS393" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS393"/>
     </row>
     <row r="394" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
@@ -65851,9 +65515,7 @@
       <c r="R394" s="7" t="s">
         <v>3252</v>
       </c>
-      <c r="S394">
-        <v>44</v>
-      </c>
+      <c r="S394"/>
       <c r="T394">
         <v>180</v>
       </c>
@@ -65928,9 +65590,7 @@
       <c r="AR394" t="s">
         <v>3257</v>
       </c>
-      <c r="AS394" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS394"/>
     </row>
     <row r="395" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
@@ -65987,9 +65647,7 @@
       <c r="R395" s="7" t="s">
         <v>3252</v>
       </c>
-      <c r="S395">
-        <v>44</v>
-      </c>
+      <c r="S395"/>
       <c r="T395">
         <v>180</v>
       </c>
@@ -66061,9 +65719,7 @@
       <c r="AR395" t="s">
         <v>3257</v>
       </c>
-      <c r="AS395" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS395"/>
     </row>
     <row r="396" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
@@ -66120,9 +65776,7 @@
       <c r="R396" s="7" t="s">
         <v>3252</v>
       </c>
-      <c r="S396">
-        <v>44</v>
-      </c>
+      <c r="S396"/>
       <c r="T396">
         <v>180</v>
       </c>
@@ -66197,9 +65851,7 @@
       <c r="AR396" t="s">
         <v>3270</v>
       </c>
-      <c r="AS396" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS396"/>
     </row>
     <row r="397" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
@@ -66256,9 +65908,7 @@
       <c r="R397" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S397">
-        <v>44</v>
-      </c>
+      <c r="S397"/>
       <c r="T397">
         <v>180</v>
       </c>
@@ -66330,9 +65980,7 @@
       <c r="AR397" t="s">
         <v>3277</v>
       </c>
-      <c r="AS397" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS397"/>
     </row>
     <row r="398" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
@@ -66389,9 +66037,7 @@
       <c r="R398" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S398">
-        <v>44</v>
-      </c>
+      <c r="S398"/>
       <c r="T398">
         <v>180</v>
       </c>
@@ -66466,9 +66112,7 @@
       <c r="AR398" t="s">
         <v>3284</v>
       </c>
-      <c r="AS398" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS398"/>
     </row>
     <row r="399" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
@@ -66525,9 +66169,7 @@
       <c r="R399" s="7" t="s">
         <v>3289</v>
       </c>
-      <c r="S399">
-        <v>44</v>
-      </c>
+      <c r="S399"/>
       <c r="T399">
         <v>180</v>
       </c>
@@ -66602,9 +66244,7 @@
       <c r="AR399" t="s">
         <v>3154</v>
       </c>
-      <c r="AS399" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS399"/>
     </row>
     <row r="400" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
@@ -66661,9 +66301,7 @@
       <c r="R400" s="7" t="s">
         <v>3296</v>
       </c>
-      <c r="S400">
-        <v>0.7</v>
-      </c>
+      <c r="S400"/>
       <c r="T400">
         <v>180</v>
       </c>
@@ -66736,9 +66374,7 @@
       <c r="AR400" t="s">
         <v>3300</v>
       </c>
-      <c r="AS400" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS400"/>
     </row>
     <row r="401" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
@@ -66795,9 +66431,7 @@
       <c r="R401" s="7" t="s">
         <v>3305</v>
       </c>
-      <c r="S401">
-        <v>0.7</v>
-      </c>
+      <c r="S401"/>
       <c r="T401">
         <v>180</v>
       </c>
@@ -66870,9 +66504,7 @@
       <c r="AR401" t="s">
         <v>3161</v>
       </c>
-      <c r="AS401" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS401"/>
     </row>
     <row r="402" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
@@ -66929,9 +66561,7 @@
       <c r="R402" s="7" t="s">
         <v>3312</v>
       </c>
-      <c r="S402">
-        <v>44</v>
-      </c>
+      <c r="S402"/>
       <c r="T402">
         <v>180</v>
       </c>
@@ -67006,9 +66636,7 @@
       <c r="AR402" t="s">
         <v>3161</v>
       </c>
-      <c r="AS402" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS402"/>
     </row>
     <row r="403" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
@@ -67065,9 +66693,7 @@
       <c r="R403" s="7" t="s">
         <v>3321</v>
       </c>
-      <c r="S403">
-        <v>0.7</v>
-      </c>
+      <c r="S403"/>
       <c r="T403">
         <v>180</v>
       </c>
@@ -67140,9 +66766,7 @@
       <c r="AR403" t="s">
         <v>3325</v>
       </c>
-      <c r="AS403" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS403"/>
     </row>
     <row r="404" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
@@ -67199,9 +66823,7 @@
       <c r="R404" s="7" t="s">
         <v>3330</v>
       </c>
-      <c r="S404">
-        <v>0.7</v>
-      </c>
+      <c r="S404"/>
       <c r="T404">
         <v>180</v>
       </c>
@@ -67271,9 +66893,7 @@
       <c r="AR404" t="s">
         <v>3333</v>
       </c>
-      <c r="AS404" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS404"/>
     </row>
     <row r="405" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
@@ -67330,9 +66950,7 @@
       <c r="R405" s="7" t="s">
         <v>3338</v>
       </c>
-      <c r="S405">
-        <v>0.7</v>
-      </c>
+      <c r="S405"/>
       <c r="T405">
         <v>180</v>
       </c>
@@ -67405,9 +67023,7 @@
       <c r="AR405" t="s">
         <v>3161</v>
       </c>
-      <c r="AS405" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS405"/>
     </row>
     <row r="406" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
@@ -67464,9 +67080,7 @@
       <c r="R406" s="7" t="s">
         <v>3312</v>
       </c>
-      <c r="S406">
-        <v>44</v>
-      </c>
+      <c r="S406"/>
       <c r="T406">
         <v>180</v>
       </c>
@@ -67538,9 +67152,7 @@
       <c r="AR406" t="s">
         <v>3347</v>
       </c>
-      <c r="AS406" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS406"/>
     </row>
     <row r="407" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
@@ -67597,9 +67209,7 @@
       <c r="R407" s="7" t="s">
         <v>3352</v>
       </c>
-      <c r="S407">
-        <v>44</v>
-      </c>
+      <c r="S407"/>
       <c r="T407">
         <v>180</v>
       </c>
@@ -67671,9 +67281,7 @@
       <c r="AR407" t="s">
         <v>3347</v>
       </c>
-      <c r="AS407" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS407"/>
     </row>
     <row r="408" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
@@ -67730,9 +67338,7 @@
       <c r="R408" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S408">
-        <v>44</v>
-      </c>
+      <c r="S408"/>
       <c r="T408">
         <v>180</v>
       </c>
@@ -67804,9 +67410,7 @@
       <c r="AR408" t="s">
         <v>3168</v>
       </c>
-      <c r="AS408" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS408"/>
     </row>
     <row r="409" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
@@ -67863,9 +67467,7 @@
       <c r="R409" s="7" t="s">
         <v>3365</v>
       </c>
-      <c r="S409">
-        <v>0.7</v>
-      </c>
+      <c r="S409"/>
       <c r="T409">
         <v>180</v>
       </c>
@@ -67935,9 +67537,7 @@
       <c r="AR409" t="s">
         <v>3168</v>
       </c>
-      <c r="AS409" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS409"/>
     </row>
     <row r="410" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
@@ -67994,9 +67594,7 @@
       <c r="R410" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S410">
-        <v>44</v>
-      </c>
+      <c r="S410"/>
       <c r="T410">
         <v>180</v>
       </c>
@@ -68068,9 +67666,7 @@
       <c r="AR410" t="s">
         <v>3375</v>
       </c>
-      <c r="AS410" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS410"/>
     </row>
     <row r="411" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
@@ -68127,9 +67723,7 @@
       <c r="R411" s="7" t="s">
         <v>3380</v>
       </c>
-      <c r="S411">
-        <v>44</v>
-      </c>
+      <c r="S411"/>
       <c r="T411">
         <v>180</v>
       </c>
@@ -68204,9 +67798,7 @@
       <c r="AR411" t="s">
         <v>3161</v>
       </c>
-      <c r="AS411" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS411"/>
     </row>
     <row r="412" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
@@ -68263,9 +67855,7 @@
       <c r="R412" s="7" t="s">
         <v>3388</v>
       </c>
-      <c r="S412">
-        <v>0.7</v>
-      </c>
+      <c r="S412"/>
       <c r="T412">
         <v>180</v>
       </c>
@@ -68335,9 +67925,7 @@
       <c r="AR412" t="s">
         <v>3257</v>
       </c>
-      <c r="AS412" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS412"/>
     </row>
     <row r="413" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
@@ -68394,9 +67982,7 @@
       <c r="R413" s="7" t="s">
         <v>3380</v>
       </c>
-      <c r="S413">
-        <v>44</v>
-      </c>
+      <c r="S413"/>
       <c r="T413">
         <v>180</v>
       </c>
@@ -68468,9 +68054,7 @@
       <c r="AR413" t="s">
         <v>3397</v>
       </c>
-      <c r="AS413" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS413"/>
     </row>
     <row r="414" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
@@ -68658,9 +68242,7 @@
       <c r="R415" s="7" t="s">
         <v>3252</v>
       </c>
-      <c r="S415">
-        <v>44</v>
-      </c>
+      <c r="S415"/>
       <c r="T415">
         <v>180</v>
       </c>
@@ -68735,9 +68317,7 @@
       <c r="AR415" t="s">
         <v>3413</v>
       </c>
-      <c r="AS415" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS415"/>
     </row>
     <row r="416" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
@@ -68794,9 +68374,7 @@
       <c r="R416" s="7" t="s">
         <v>3252</v>
       </c>
-      <c r="S416">
-        <v>44</v>
-      </c>
+      <c r="S416"/>
       <c r="T416">
         <v>180</v>
       </c>
@@ -68868,9 +68446,7 @@
       <c r="AR416" t="s">
         <v>3420</v>
       </c>
-      <c r="AS416" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS416"/>
     </row>
     <row r="417" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
@@ -68927,9 +68503,7 @@
       <c r="R417" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S417">
-        <v>44</v>
-      </c>
+      <c r="S417"/>
       <c r="T417">
         <v>180</v>
       </c>
@@ -69001,9 +68575,7 @@
       <c r="AR417" t="s">
         <v>3420</v>
       </c>
-      <c r="AS417" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS417"/>
     </row>
     <row r="418" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
@@ -69060,9 +68632,7 @@
       <c r="R418" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S418">
-        <v>44</v>
-      </c>
+      <c r="S418"/>
       <c r="T418">
         <v>180</v>
       </c>
@@ -69137,9 +68707,7 @@
       <c r="AR418" t="s">
         <v>3434</v>
       </c>
-      <c r="AS418" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS418"/>
     </row>
     <row r="419" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
@@ -69196,9 +68764,7 @@
       <c r="R419" s="7" t="s">
         <v>3252</v>
       </c>
-      <c r="S419">
-        <v>44</v>
-      </c>
+      <c r="S419"/>
       <c r="T419">
         <v>180</v>
       </c>
@@ -69273,9 +68839,7 @@
       <c r="AR419" t="s">
         <v>3375</v>
       </c>
-      <c r="AS419" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS419"/>
     </row>
     <row r="420" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
@@ -69332,9 +68896,7 @@
       <c r="R420" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S420">
-        <v>44</v>
-      </c>
+      <c r="S420"/>
       <c r="T420">
         <v>180</v>
       </c>
@@ -69409,9 +68971,7 @@
       <c r="AR420" t="s">
         <v>3154</v>
       </c>
-      <c r="AS420" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS420"/>
     </row>
     <row r="421" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
@@ -69468,9 +69028,7 @@
       <c r="R421" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S421">
-        <v>44</v>
-      </c>
+      <c r="S421"/>
       <c r="T421">
         <v>180</v>
       </c>
@@ -69545,9 +69103,7 @@
       <c r="AR421" t="s">
         <v>3375</v>
       </c>
-      <c r="AS421" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS421"/>
     </row>
     <row r="422" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
@@ -69604,9 +69160,7 @@
       <c r="R422" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S422">
-        <v>44</v>
-      </c>
+      <c r="S422"/>
       <c r="T422">
         <v>180</v>
       </c>
@@ -69678,9 +69232,7 @@
       <c r="AR422" t="s">
         <v>3161</v>
       </c>
-      <c r="AS422" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS422"/>
     </row>
     <row r="423" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
@@ -69737,9 +69289,7 @@
       <c r="R423" s="7" t="s">
         <v>3463</v>
       </c>
-      <c r="S423">
-        <v>0.7</v>
-      </c>
+      <c r="S423"/>
       <c r="T423">
         <v>180</v>
       </c>
@@ -69812,9 +69362,7 @@
       <c r="AR423" t="s">
         <v>3466</v>
       </c>
-      <c r="AS423" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS423"/>
     </row>
     <row r="424" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
@@ -69871,9 +69419,7 @@
       <c r="R424" s="7" t="s">
         <v>3471</v>
       </c>
-      <c r="S424">
-        <v>0.7</v>
-      </c>
+      <c r="S424"/>
       <c r="T424">
         <v>180</v>
       </c>
@@ -69943,9 +69489,7 @@
       <c r="AR424" t="s">
         <v>3474</v>
       </c>
-      <c r="AS424" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS424"/>
     </row>
     <row r="425" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
@@ -70002,9 +69546,7 @@
       <c r="R425" s="7" t="s">
         <v>3479</v>
       </c>
-      <c r="S425">
-        <v>0.7</v>
-      </c>
+      <c r="S425"/>
       <c r="T425">
         <v>180</v>
       </c>
@@ -70071,9 +69613,7 @@
       <c r="AQ425" t="s">
         <v>70</v>
       </c>
-      <c r="AS425" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS425"/>
     </row>
     <row r="426" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
@@ -70130,9 +69670,7 @@
       <c r="R426" s="7" t="s">
         <v>3487</v>
       </c>
-      <c r="S426">
-        <v>44</v>
-      </c>
+      <c r="S426"/>
       <c r="T426">
         <v>180</v>
       </c>
@@ -70201,9 +69739,7 @@
       <c r="AQ426" t="s">
         <v>70</v>
       </c>
-      <c r="AS426" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS426"/>
     </row>
     <row r="427" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
@@ -70260,9 +69796,7 @@
       <c r="R427" s="7" t="s">
         <v>3495</v>
       </c>
-      <c r="S427">
-        <v>2.0110000000000001</v>
-      </c>
+      <c r="S427"/>
       <c r="T427">
         <v>180</v>
       </c>
@@ -70329,9 +69863,7 @@
       <c r="AQ427" t="s">
         <v>70</v>
       </c>
-      <c r="AS427" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS427"/>
     </row>
     <row r="428" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
@@ -70388,9 +69920,7 @@
       <c r="R428" s="7" t="s">
         <v>3503</v>
       </c>
-      <c r="S428">
-        <v>0.7</v>
-      </c>
+      <c r="S428"/>
       <c r="T428">
         <v>180</v>
       </c>
@@ -70457,9 +69987,7 @@
       <c r="AQ428" t="s">
         <v>70</v>
       </c>
-      <c r="AS428" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS428"/>
     </row>
     <row r="429" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
@@ -70516,9 +70044,7 @@
       <c r="R429" s="7" t="s">
         <v>3510</v>
       </c>
-      <c r="S429">
-        <v>0.7</v>
-      </c>
+      <c r="S429"/>
       <c r="T429">
         <v>180</v>
       </c>
@@ -70585,9 +70111,7 @@
       <c r="AQ429" t="s">
         <v>70</v>
       </c>
-      <c r="AS429" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS429"/>
     </row>
     <row r="430" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
@@ -70644,9 +70168,7 @@
       <c r="R430" s="7" t="s">
         <v>3517</v>
       </c>
-      <c r="S430">
-        <v>0.7</v>
-      </c>
+      <c r="S430"/>
       <c r="T430">
         <v>180</v>
       </c>
@@ -70716,9 +70238,7 @@
       <c r="AQ430" t="s">
         <v>70</v>
       </c>
-      <c r="AS430" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS430"/>
     </row>
     <row r="431" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
@@ -70775,9 +70295,7 @@
       <c r="R431" s="7" t="s">
         <v>3524</v>
       </c>
-      <c r="S431">
-        <v>44</v>
-      </c>
+      <c r="S431"/>
       <c r="T431">
         <v>230</v>
       </c>
@@ -70844,9 +70362,7 @@
       <c r="AQ431" t="s">
         <v>70</v>
       </c>
-      <c r="AS431" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS431"/>
     </row>
     <row r="432" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
@@ -71032,7 +70548,7 @@
         <v>3538</v>
       </c>
       <c r="S433">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="T433">
         <v>230</v>
@@ -71159,9 +70675,7 @@
       <c r="R434" s="7" t="s">
         <v>3546</v>
       </c>
-      <c r="S434">
-        <v>44</v>
-      </c>
+      <c r="S434"/>
       <c r="T434">
         <v>230</v>
       </c>
@@ -71228,9 +70742,7 @@
       <c r="AQ434" t="s">
         <v>70</v>
       </c>
-      <c r="AS434" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS434"/>
     </row>
     <row r="435" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
@@ -71287,9 +70799,7 @@
       <c r="R435" s="7" t="s">
         <v>3552</v>
       </c>
-      <c r="S435">
-        <v>44</v>
-      </c>
+      <c r="S435"/>
       <c r="T435">
         <v>230</v>
       </c>
@@ -71356,9 +70866,7 @@
       <c r="AQ435" t="s">
         <v>70</v>
       </c>
-      <c r="AS435" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS435"/>
     </row>
     <row r="436" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
@@ -71415,9 +70923,7 @@
       <c r="R436" s="7" t="s">
         <v>2930</v>
       </c>
-      <c r="S436">
-        <v>44</v>
-      </c>
+      <c r="S436"/>
       <c r="T436">
         <v>180</v>
       </c>
@@ -71486,9 +70992,7 @@
       <c r="AQ436" t="s">
         <v>70</v>
       </c>
-      <c r="AS436" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS436"/>
     </row>
     <row r="437" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
@@ -71545,9 +71049,7 @@
       <c r="R437" s="7" t="s">
         <v>3565</v>
       </c>
-      <c r="S437">
-        <v>0.6</v>
-      </c>
+      <c r="S437"/>
       <c r="T437">
         <v>200</v>
       </c>
@@ -71614,9 +71116,7 @@
       <c r="AQ437" t="s">
         <v>70</v>
       </c>
-      <c r="AS437" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS437"/>
     </row>
     <row r="438" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
@@ -71673,9 +71173,7 @@
       <c r="R438" s="7" t="s">
         <v>3573</v>
       </c>
-      <c r="S438">
-        <v>0.6</v>
-      </c>
+      <c r="S438"/>
       <c r="T438">
         <v>200</v>
       </c>
@@ -71745,9 +71243,7 @@
       <c r="AQ438" t="s">
         <v>70</v>
       </c>
-      <c r="AS438" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS438"/>
     </row>
     <row r="439" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
@@ -71804,9 +71300,7 @@
       <c r="R439" s="7" t="s">
         <v>3581</v>
       </c>
-      <c r="S439">
-        <v>400</v>
-      </c>
+      <c r="S439"/>
       <c r="T439">
         <v>200</v>
       </c>
@@ -71878,9 +71372,7 @@
       <c r="AQ439" t="s">
         <v>70</v>
       </c>
-      <c r="AS439" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS439"/>
     </row>
     <row r="440" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
@@ -71937,9 +71429,7 @@
       <c r="R440" s="7" t="s">
         <v>3590</v>
       </c>
-      <c r="S440">
-        <v>1000</v>
-      </c>
+      <c r="S440"/>
       <c r="T440">
         <v>333</v>
       </c>
@@ -72008,9 +71498,7 @@
       <c r="AR440" t="s">
         <v>3593</v>
       </c>
-      <c r="AS440" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS440"/>
     </row>
     <row r="441" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
@@ -72067,9 +71555,7 @@
       <c r="R441" s="7" t="s">
         <v>3598</v>
       </c>
-      <c r="S441">
-        <v>44</v>
-      </c>
+      <c r="S441"/>
       <c r="T441">
         <v>200</v>
       </c>
@@ -72141,9 +71627,7 @@
       <c r="AQ441" t="s">
         <v>70</v>
       </c>
-      <c r="AS441" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS441"/>
     </row>
     <row r="442" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
@@ -72200,9 +71684,7 @@
       <c r="R442" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S442">
-        <v>44</v>
-      </c>
+      <c r="S442"/>
       <c r="T442">
         <v>180</v>
       </c>
@@ -72271,9 +71753,7 @@
       <c r="AQ442" t="s">
         <v>70</v>
       </c>
-      <c r="AS442" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS442"/>
     </row>
     <row r="443" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
@@ -72330,9 +71810,7 @@
       <c r="R443" s="7" t="s">
         <v>3614</v>
       </c>
-      <c r="S443">
-        <v>0.7</v>
-      </c>
+      <c r="S443"/>
       <c r="T443">
         <v>180</v>
       </c>
@@ -72399,9 +71877,7 @@
       <c r="AQ443" t="s">
         <v>70</v>
       </c>
-      <c r="AS443" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS443"/>
     </row>
     <row r="444" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
@@ -72458,9 +71934,7 @@
       <c r="R444" s="7" t="s">
         <v>3621</v>
       </c>
-      <c r="S444">
-        <v>0.7</v>
-      </c>
+      <c r="S444"/>
       <c r="T444">
         <v>180</v>
       </c>
@@ -72524,9 +71998,7 @@
       <c r="AQ444" t="s">
         <v>70</v>
       </c>
-      <c r="AS444" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS444"/>
     </row>
     <row r="445" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
@@ -72583,9 +72055,7 @@
       <c r="R445" s="7" t="s">
         <v>3628</v>
       </c>
-      <c r="S445">
-        <v>44</v>
-      </c>
+      <c r="S445"/>
       <c r="T445">
         <v>180</v>
       </c>
@@ -72651,9 +72121,7 @@
       <c r="AQ445" t="s">
         <v>70</v>
       </c>
-      <c r="AS445" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS445"/>
     </row>
     <row r="446" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
@@ -72710,9 +72178,7 @@
       <c r="R446" s="7" t="s">
         <v>3628</v>
       </c>
-      <c r="S446">
-        <v>44</v>
-      </c>
+      <c r="S446"/>
       <c r="T446">
         <v>180</v>
       </c>
@@ -72781,9 +72247,7 @@
       <c r="AQ446" t="s">
         <v>70</v>
       </c>
-      <c r="AS446" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS446"/>
     </row>
     <row r="447" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
@@ -72840,9 +72304,7 @@
       <c r="R447" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S447">
-        <v>44</v>
-      </c>
+      <c r="S447"/>
       <c r="T447">
         <v>180</v>
       </c>
@@ -72914,9 +72376,7 @@
       <c r="AQ447" t="s">
         <v>70</v>
       </c>
-      <c r="AS447" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS447"/>
     </row>
     <row r="448" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
@@ -72973,9 +72433,7 @@
       <c r="R448" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S448">
-        <v>2.012</v>
-      </c>
+      <c r="S448"/>
       <c r="T448">
         <v>180</v>
       </c>
@@ -73041,9 +72499,7 @@
       <c r="AQ448" t="s">
         <v>70</v>
       </c>
-      <c r="AS448" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS448"/>
     </row>
     <row r="449" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
@@ -73100,9 +72556,7 @@
       <c r="R449" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S449">
-        <v>44</v>
-      </c>
+      <c r="S449"/>
       <c r="T449">
         <v>180</v>
       </c>
@@ -73171,9 +72625,7 @@
       <c r="AQ449" t="s">
         <v>70</v>
       </c>
-      <c r="AS449" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS449"/>
     </row>
     <row r="450" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
@@ -73230,9 +72682,7 @@
       <c r="R450" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S450">
-        <v>44</v>
-      </c>
+      <c r="S450"/>
       <c r="T450">
         <v>180</v>
       </c>
@@ -73304,9 +72754,7 @@
       <c r="AQ450" t="s">
         <v>70</v>
       </c>
-      <c r="AS450" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS450"/>
     </row>
     <row r="451" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
@@ -73363,9 +72811,7 @@
       <c r="R451" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S451">
-        <v>44</v>
-      </c>
+      <c r="S451"/>
       <c r="T451">
         <v>180</v>
       </c>
@@ -73431,9 +72877,7 @@
       <c r="AQ451" t="s">
         <v>70</v>
       </c>
-      <c r="AS451" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS451"/>
     </row>
     <row r="452" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
@@ -73490,9 +72934,7 @@
       <c r="R452" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S452">
-        <v>2.0139999999999998</v>
-      </c>
+      <c r="S452"/>
       <c r="T452">
         <v>180</v>
       </c>
@@ -73564,9 +73006,7 @@
       <c r="AR452" t="s">
         <v>3161</v>
       </c>
-      <c r="AS452" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS452"/>
     </row>
     <row r="453" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
@@ -73623,9 +73063,7 @@
       <c r="R453" s="7" t="s">
         <v>3681</v>
       </c>
-      <c r="S453">
-        <v>0.7</v>
-      </c>
+      <c r="S453"/>
       <c r="T453">
         <v>180</v>
       </c>
@@ -73695,9 +73133,7 @@
       <c r="AR453" t="s">
         <v>3161</v>
       </c>
-      <c r="AS453" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS453"/>
     </row>
     <row r="454" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
@@ -73754,9 +73190,7 @@
       <c r="R454" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S454">
-        <v>44</v>
-      </c>
+      <c r="S454"/>
       <c r="T454">
         <v>180</v>
       </c>
@@ -73822,9 +73256,7 @@
       <c r="AQ454" t="s">
         <v>70</v>
       </c>
-      <c r="AS454" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS454"/>
     </row>
     <row r="455" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
@@ -73881,9 +73313,7 @@
       <c r="R455" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S455">
-        <v>44</v>
-      </c>
+      <c r="S455"/>
       <c r="T455">
         <v>180</v>
       </c>
@@ -73955,9 +73385,7 @@
       <c r="AQ455" t="s">
         <v>70</v>
       </c>
-      <c r="AS455" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS455"/>
     </row>
     <row r="456" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
@@ -74014,9 +73442,7 @@
       <c r="R456" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S456">
-        <v>44</v>
-      </c>
+      <c r="S456"/>
       <c r="T456">
         <v>180</v>
       </c>
@@ -74085,9 +73511,7 @@
       <c r="AQ456" t="s">
         <v>70</v>
       </c>
-      <c r="AS456" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS456"/>
     </row>
     <row r="457" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
@@ -74144,9 +73568,7 @@
       <c r="R457" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S457">
-        <v>44</v>
-      </c>
+      <c r="S457"/>
       <c r="T457">
         <v>180</v>
       </c>
@@ -74215,9 +73637,7 @@
       <c r="AQ457" t="s">
         <v>70</v>
       </c>
-      <c r="AS457" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS457"/>
     </row>
     <row r="458" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A458" t="s">
@@ -74274,9 +73694,7 @@
       <c r="R458" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S458">
-        <v>44</v>
-      </c>
+      <c r="S458"/>
       <c r="T458">
         <v>180</v>
       </c>
@@ -74345,9 +73763,7 @@
       <c r="AQ458" t="s">
         <v>70</v>
       </c>
-      <c r="AS458" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS458"/>
     </row>
     <row r="459" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A459" t="s">
@@ -74404,9 +73820,7 @@
       <c r="R459" s="7" t="s">
         <v>3724</v>
       </c>
-      <c r="S459">
-        <v>2.0110000000000001</v>
-      </c>
+      <c r="S459"/>
       <c r="T459">
         <v>180</v>
       </c>
@@ -74473,9 +73887,7 @@
       <c r="AR459" t="s">
         <v>3728</v>
       </c>
-      <c r="AS459" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS459"/>
     </row>
     <row r="460" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
@@ -74532,9 +73944,7 @@
       <c r="R460" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S460">
-        <v>44</v>
-      </c>
+      <c r="S460"/>
       <c r="T460">
         <v>180</v>
       </c>
@@ -74603,9 +74013,7 @@
       <c r="AQ460" t="s">
         <v>70</v>
       </c>
-      <c r="AS460" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS460"/>
     </row>
     <row r="461" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A461" t="s">
@@ -74662,9 +74070,7 @@
       <c r="R461" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S461">
-        <v>2</v>
-      </c>
+      <c r="S461"/>
       <c r="T461">
         <v>180</v>
       </c>
@@ -74733,9 +74139,7 @@
       <c r="AQ461" t="s">
         <v>70</v>
       </c>
-      <c r="AS461" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS461"/>
     </row>
     <row r="462" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A462" t="s">
@@ -74792,9 +74196,7 @@
       <c r="R462" s="7" t="s">
         <v>3103</v>
       </c>
-      <c r="S462">
-        <v>44</v>
-      </c>
+      <c r="S462"/>
       <c r="T462">
         <v>180</v>
       </c>
@@ -74860,9 +74262,7 @@
       <c r="AQ462" t="s">
         <v>70</v>
       </c>
-      <c r="AS462" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS462"/>
     </row>
     <row r="463" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A463" t="s">
@@ -74919,9 +74319,7 @@
       <c r="R463" s="7" t="s">
         <v>3754</v>
       </c>
-      <c r="S463">
-        <v>44</v>
-      </c>
+      <c r="S463"/>
       <c r="T463">
         <v>230</v>
       </c>
@@ -74988,9 +74386,7 @@
       <c r="AQ463" t="s">
         <v>70</v>
       </c>
-      <c r="AS463" t="s">
-        <v>197</v>
-      </c>
+      <c r="AS463"/>
     </row>
     <row r="464" spans="1:45" x14ac:dyDescent="0.3">
       <c r="A464" t="s">

</xml_diff>